<commit_message>
add calendar endpoints tests
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Smart-University-Scheduler\helpers\db_seeder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FCB22A-F8D1-4747-BE76-C5A0D56C2E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3A858D-60E3-4B0F-AE8A-BF5C54CAA66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-6370" yWindow="-18960" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -712,11 +712,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1046,10 +1046,10 @@
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
@@ -1081,8 +1081,8 @@
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -1112,8 +1112,8 @@
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
       <c r="C4" t="s">
         <v>13</v>
       </c>
@@ -1143,8 +1143,8 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
       <c r="C5" t="s">
         <v>14</v>
       </c>
@@ -1174,8 +1174,8 @@
       </c>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
       <c r="C6" t="s">
         <v>15</v>
       </c>
@@ -1205,8 +1205,8 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
@@ -1238,8 +1238,8 @@
       </c>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
       <c r="C8" t="s">
         <v>18</v>
       </c>
@@ -1269,8 +1269,8 @@
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -1300,8 +1300,8 @@
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
       <c r="C10" t="s">
         <v>20</v>
       </c>
@@ -1331,8 +1331,8 @@
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
       <c r="C11" t="s">
         <v>21</v>
       </c>
@@ -1362,8 +1362,8 @@
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C12" t="s">
@@ -1395,8 +1395,8 @@
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
       <c r="C13" t="s">
         <v>24</v>
       </c>
@@ -1426,8 +1426,8 @@
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
       <c r="C14" t="s">
         <v>25</v>
       </c>
@@ -1457,8 +1457,8 @@
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
       <c r="C15" t="s">
         <v>26</v>
       </c>
@@ -1488,8 +1488,8 @@
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
       <c r="C16" t="s">
         <v>27</v>
       </c>
@@ -1519,8 +1519,8 @@
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C17" t="s">
@@ -1552,8 +1552,8 @@
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
       <c r="C18" t="s">
         <v>30</v>
       </c>
@@ -1583,8 +1583,8 @@
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
       <c r="C19" t="s">
         <v>31</v>
       </c>
@@ -1614,8 +1614,8 @@
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
       <c r="C20" t="s">
         <v>32</v>
       </c>
@@ -1645,8 +1645,8 @@
       </c>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
       <c r="C21" t="s">
         <v>33</v>
       </c>
@@ -1676,8 +1676,8 @@
       </c>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C22" t="s">
@@ -1709,8 +1709,8 @@
       </c>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
       <c r="C23" t="s">
         <v>36</v>
       </c>
@@ -1740,8 +1740,8 @@
       </c>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
       <c r="C24" t="s">
         <v>37</v>
       </c>
@@ -1771,8 +1771,8 @@
       </c>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
       <c r="C25" t="s">
         <v>38</v>
       </c>
@@ -1802,8 +1802,8 @@
       </c>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
       <c r="C26" t="s">
         <v>39</v>
       </c>
@@ -1833,10 +1833,10 @@
       </c>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1868,8 +1868,8 @@
       </c>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
       <c r="C28" t="s">
         <v>43</v>
       </c>
@@ -1899,8 +1899,8 @@
       </c>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
       <c r="C29" t="s">
         <v>44</v>
       </c>
@@ -1930,8 +1930,8 @@
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
       <c r="C30" t="s">
         <v>45</v>
       </c>
@@ -1961,8 +1961,8 @@
       </c>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
       <c r="C31" t="s">
         <v>46</v>
       </c>
@@ -1992,8 +1992,8 @@
       </c>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4" t="s">
+      <c r="A32" s="5"/>
+      <c r="B32" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C32" t="s">
@@ -2025,8 +2025,8 @@
       </c>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
       <c r="C33" t="s">
         <v>49</v>
       </c>
@@ -2056,8 +2056,8 @@
       </c>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
       <c r="C34" t="s">
         <v>50</v>
       </c>
@@ -2087,8 +2087,8 @@
       </c>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
       <c r="C35" t="s">
         <v>51</v>
       </c>
@@ -2118,8 +2118,8 @@
       </c>
     </row>
     <row r="36" spans="1:11">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
       <c r="C36" t="s">
         <v>52</v>
       </c>
@@ -2149,8 +2149,8 @@
       </c>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4" t="s">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C37" t="s">
@@ -2182,8 +2182,8 @@
       </c>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
       <c r="C38" t="s">
         <v>55</v>
       </c>
@@ -2213,8 +2213,8 @@
       </c>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
       <c r="C39" t="s">
         <v>56</v>
       </c>
@@ -2244,8 +2244,8 @@
       </c>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="4"/>
-      <c r="B40" s="4"/>
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
       <c r="C40" t="s">
         <v>57</v>
       </c>
@@ -2275,8 +2275,8 @@
       </c>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
       <c r="C41" t="s">
         <v>58</v>
       </c>
@@ -2306,8 +2306,8 @@
       </c>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4" t="s">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C42" t="s">
@@ -2339,8 +2339,8 @@
       </c>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4"/>
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
       <c r="C43" t="s">
         <v>61</v>
       </c>
@@ -2370,8 +2370,8 @@
       </c>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
       <c r="C44" t="s">
         <v>62</v>
       </c>
@@ -2401,8 +2401,8 @@
       </c>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
       <c r="C45" t="s">
         <v>63</v>
       </c>
@@ -2432,8 +2432,8 @@
       </c>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
       <c r="C46" t="s">
         <v>64</v>
       </c>
@@ -2463,8 +2463,8 @@
       </c>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4" t="s">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
         <v>65</v>
       </c>
       <c r="C47" t="s">
@@ -2496,8 +2496,8 @@
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
       <c r="C48" t="s">
         <v>67</v>
       </c>
@@ -2527,8 +2527,8 @@
       </c>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
       <c r="C49" t="s">
         <v>68</v>
       </c>
@@ -2558,8 +2558,8 @@
       </c>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2589,8 +2589,8 @@
       </c>
     </row>
     <row r="51" spans="1:11">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
       <c r="C51" t="s">
         <v>70</v>
       </c>
@@ -2620,8 +2620,8 @@
       </c>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4" t="s">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C52" t="s">
@@ -2653,8 +2653,8 @@
       </c>
     </row>
     <row r="53" spans="1:11">
-      <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
       <c r="C53" t="s">
         <v>72</v>
       </c>
@@ -2684,8 +2684,8 @@
       </c>
     </row>
     <row r="54" spans="1:11">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
+      <c r="A54" s="5"/>
+      <c r="B54" s="5"/>
       <c r="C54" t="s">
         <v>73</v>
       </c>
@@ -2715,8 +2715,8 @@
       </c>
     </row>
     <row r="55" spans="1:11">
-      <c r="A55" s="4"/>
-      <c r="B55" s="4"/>
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
       <c r="C55" t="s">
         <v>74</v>
       </c>
@@ -2746,8 +2746,8 @@
       </c>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
       <c r="C56" t="s">
         <v>75</v>
       </c>
@@ -2777,8 +2777,8 @@
       </c>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4" t="s">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C57" t="s">
@@ -2810,8 +2810,8 @@
       </c>
     </row>
     <row r="58" spans="1:11">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
       <c r="C58" t="s">
         <v>78</v>
       </c>
@@ -2841,8 +2841,8 @@
       </c>
     </row>
     <row r="59" spans="1:11">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
       <c r="C59" t="s">
         <v>79</v>
       </c>
@@ -2872,8 +2872,8 @@
       </c>
     </row>
     <row r="60" spans="1:11">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
       <c r="C60" t="s">
         <v>80</v>
       </c>
@@ -2903,8 +2903,8 @@
       </c>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
       <c r="C61" t="s">
         <v>81</v>
       </c>
@@ -2934,8 +2934,8 @@
       </c>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="4"/>
-      <c r="B62" s="4" t="s">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5" t="s">
         <v>82</v>
       </c>
       <c r="C62" t="s">
@@ -2967,8 +2967,8 @@
       </c>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="4"/>
-      <c r="B63" s="4"/>
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
       <c r="C63" t="s">
         <v>84</v>
       </c>
@@ -2998,8 +2998,8 @@
       </c>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="4"/>
-      <c r="B64" s="4"/>
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
       <c r="C64" t="s">
         <v>85</v>
       </c>
@@ -3029,8 +3029,8 @@
       </c>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="4"/>
-      <c r="B65" s="4"/>
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
       <c r="C65" t="s">
         <v>86</v>
       </c>
@@ -3060,8 +3060,8 @@
       </c>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="4"/>
-      <c r="B66" s="4"/>
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
       <c r="C66" t="s">
         <v>87</v>
       </c>
@@ -3091,10 +3091,10 @@
       </c>
     </row>
     <row r="67" spans="1:11">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C67" t="s">
@@ -3126,8 +3126,8 @@
       </c>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="4"/>
-      <c r="B68" s="4"/>
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
       <c r="C68" t="s">
         <v>91</v>
       </c>
@@ -3157,8 +3157,8 @@
       </c>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="4"/>
-      <c r="B69" s="4"/>
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
       <c r="C69" t="s">
         <v>92</v>
       </c>
@@ -3188,8 +3188,8 @@
       </c>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="4"/>
-      <c r="B70" s="4"/>
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
       <c r="C70" t="s">
         <v>93</v>
       </c>
@@ -3219,8 +3219,8 @@
       </c>
     </row>
     <row r="71" spans="1:11">
-      <c r="A71" s="4"/>
-      <c r="B71" s="4"/>
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
       <c r="C71" t="s">
         <v>94</v>
       </c>
@@ -3250,8 +3250,8 @@
       </c>
     </row>
     <row r="72" spans="1:11">
-      <c r="A72" s="4"/>
-      <c r="B72" s="4" t="s">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5" t="s">
         <v>95</v>
       </c>
       <c r="C72" t="s">
@@ -3283,8 +3283,8 @@
       </c>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="4"/>
-      <c r="B73" s="4"/>
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
       <c r="C73" t="s">
         <v>97</v>
       </c>
@@ -3314,8 +3314,8 @@
       </c>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="4"/>
-      <c r="B74" s="4"/>
+      <c r="A74" s="5"/>
+      <c r="B74" s="5"/>
       <c r="C74" t="s">
         <v>98</v>
       </c>
@@ -3345,8 +3345,8 @@
       </c>
     </row>
     <row r="75" spans="1:11">
-      <c r="A75" s="4"/>
-      <c r="B75" s="4"/>
+      <c r="A75" s="5"/>
+      <c r="B75" s="5"/>
       <c r="C75" t="s">
         <v>99</v>
       </c>
@@ -3376,8 +3376,8 @@
       </c>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="4"/>
-      <c r="B76" s="4"/>
+      <c r="A76" s="5"/>
+      <c r="B76" s="5"/>
       <c r="C76" t="s">
         <v>100</v>
       </c>
@@ -3407,8 +3407,8 @@
       </c>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="4"/>
-      <c r="B77" s="4" t="s">
+      <c r="A77" s="5"/>
+      <c r="B77" s="5" t="s">
         <v>101</v>
       </c>
       <c r="C77" t="s">
@@ -3440,8 +3440,8 @@
       </c>
     </row>
     <row r="78" spans="1:11">
-      <c r="A78" s="4"/>
-      <c r="B78" s="4"/>
+      <c r="A78" s="5"/>
+      <c r="B78" s="5"/>
       <c r="C78" t="s">
         <v>103</v>
       </c>
@@ -3471,8 +3471,8 @@
       </c>
     </row>
     <row r="79" spans="1:11">
-      <c r="A79" s="4"/>
-      <c r="B79" s="4"/>
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
       <c r="C79" t="s">
         <v>104</v>
       </c>
@@ -3502,8 +3502,8 @@
       </c>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="4"/>
-      <c r="B80" s="4"/>
+      <c r="A80" s="5"/>
+      <c r="B80" s="5"/>
       <c r="C80" t="s">
         <v>105</v>
       </c>
@@ -3533,8 +3533,8 @@
       </c>
     </row>
     <row r="81" spans="1:11">
-      <c r="A81" s="4"/>
-      <c r="B81" s="4"/>
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
       <c r="C81" t="s">
         <v>106</v>
       </c>
@@ -3564,8 +3564,8 @@
       </c>
     </row>
     <row r="82" spans="1:11">
-      <c r="A82" s="4"/>
-      <c r="B82" s="4" t="s">
+      <c r="A82" s="5"/>
+      <c r="B82" s="5" t="s">
         <v>107</v>
       </c>
       <c r="C82" t="s">
@@ -3597,8 +3597,8 @@
       </c>
     </row>
     <row r="83" spans="1:11">
-      <c r="A83" s="4"/>
-      <c r="B83" s="4"/>
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
       <c r="C83" t="s">
         <v>109</v>
       </c>
@@ -3628,8 +3628,8 @@
       </c>
     </row>
     <row r="84" spans="1:11">
-      <c r="A84" s="4"/>
-      <c r="B84" s="4"/>
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
       <c r="C84" t="s">
         <v>110</v>
       </c>
@@ -3659,8 +3659,8 @@
       </c>
     </row>
     <row r="85" spans="1:11">
-      <c r="A85" s="4"/>
-      <c r="B85" s="4"/>
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
       <c r="C85" t="s">
         <v>111</v>
       </c>
@@ -3690,8 +3690,8 @@
       </c>
     </row>
     <row r="86" spans="1:11">
-      <c r="A86" s="4"/>
-      <c r="B86" s="4"/>
+      <c r="A86" s="5"/>
+      <c r="B86" s="5"/>
       <c r="C86" t="s">
         <v>112</v>
       </c>
@@ -3721,10 +3721,10 @@
       </c>
     </row>
     <row r="87" spans="1:11">
-      <c r="A87" s="4" t="s">
+      <c r="A87" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="B87" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C87" t="s">
@@ -3756,8 +3756,8 @@
       </c>
     </row>
     <row r="88" spans="1:11">
-      <c r="A88" s="4"/>
-      <c r="B88" s="4"/>
+      <c r="A88" s="5"/>
+      <c r="B88" s="5"/>
       <c r="C88" t="s">
         <v>116</v>
       </c>
@@ -3787,8 +3787,8 @@
       </c>
     </row>
     <row r="89" spans="1:11">
-      <c r="A89" s="4"/>
-      <c r="B89" s="4"/>
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
       <c r="C89" t="s">
         <v>117</v>
       </c>
@@ -3818,8 +3818,8 @@
       </c>
     </row>
     <row r="90" spans="1:11">
-      <c r="A90" s="4"/>
-      <c r="B90" s="4"/>
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
       <c r="C90" t="s">
         <v>118</v>
       </c>
@@ -3849,8 +3849,8 @@
       </c>
     </row>
     <row r="91" spans="1:11">
-      <c r="A91" s="4"/>
-      <c r="B91" s="4"/>
+      <c r="A91" s="5"/>
+      <c r="B91" s="5"/>
       <c r="C91" t="s">
         <v>119</v>
       </c>
@@ -3880,8 +3880,8 @@
       </c>
     </row>
     <row r="92" spans="1:11">
-      <c r="A92" s="4"/>
-      <c r="B92" s="4" t="s">
+      <c r="A92" s="5"/>
+      <c r="B92" s="5" t="s">
         <v>120</v>
       </c>
       <c r="C92" t="s">
@@ -3913,8 +3913,8 @@
       </c>
     </row>
     <row r="93" spans="1:11">
-      <c r="A93" s="4"/>
-      <c r="B93" s="4"/>
+      <c r="A93" s="5"/>
+      <c r="B93" s="5"/>
       <c r="C93" t="s">
         <v>122</v>
       </c>
@@ -3944,8 +3944,8 @@
       </c>
     </row>
     <row r="94" spans="1:11">
-      <c r="A94" s="4"/>
-      <c r="B94" s="4"/>
+      <c r="A94" s="5"/>
+      <c r="B94" s="5"/>
       <c r="C94" t="s">
         <v>123</v>
       </c>
@@ -3975,8 +3975,8 @@
       </c>
     </row>
     <row r="95" spans="1:11">
-      <c r="A95" s="4"/>
-      <c r="B95" s="4"/>
+      <c r="A95" s="5"/>
+      <c r="B95" s="5"/>
       <c r="C95" t="s">
         <v>124</v>
       </c>
@@ -4006,8 +4006,8 @@
       </c>
     </row>
     <row r="96" spans="1:11">
-      <c r="A96" s="4"/>
-      <c r="B96" s="4"/>
+      <c r="A96" s="5"/>
+      <c r="B96" s="5"/>
       <c r="C96" t="s">
         <v>125</v>
       </c>
@@ -4037,8 +4037,8 @@
       </c>
     </row>
     <row r="97" spans="1:11">
-      <c r="A97" s="4"/>
-      <c r="B97" s="4" t="s">
+      <c r="A97" s="5"/>
+      <c r="B97" s="5" t="s">
         <v>126</v>
       </c>
       <c r="C97" t="s">
@@ -4070,8 +4070,8 @@
       </c>
     </row>
     <row r="98" spans="1:11">
-      <c r="A98" s="4"/>
-      <c r="B98" s="4"/>
+      <c r="A98" s="5"/>
+      <c r="B98" s="5"/>
       <c r="C98" t="s">
         <v>128</v>
       </c>
@@ -4101,8 +4101,8 @@
       </c>
     </row>
     <row r="99" spans="1:11">
-      <c r="A99" s="4"/>
-      <c r="B99" s="4"/>
+      <c r="A99" s="5"/>
+      <c r="B99" s="5"/>
       <c r="C99" t="s">
         <v>129</v>
       </c>
@@ -4132,8 +4132,8 @@
       </c>
     </row>
     <row r="100" spans="1:11">
-      <c r="A100" s="4"/>
-      <c r="B100" s="4"/>
+      <c r="A100" s="5"/>
+      <c r="B100" s="5"/>
       <c r="C100" t="s">
         <v>130</v>
       </c>
@@ -4163,8 +4163,8 @@
       </c>
     </row>
     <row r="101" spans="1:11">
-      <c r="A101" s="4"/>
-      <c r="B101" s="4"/>
+      <c r="A101" s="5"/>
+      <c r="B101" s="5"/>
       <c r="C101" t="s">
         <v>131</v>
       </c>
@@ -4194,10 +4194,10 @@
       </c>
     </row>
     <row r="102" spans="1:11">
-      <c r="A102" s="4" t="s">
+      <c r="A102" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="5" t="s">
         <v>133</v>
       </c>
       <c r="C102" s="2" t="s">
@@ -4229,8 +4229,8 @@
       </c>
     </row>
     <row r="103" spans="1:11">
-      <c r="A103" s="4"/>
-      <c r="B103" s="4"/>
+      <c r="A103" s="5"/>
+      <c r="B103" s="5"/>
       <c r="C103" s="2" t="s">
         <v>135</v>
       </c>
@@ -4260,8 +4260,8 @@
       </c>
     </row>
     <row r="104" spans="1:11">
-      <c r="A104" s="4"/>
-      <c r="B104" s="4"/>
+      <c r="A104" s="5"/>
+      <c r="B104" s="5"/>
       <c r="C104" s="2" t="s">
         <v>136</v>
       </c>
@@ -4291,8 +4291,8 @@
       </c>
     </row>
     <row r="105" spans="1:11">
-      <c r="A105" s="4"/>
-      <c r="B105" s="4"/>
+      <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
       <c r="C105" s="2" t="s">
         <v>137</v>
       </c>
@@ -4322,8 +4322,8 @@
       </c>
     </row>
     <row r="106" spans="1:11">
-      <c r="A106" s="4"/>
-      <c r="B106" s="4"/>
+      <c r="A106" s="5"/>
+      <c r="B106" s="5"/>
       <c r="C106" s="2" t="s">
         <v>138</v>
       </c>
@@ -4353,8 +4353,8 @@
       </c>
     </row>
     <row r="107" spans="1:11">
-      <c r="A107" s="4"/>
-      <c r="B107" s="4"/>
+      <c r="A107" s="5"/>
+      <c r="B107" s="5"/>
       <c r="C107" s="2" t="s">
         <v>139</v>
       </c>
@@ -4384,8 +4384,8 @@
       </c>
     </row>
     <row r="108" spans="1:11">
-      <c r="A108" s="4"/>
-      <c r="B108" s="4" t="s">
+      <c r="A108" s="5"/>
+      <c r="B108" s="5" t="s">
         <v>140</v>
       </c>
       <c r="C108" s="2" t="s">
@@ -4417,8 +4417,8 @@
       </c>
     </row>
     <row r="109" spans="1:11">
-      <c r="A109" s="4"/>
-      <c r="B109" s="4"/>
+      <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
       <c r="C109" s="2" t="s">
         <v>142</v>
       </c>
@@ -4448,8 +4448,8 @@
       </c>
     </row>
     <row r="110" spans="1:11">
-      <c r="A110" s="4"/>
-      <c r="B110" s="4"/>
+      <c r="A110" s="5"/>
+      <c r="B110" s="5"/>
       <c r="C110" s="2" t="s">
         <v>143</v>
       </c>
@@ -4479,8 +4479,8 @@
       </c>
     </row>
     <row r="111" spans="1:11">
-      <c r="A111" s="4"/>
-      <c r="B111" s="4" t="s">
+      <c r="A111" s="5"/>
+      <c r="B111" s="5" t="s">
         <v>144</v>
       </c>
       <c r="C111" s="2" t="s">
@@ -4512,8 +4512,8 @@
       </c>
     </row>
     <row r="112" spans="1:11">
-      <c r="A112" s="4"/>
-      <c r="B112" s="4"/>
+      <c r="A112" s="5"/>
+      <c r="B112" s="5"/>
       <c r="C112" s="2" t="s">
         <v>146</v>
       </c>
@@ -4543,8 +4543,8 @@
       </c>
     </row>
     <row r="113" spans="1:11">
-      <c r="A113" s="4"/>
-      <c r="B113" s="4"/>
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
       <c r="C113" s="2" t="s">
         <v>147</v>
       </c>
@@ -4574,8 +4574,8 @@
       </c>
     </row>
     <row r="114" spans="1:11">
-      <c r="A114" s="4"/>
-      <c r="B114" s="4"/>
+      <c r="A114" s="5"/>
+      <c r="B114" s="5"/>
       <c r="C114" s="2" t="s">
         <v>148</v>
       </c>
@@ -4605,8 +4605,8 @@
       </c>
     </row>
     <row r="115" spans="1:11">
-      <c r="A115" s="4"/>
-      <c r="B115" s="4"/>
+      <c r="A115" s="5"/>
+      <c r="B115" s="5"/>
       <c r="C115" s="2" t="s">
         <v>149</v>
       </c>
@@ -4636,8 +4636,8 @@
       </c>
     </row>
     <row r="116" spans="1:11">
-      <c r="A116" s="4"/>
-      <c r="B116" s="4" t="s">
+      <c r="A116" s="5"/>
+      <c r="B116" s="5" t="s">
         <v>150</v>
       </c>
       <c r="C116" s="2" t="s">
@@ -4669,8 +4669,8 @@
       </c>
     </row>
     <row r="117" spans="1:11">
-      <c r="A117" s="4"/>
-      <c r="B117" s="4"/>
+      <c r="A117" s="5"/>
+      <c r="B117" s="5"/>
       <c r="C117" s="2" t="s">
         <v>152</v>
       </c>
@@ -4700,8 +4700,8 @@
       </c>
     </row>
     <row r="118" spans="1:11">
-      <c r="A118" s="4"/>
-      <c r="B118" s="4"/>
+      <c r="A118" s="5"/>
+      <c r="B118" s="5"/>
       <c r="C118" s="2" t="s">
         <v>153</v>
       </c>
@@ -4731,8 +4731,8 @@
       </c>
     </row>
     <row r="119" spans="1:11">
-      <c r="A119" s="4"/>
-      <c r="B119" s="4"/>
+      <c r="A119" s="5"/>
+      <c r="B119" s="5"/>
       <c r="C119" s="2" t="s">
         <v>154</v>
       </c>
@@ -4762,8 +4762,8 @@
       </c>
     </row>
     <row r="120" spans="1:11">
-      <c r="A120" s="4"/>
-      <c r="B120" s="4"/>
+      <c r="A120" s="5"/>
+      <c r="B120" s="5"/>
       <c r="C120" s="2" t="s">
         <v>155</v>
       </c>
@@ -4793,8 +4793,8 @@
       </c>
     </row>
     <row r="121" spans="1:11">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
+      <c r="A121" s="5"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="2" t="s">
         <v>156</v>
       </c>
@@ -4824,8 +4824,8 @@
       </c>
     </row>
     <row r="122" spans="1:11">
-      <c r="A122" s="4"/>
-      <c r="B122" s="4"/>
+      <c r="A122" s="5"/>
+      <c r="B122" s="5"/>
       <c r="C122" s="2" t="s">
         <v>157</v>
       </c>
@@ -4855,8 +4855,8 @@
       </c>
     </row>
     <row r="123" spans="1:11">
-      <c r="A123" s="4"/>
-      <c r="B123" s="4" t="s">
+      <c r="A123" s="5"/>
+      <c r="B123" s="5" t="s">
         <v>158</v>
       </c>
       <c r="C123" s="2" t="s">
@@ -4888,8 +4888,8 @@
       </c>
     </row>
     <row r="124" spans="1:11">
-      <c r="A124" s="4"/>
-      <c r="B124" s="4"/>
+      <c r="A124" s="5"/>
+      <c r="B124" s="5"/>
       <c r="C124" s="2" t="s">
         <v>160</v>
       </c>
@@ -4919,8 +4919,8 @@
       </c>
     </row>
     <row r="125" spans="1:11">
-      <c r="A125" s="4"/>
-      <c r="B125" s="4"/>
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
       <c r="C125" s="2" t="s">
         <v>161</v>
       </c>
@@ -4950,8 +4950,8 @@
       </c>
     </row>
     <row r="126" spans="1:11">
-      <c r="A126" s="4"/>
-      <c r="B126" s="4"/>
+      <c r="A126" s="5"/>
+      <c r="B126" s="5"/>
       <c r="C126" s="2" t="s">
         <v>162</v>
       </c>
@@ -4981,8 +4981,8 @@
       </c>
     </row>
     <row r="127" spans="1:11">
-      <c r="A127" s="4"/>
-      <c r="B127" s="4"/>
+      <c r="A127" s="5"/>
+      <c r="B127" s="5"/>
       <c r="C127" s="2" t="s">
         <v>163</v>
       </c>
@@ -5012,132 +5012,348 @@
       </c>
     </row>
     <row r="128" spans="1:11">
-      <c r="A128" s="4" t="s">
+      <c r="A128" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B128" s="5" t="s">
         <v>165</v>
       </c>
       <c r="C128" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="129" spans="1:3">
-      <c r="A129" s="4"/>
-      <c r="B129" s="4"/>
+      <c r="D128">
+        <v>1</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>0</v>
+      </c>
+      <c r="G128">
+        <v>0</v>
+      </c>
+      <c r="H128">
+        <v>0</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11">
+      <c r="A129" s="5"/>
+      <c r="B129" s="5"/>
       <c r="C129" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="130" spans="1:3">
-      <c r="A130" s="4"/>
-      <c r="B130" s="4"/>
+      <c r="D129">
+        <v>1</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>0</v>
+      </c>
+      <c r="G129">
+        <v>0</v>
+      </c>
+      <c r="H129">
+        <v>0</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11">
+      <c r="A130" s="5"/>
+      <c r="B130" s="5"/>
       <c r="C130" s="3" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="131" spans="1:3">
-      <c r="A131" s="4" t="s">
+      <c r="D130">
+        <v>1</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>0</v>
+      </c>
+      <c r="G130">
+        <v>0</v>
+      </c>
+      <c r="H130">
+        <v>0</v>
+      </c>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11">
+      <c r="A131" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="4" t="s">
+      <c r="B131" s="5" t="s">
         <v>169</v>
       </c>
       <c r="C131" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131">
+        <v>1</v>
+      </c>
+      <c r="F131">
+        <v>1</v>
+      </c>
+      <c r="G131">
+        <v>0</v>
+      </c>
+      <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11">
+      <c r="A132" s="5"/>
+      <c r="B132" s="5"/>
       <c r="C132" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132">
+        <v>1</v>
+      </c>
+      <c r="F132">
+        <v>1</v>
+      </c>
+      <c r="G132">
+        <v>0</v>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11">
+      <c r="A133" s="5"/>
+      <c r="B133" s="5"/>
       <c r="C133" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
+      <c r="D133">
+        <v>1</v>
+      </c>
+      <c r="E133">
+        <v>1</v>
+      </c>
+      <c r="F133">
+        <v>1</v>
+      </c>
+      <c r="G133">
+        <v>1</v>
+      </c>
+      <c r="H133">
+        <v>1</v>
+      </c>
+      <c r="I133">
+        <v>1</v>
+      </c>
+      <c r="J133">
+        <v>1</v>
+      </c>
+      <c r="K133">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11">
+      <c r="A134" s="5"/>
+      <c r="B134" s="5"/>
       <c r="C134" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134">
+        <v>1</v>
+      </c>
+      <c r="F134">
+        <v>1</v>
+      </c>
+      <c r="G134">
+        <v>1</v>
+      </c>
+      <c r="H134">
+        <v>1</v>
+      </c>
+      <c r="I134">
+        <v>1</v>
+      </c>
+      <c r="J134">
+        <v>1</v>
+      </c>
+      <c r="K134">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11">
+      <c r="A135" s="5"/>
+      <c r="B135" s="5"/>
       <c r="C135" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="136" spans="1:3">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135">
+        <v>1</v>
+      </c>
+      <c r="F135">
+        <v>1</v>
+      </c>
+      <c r="G135">
+        <v>0</v>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11">
+      <c r="A136" s="5"/>
+      <c r="B136" s="5"/>
       <c r="C136" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="137" spans="1:3">
-      <c r="A137" s="4" t="s">
+      <c r="D136">
+        <v>1</v>
+      </c>
+      <c r="E136">
+        <v>1</v>
+      </c>
+      <c r="F136">
+        <v>1</v>
+      </c>
+      <c r="G136">
+        <v>0</v>
+      </c>
+      <c r="H136">
+        <v>0</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+      <c r="J136">
+        <v>0</v>
+      </c>
+      <c r="K136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11">
+      <c r="A137" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B137" s="4" t="s">
+      <c r="B137" s="5" t="s">
         <v>177</v>
       </c>
       <c r="C137" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
-      <c r="A138" s="4"/>
-      <c r="B138" s="4"/>
+    <row r="138" spans="1:11">
+      <c r="A138" s="5"/>
+      <c r="B138" s="5"/>
       <c r="C138" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
-      <c r="A139" s="4"/>
-      <c r="B139" s="4"/>
+    <row r="139" spans="1:11">
+      <c r="A139" s="5"/>
+      <c r="B139" s="5"/>
       <c r="C139" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
-      <c r="A140" s="4"/>
-      <c r="B140" s="4"/>
+    <row r="140" spans="1:11">
+      <c r="A140" s="5"/>
+      <c r="B140" s="5"/>
       <c r="C140" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
-      <c r="A141" s="4"/>
-      <c r="B141" s="4"/>
+    <row r="141" spans="1:11">
+      <c r="A141" s="5"/>
+      <c r="B141" s="5"/>
       <c r="C141" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
-      <c r="A142" s="4"/>
-      <c r="B142" s="4" t="s">
+    <row r="142" spans="1:11">
+      <c r="A142" s="5"/>
+      <c r="B142" s="5" t="s">
         <v>183</v>
       </c>
       <c r="C142" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
-      <c r="A143" s="4"/>
-      <c r="B143" s="4"/>
+    <row r="143" spans="1:11">
+      <c r="A143" s="5"/>
+      <c r="B143" s="5"/>
       <c r="C143" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" spans="1:11">
       <c r="A144" s="1" t="s">
         <v>164</v>
       </c>
@@ -5147,15 +5363,63 @@
       <c r="C144" t="s">
         <v>186</v>
       </c>
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
+        <v>1</v>
+      </c>
+      <c r="H144">
+        <v>1</v>
+      </c>
+      <c r="I144">
+        <v>1</v>
+      </c>
+      <c r="J144">
+        <v>1</v>
+      </c>
+      <c r="K144">
+        <v>0</v>
+      </c>
     </row>
     <row r="145" spans="3:3">
-      <c r="C145" s="5"/>
+      <c r="C145" s="4"/>
     </row>
     <row r="146" spans="3:3">
-      <c r="C146" s="5"/>
+      <c r="C146" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="A87:A101"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B87:B91"/>
+    <mergeCell ref="B92:B96"/>
+    <mergeCell ref="B97:B101"/>
     <mergeCell ref="A102:A127"/>
     <mergeCell ref="A128:A130"/>
     <mergeCell ref="A131:A136"/>
@@ -5169,30 +5433,6 @@
     <mergeCell ref="B131:B136"/>
     <mergeCell ref="B137:B141"/>
     <mergeCell ref="B142:B143"/>
-    <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A101"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B87:B91"/>
-    <mergeCell ref="B92:B96"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5200,26 +5440,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EC4E686503E2F943B8E5E5655A7FD1F0" ma:contentTypeVersion="10" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="f2732ee9c33e97baf8920e24934e29c2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36e2ff40-ab52-4240-babf-7476b65fdfdc" xmlns:ns3="d3830623-0ee5-4634-96e5-1fabe66116f4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2a88aeb4517fc5801f374367f5cb1408" ns2:_="" ns3:_="">
     <xsd:import namespace="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
@@ -5408,26 +5628,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
-    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90CF6C77-55D4-44ED-8F28-2A0B0624A3F2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5444,4 +5665,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
+    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add conversations endpoints tests
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Smart-University-Scheduler\helpers\db_seeder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3A858D-60E3-4B0F-AE8A-BF5C54CAA66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE114081-A896-470D-A399-790D93694E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6370" yWindow="-18960" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9240" yWindow="-21600" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -5308,6 +5308,30 @@
       <c r="C137" t="s">
         <v>178</v>
       </c>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>1</v>
+      </c>
+      <c r="F137">
+        <v>1</v>
+      </c>
+      <c r="G137">
+        <v>1</v>
+      </c>
+      <c r="H137">
+        <v>1</v>
+      </c>
+      <c r="I137">
+        <v>1</v>
+      </c>
+      <c r="J137">
+        <v>1</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
     </row>
     <row r="138" spans="1:11">
       <c r="A138" s="5"/>
@@ -5315,6 +5339,30 @@
       <c r="C138" t="s">
         <v>179</v>
       </c>
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>1</v>
+      </c>
+      <c r="F138">
+        <v>1</v>
+      </c>
+      <c r="G138">
+        <v>1</v>
+      </c>
+      <c r="H138">
+        <v>1</v>
+      </c>
+      <c r="I138">
+        <v>1</v>
+      </c>
+      <c r="J138">
+        <v>1</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
     </row>
     <row r="139" spans="1:11">
       <c r="A139" s="5"/>
@@ -5322,6 +5370,30 @@
       <c r="C139" t="s">
         <v>180</v>
       </c>
+      <c r="D139">
+        <v>1</v>
+      </c>
+      <c r="E139">
+        <v>1</v>
+      </c>
+      <c r="F139">
+        <v>1</v>
+      </c>
+      <c r="G139">
+        <v>1</v>
+      </c>
+      <c r="H139">
+        <v>1</v>
+      </c>
+      <c r="I139">
+        <v>1</v>
+      </c>
+      <c r="J139">
+        <v>1</v>
+      </c>
+      <c r="K139">
+        <v>0</v>
+      </c>
     </row>
     <row r="140" spans="1:11">
       <c r="A140" s="5"/>
@@ -5329,6 +5401,30 @@
       <c r="C140" t="s">
         <v>181</v>
       </c>
+      <c r="D140">
+        <v>1</v>
+      </c>
+      <c r="E140">
+        <v>1</v>
+      </c>
+      <c r="F140">
+        <v>1</v>
+      </c>
+      <c r="G140">
+        <v>1</v>
+      </c>
+      <c r="H140">
+        <v>1</v>
+      </c>
+      <c r="I140">
+        <v>1</v>
+      </c>
+      <c r="J140">
+        <v>1</v>
+      </c>
+      <c r="K140">
+        <v>0</v>
+      </c>
     </row>
     <row r="141" spans="1:11">
       <c r="A141" s="5"/>
@@ -5336,6 +5432,30 @@
       <c r="C141" t="s">
         <v>182</v>
       </c>
+      <c r="D141">
+        <v>1</v>
+      </c>
+      <c r="E141">
+        <v>1</v>
+      </c>
+      <c r="F141">
+        <v>1</v>
+      </c>
+      <c r="G141">
+        <v>1</v>
+      </c>
+      <c r="H141">
+        <v>1</v>
+      </c>
+      <c r="I141">
+        <v>1</v>
+      </c>
+      <c r="J141">
+        <v>1</v>
+      </c>
+      <c r="K141">
+        <v>0</v>
+      </c>
     </row>
     <row r="142" spans="1:11">
       <c r="A142" s="5"/>
@@ -5344,6 +5464,30 @@
       </c>
       <c r="C142" t="s">
         <v>184</v>
+      </c>
+      <c r="D142">
+        <v>1</v>
+      </c>
+      <c r="E142">
+        <v>1</v>
+      </c>
+      <c r="F142">
+        <v>1</v>
+      </c>
+      <c r="G142">
+        <v>1</v>
+      </c>
+      <c r="H142">
+        <v>1</v>
+      </c>
+      <c r="I142">
+        <v>1</v>
+      </c>
+      <c r="J142">
+        <v>1</v>
+      </c>
+      <c r="K142">
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:11">
@@ -5351,6 +5495,30 @@
       <c r="B143" s="5"/>
       <c r="C143" t="s">
         <v>185</v>
+      </c>
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143">
+        <v>1</v>
+      </c>
+      <c r="G143">
+        <v>1</v>
+      </c>
+      <c r="H143">
+        <v>1</v>
+      </c>
+      <c r="I143">
+        <v>1</v>
+      </c>
+      <c r="J143">
+        <v>1</v>
+      </c>
+      <c r="K143">
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">

</xml_diff>

<commit_message>
Filled excel file with roles and perms
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FCB22A-F8D1-4747-BE76-C5A0D56C2E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE6D5C1-5850-4799-8E3E-6CD3A8E2F55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -712,11 +712,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1046,10 +1046,10 @@
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
@@ -1081,8 +1081,8 @@
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -1112,8 +1112,8 @@
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
       <c r="C4" t="s">
         <v>13</v>
       </c>
@@ -1143,8 +1143,8 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
       <c r="C5" t="s">
         <v>14</v>
       </c>
@@ -1174,8 +1174,8 @@
       </c>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
       <c r="C6" t="s">
         <v>15</v>
       </c>
@@ -1205,8 +1205,8 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
@@ -1238,8 +1238,8 @@
       </c>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
       <c r="C8" t="s">
         <v>18</v>
       </c>
@@ -1269,8 +1269,8 @@
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -1300,8 +1300,8 @@
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
       <c r="C10" t="s">
         <v>20</v>
       </c>
@@ -1331,8 +1331,8 @@
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
       <c r="C11" t="s">
         <v>21</v>
       </c>
@@ -1362,8 +1362,8 @@
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C12" t="s">
@@ -1395,8 +1395,8 @@
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
       <c r="C13" t="s">
         <v>24</v>
       </c>
@@ -1426,8 +1426,8 @@
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
       <c r="C14" t="s">
         <v>25</v>
       </c>
@@ -1457,8 +1457,8 @@
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
       <c r="C15" t="s">
         <v>26</v>
       </c>
@@ -1488,8 +1488,8 @@
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
       <c r="C16" t="s">
         <v>27</v>
       </c>
@@ -1519,8 +1519,8 @@
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C17" t="s">
@@ -1552,8 +1552,8 @@
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
       <c r="C18" t="s">
         <v>30</v>
       </c>
@@ -1583,8 +1583,8 @@
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
       <c r="C19" t="s">
         <v>31</v>
       </c>
@@ -1614,8 +1614,8 @@
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
       <c r="C20" t="s">
         <v>32</v>
       </c>
@@ -1645,8 +1645,8 @@
       </c>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
       <c r="C21" t="s">
         <v>33</v>
       </c>
@@ -1676,8 +1676,8 @@
       </c>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C22" t="s">
@@ -1709,8 +1709,8 @@
       </c>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
       <c r="C23" t="s">
         <v>36</v>
       </c>
@@ -1740,8 +1740,8 @@
       </c>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
       <c r="C24" t="s">
         <v>37</v>
       </c>
@@ -1771,8 +1771,8 @@
       </c>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
       <c r="C25" t="s">
         <v>38</v>
       </c>
@@ -1802,8 +1802,8 @@
       </c>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
       <c r="C26" t="s">
         <v>39</v>
       </c>
@@ -1833,10 +1833,10 @@
       </c>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1868,8 +1868,8 @@
       </c>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
       <c r="C28" t="s">
         <v>43</v>
       </c>
@@ -1899,8 +1899,8 @@
       </c>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
       <c r="C29" t="s">
         <v>44</v>
       </c>
@@ -1930,8 +1930,8 @@
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
       <c r="C30" t="s">
         <v>45</v>
       </c>
@@ -1961,8 +1961,8 @@
       </c>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
       <c r="C31" t="s">
         <v>46</v>
       </c>
@@ -1992,8 +1992,8 @@
       </c>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4" t="s">
+      <c r="A32" s="5"/>
+      <c r="B32" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C32" t="s">
@@ -2025,8 +2025,8 @@
       </c>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
       <c r="C33" t="s">
         <v>49</v>
       </c>
@@ -2056,8 +2056,8 @@
       </c>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
       <c r="C34" t="s">
         <v>50</v>
       </c>
@@ -2087,8 +2087,8 @@
       </c>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
       <c r="C35" t="s">
         <v>51</v>
       </c>
@@ -2118,8 +2118,8 @@
       </c>
     </row>
     <row r="36" spans="1:11">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
       <c r="C36" t="s">
         <v>52</v>
       </c>
@@ -2149,8 +2149,8 @@
       </c>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4" t="s">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C37" t="s">
@@ -2182,8 +2182,8 @@
       </c>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
       <c r="C38" t="s">
         <v>55</v>
       </c>
@@ -2213,8 +2213,8 @@
       </c>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
       <c r="C39" t="s">
         <v>56</v>
       </c>
@@ -2244,8 +2244,8 @@
       </c>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="4"/>
-      <c r="B40" s="4"/>
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
       <c r="C40" t="s">
         <v>57</v>
       </c>
@@ -2275,8 +2275,8 @@
       </c>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
       <c r="C41" t="s">
         <v>58</v>
       </c>
@@ -2306,8 +2306,8 @@
       </c>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4" t="s">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C42" t="s">
@@ -2339,8 +2339,8 @@
       </c>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4"/>
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
       <c r="C43" t="s">
         <v>61</v>
       </c>
@@ -2370,8 +2370,8 @@
       </c>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
       <c r="C44" t="s">
         <v>62</v>
       </c>
@@ -2401,8 +2401,8 @@
       </c>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
       <c r="C45" t="s">
         <v>63</v>
       </c>
@@ -2432,8 +2432,8 @@
       </c>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
       <c r="C46" t="s">
         <v>64</v>
       </c>
@@ -2463,8 +2463,8 @@
       </c>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4" t="s">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
         <v>65</v>
       </c>
       <c r="C47" t="s">
@@ -2496,8 +2496,8 @@
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
       <c r="C48" t="s">
         <v>67</v>
       </c>
@@ -2527,8 +2527,8 @@
       </c>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
       <c r="C49" t="s">
         <v>68</v>
       </c>
@@ -2558,8 +2558,8 @@
       </c>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2589,8 +2589,8 @@
       </c>
     </row>
     <row r="51" spans="1:11">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
       <c r="C51" t="s">
         <v>70</v>
       </c>
@@ -2620,8 +2620,8 @@
       </c>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4" t="s">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C52" t="s">
@@ -2653,8 +2653,8 @@
       </c>
     </row>
     <row r="53" spans="1:11">
-      <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
       <c r="C53" t="s">
         <v>72</v>
       </c>
@@ -2684,8 +2684,8 @@
       </c>
     </row>
     <row r="54" spans="1:11">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
+      <c r="A54" s="5"/>
+      <c r="B54" s="5"/>
       <c r="C54" t="s">
         <v>73</v>
       </c>
@@ -2715,8 +2715,8 @@
       </c>
     </row>
     <row r="55" spans="1:11">
-      <c r="A55" s="4"/>
-      <c r="B55" s="4"/>
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
       <c r="C55" t="s">
         <v>74</v>
       </c>
@@ -2746,8 +2746,8 @@
       </c>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
       <c r="C56" t="s">
         <v>75</v>
       </c>
@@ -2777,8 +2777,8 @@
       </c>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4" t="s">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C57" t="s">
@@ -2810,8 +2810,8 @@
       </c>
     </row>
     <row r="58" spans="1:11">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
       <c r="C58" t="s">
         <v>78</v>
       </c>
@@ -2841,8 +2841,8 @@
       </c>
     </row>
     <row r="59" spans="1:11">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
       <c r="C59" t="s">
         <v>79</v>
       </c>
@@ -2872,8 +2872,8 @@
       </c>
     </row>
     <row r="60" spans="1:11">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
       <c r="C60" t="s">
         <v>80</v>
       </c>
@@ -2903,8 +2903,8 @@
       </c>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
       <c r="C61" t="s">
         <v>81</v>
       </c>
@@ -2934,8 +2934,8 @@
       </c>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="4"/>
-      <c r="B62" s="4" t="s">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5" t="s">
         <v>82</v>
       </c>
       <c r="C62" t="s">
@@ -2967,8 +2967,8 @@
       </c>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="4"/>
-      <c r="B63" s="4"/>
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
       <c r="C63" t="s">
         <v>84</v>
       </c>
@@ -2998,8 +2998,8 @@
       </c>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="4"/>
-      <c r="B64" s="4"/>
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
       <c r="C64" t="s">
         <v>85</v>
       </c>
@@ -3029,8 +3029,8 @@
       </c>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="4"/>
-      <c r="B65" s="4"/>
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
       <c r="C65" t="s">
         <v>86</v>
       </c>
@@ -3060,8 +3060,8 @@
       </c>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="4"/>
-      <c r="B66" s="4"/>
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
       <c r="C66" t="s">
         <v>87</v>
       </c>
@@ -3091,10 +3091,10 @@
       </c>
     </row>
     <row r="67" spans="1:11">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C67" t="s">
@@ -3126,8 +3126,8 @@
       </c>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="4"/>
-      <c r="B68" s="4"/>
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
       <c r="C68" t="s">
         <v>91</v>
       </c>
@@ -3157,8 +3157,8 @@
       </c>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="4"/>
-      <c r="B69" s="4"/>
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
       <c r="C69" t="s">
         <v>92</v>
       </c>
@@ -3188,8 +3188,8 @@
       </c>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="4"/>
-      <c r="B70" s="4"/>
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
       <c r="C70" t="s">
         <v>93</v>
       </c>
@@ -3219,8 +3219,8 @@
       </c>
     </row>
     <row r="71" spans="1:11">
-      <c r="A71" s="4"/>
-      <c r="B71" s="4"/>
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
       <c r="C71" t="s">
         <v>94</v>
       </c>
@@ -3250,8 +3250,8 @@
       </c>
     </row>
     <row r="72" spans="1:11">
-      <c r="A72" s="4"/>
-      <c r="B72" s="4" t="s">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5" t="s">
         <v>95</v>
       </c>
       <c r="C72" t="s">
@@ -3283,8 +3283,8 @@
       </c>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="4"/>
-      <c r="B73" s="4"/>
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
       <c r="C73" t="s">
         <v>97</v>
       </c>
@@ -3314,8 +3314,8 @@
       </c>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="4"/>
-      <c r="B74" s="4"/>
+      <c r="A74" s="5"/>
+      <c r="B74" s="5"/>
       <c r="C74" t="s">
         <v>98</v>
       </c>
@@ -3345,8 +3345,8 @@
       </c>
     </row>
     <row r="75" spans="1:11">
-      <c r="A75" s="4"/>
-      <c r="B75" s="4"/>
+      <c r="A75" s="5"/>
+      <c r="B75" s="5"/>
       <c r="C75" t="s">
         <v>99</v>
       </c>
@@ -3376,8 +3376,8 @@
       </c>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="4"/>
-      <c r="B76" s="4"/>
+      <c r="A76" s="5"/>
+      <c r="B76" s="5"/>
       <c r="C76" t="s">
         <v>100</v>
       </c>
@@ -3407,8 +3407,8 @@
       </c>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="4"/>
-      <c r="B77" s="4" t="s">
+      <c r="A77" s="5"/>
+      <c r="B77" s="5" t="s">
         <v>101</v>
       </c>
       <c r="C77" t="s">
@@ -3440,8 +3440,8 @@
       </c>
     </row>
     <row r="78" spans="1:11">
-      <c r="A78" s="4"/>
-      <c r="B78" s="4"/>
+      <c r="A78" s="5"/>
+      <c r="B78" s="5"/>
       <c r="C78" t="s">
         <v>103</v>
       </c>
@@ -3471,8 +3471,8 @@
       </c>
     </row>
     <row r="79" spans="1:11">
-      <c r="A79" s="4"/>
-      <c r="B79" s="4"/>
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
       <c r="C79" t="s">
         <v>104</v>
       </c>
@@ -3502,8 +3502,8 @@
       </c>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="4"/>
-      <c r="B80" s="4"/>
+      <c r="A80" s="5"/>
+      <c r="B80" s="5"/>
       <c r="C80" t="s">
         <v>105</v>
       </c>
@@ -3533,8 +3533,8 @@
       </c>
     </row>
     <row r="81" spans="1:11">
-      <c r="A81" s="4"/>
-      <c r="B81" s="4"/>
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
       <c r="C81" t="s">
         <v>106</v>
       </c>
@@ -3564,8 +3564,8 @@
       </c>
     </row>
     <row r="82" spans="1:11">
-      <c r="A82" s="4"/>
-      <c r="B82" s="4" t="s">
+      <c r="A82" s="5"/>
+      <c r="B82" s="5" t="s">
         <v>107</v>
       </c>
       <c r="C82" t="s">
@@ -3597,8 +3597,8 @@
       </c>
     </row>
     <row r="83" spans="1:11">
-      <c r="A83" s="4"/>
-      <c r="B83" s="4"/>
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
       <c r="C83" t="s">
         <v>109</v>
       </c>
@@ -3628,8 +3628,8 @@
       </c>
     </row>
     <row r="84" spans="1:11">
-      <c r="A84" s="4"/>
-      <c r="B84" s="4"/>
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
       <c r="C84" t="s">
         <v>110</v>
       </c>
@@ -3659,8 +3659,8 @@
       </c>
     </row>
     <row r="85" spans="1:11">
-      <c r="A85" s="4"/>
-      <c r="B85" s="4"/>
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
       <c r="C85" t="s">
         <v>111</v>
       </c>
@@ -3690,8 +3690,8 @@
       </c>
     </row>
     <row r="86" spans="1:11">
-      <c r="A86" s="4"/>
-      <c r="B86" s="4"/>
+      <c r="A86" s="5"/>
+      <c r="B86" s="5"/>
       <c r="C86" t="s">
         <v>112</v>
       </c>
@@ -3721,10 +3721,10 @@
       </c>
     </row>
     <row r="87" spans="1:11">
-      <c r="A87" s="4" t="s">
+      <c r="A87" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="B87" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C87" t="s">
@@ -3756,8 +3756,8 @@
       </c>
     </row>
     <row r="88" spans="1:11">
-      <c r="A88" s="4"/>
-      <c r="B88" s="4"/>
+      <c r="A88" s="5"/>
+      <c r="B88" s="5"/>
       <c r="C88" t="s">
         <v>116</v>
       </c>
@@ -3787,8 +3787,8 @@
       </c>
     </row>
     <row r="89" spans="1:11">
-      <c r="A89" s="4"/>
-      <c r="B89" s="4"/>
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
       <c r="C89" t="s">
         <v>117</v>
       </c>
@@ -3818,8 +3818,8 @@
       </c>
     </row>
     <row r="90" spans="1:11">
-      <c r="A90" s="4"/>
-      <c r="B90" s="4"/>
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
       <c r="C90" t="s">
         <v>118</v>
       </c>
@@ -3849,8 +3849,8 @@
       </c>
     </row>
     <row r="91" spans="1:11">
-      <c r="A91" s="4"/>
-      <c r="B91" s="4"/>
+      <c r="A91" s="5"/>
+      <c r="B91" s="5"/>
       <c r="C91" t="s">
         <v>119</v>
       </c>
@@ -3880,8 +3880,8 @@
       </c>
     </row>
     <row r="92" spans="1:11">
-      <c r="A92" s="4"/>
-      <c r="B92" s="4" t="s">
+      <c r="A92" s="5"/>
+      <c r="B92" s="5" t="s">
         <v>120</v>
       </c>
       <c r="C92" t="s">
@@ -3913,8 +3913,8 @@
       </c>
     </row>
     <row r="93" spans="1:11">
-      <c r="A93" s="4"/>
-      <c r="B93" s="4"/>
+      <c r="A93" s="5"/>
+      <c r="B93" s="5"/>
       <c r="C93" t="s">
         <v>122</v>
       </c>
@@ -3944,8 +3944,8 @@
       </c>
     </row>
     <row r="94" spans="1:11">
-      <c r="A94" s="4"/>
-      <c r="B94" s="4"/>
+      <c r="A94" s="5"/>
+      <c r="B94" s="5"/>
       <c r="C94" t="s">
         <v>123</v>
       </c>
@@ -3975,8 +3975,8 @@
       </c>
     </row>
     <row r="95" spans="1:11">
-      <c r="A95" s="4"/>
-      <c r="B95" s="4"/>
+      <c r="A95" s="5"/>
+      <c r="B95" s="5"/>
       <c r="C95" t="s">
         <v>124</v>
       </c>
@@ -4006,8 +4006,8 @@
       </c>
     </row>
     <row r="96" spans="1:11">
-      <c r="A96" s="4"/>
-      <c r="B96" s="4"/>
+      <c r="A96" s="5"/>
+      <c r="B96" s="5"/>
       <c r="C96" t="s">
         <v>125</v>
       </c>
@@ -4037,8 +4037,8 @@
       </c>
     </row>
     <row r="97" spans="1:11">
-      <c r="A97" s="4"/>
-      <c r="B97" s="4" t="s">
+      <c r="A97" s="5"/>
+      <c r="B97" s="5" t="s">
         <v>126</v>
       </c>
       <c r="C97" t="s">
@@ -4070,8 +4070,8 @@
       </c>
     </row>
     <row r="98" spans="1:11">
-      <c r="A98" s="4"/>
-      <c r="B98" s="4"/>
+      <c r="A98" s="5"/>
+      <c r="B98" s="5"/>
       <c r="C98" t="s">
         <v>128</v>
       </c>
@@ -4101,8 +4101,8 @@
       </c>
     </row>
     <row r="99" spans="1:11">
-      <c r="A99" s="4"/>
-      <c r="B99" s="4"/>
+      <c r="A99" s="5"/>
+      <c r="B99" s="5"/>
       <c r="C99" t="s">
         <v>129</v>
       </c>
@@ -4132,8 +4132,8 @@
       </c>
     </row>
     <row r="100" spans="1:11">
-      <c r="A100" s="4"/>
-      <c r="B100" s="4"/>
+      <c r="A100" s="5"/>
+      <c r="B100" s="5"/>
       <c r="C100" t="s">
         <v>130</v>
       </c>
@@ -4163,8 +4163,8 @@
       </c>
     </row>
     <row r="101" spans="1:11">
-      <c r="A101" s="4"/>
-      <c r="B101" s="4"/>
+      <c r="A101" s="5"/>
+      <c r="B101" s="5"/>
       <c r="C101" t="s">
         <v>131</v>
       </c>
@@ -4194,10 +4194,10 @@
       </c>
     </row>
     <row r="102" spans="1:11">
-      <c r="A102" s="4" t="s">
+      <c r="A102" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="5" t="s">
         <v>133</v>
       </c>
       <c r="C102" s="2" t="s">
@@ -4229,8 +4229,8 @@
       </c>
     </row>
     <row r="103" spans="1:11">
-      <c r="A103" s="4"/>
-      <c r="B103" s="4"/>
+      <c r="A103" s="5"/>
+      <c r="B103" s="5"/>
       <c r="C103" s="2" t="s">
         <v>135</v>
       </c>
@@ -4260,8 +4260,8 @@
       </c>
     </row>
     <row r="104" spans="1:11">
-      <c r="A104" s="4"/>
-      <c r="B104" s="4"/>
+      <c r="A104" s="5"/>
+      <c r="B104" s="5"/>
       <c r="C104" s="2" t="s">
         <v>136</v>
       </c>
@@ -4291,8 +4291,8 @@
       </c>
     </row>
     <row r="105" spans="1:11">
-      <c r="A105" s="4"/>
-      <c r="B105" s="4"/>
+      <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
       <c r="C105" s="2" t="s">
         <v>137</v>
       </c>
@@ -4322,8 +4322,8 @@
       </c>
     </row>
     <row r="106" spans="1:11">
-      <c r="A106" s="4"/>
-      <c r="B106" s="4"/>
+      <c r="A106" s="5"/>
+      <c r="B106" s="5"/>
       <c r="C106" s="2" t="s">
         <v>138</v>
       </c>
@@ -4353,8 +4353,8 @@
       </c>
     </row>
     <row r="107" spans="1:11">
-      <c r="A107" s="4"/>
-      <c r="B107" s="4"/>
+      <c r="A107" s="5"/>
+      <c r="B107" s="5"/>
       <c r="C107" s="2" t="s">
         <v>139</v>
       </c>
@@ -4384,8 +4384,8 @@
       </c>
     </row>
     <row r="108" spans="1:11">
-      <c r="A108" s="4"/>
-      <c r="B108" s="4" t="s">
+      <c r="A108" s="5"/>
+      <c r="B108" s="5" t="s">
         <v>140</v>
       </c>
       <c r="C108" s="2" t="s">
@@ -4417,8 +4417,8 @@
       </c>
     </row>
     <row r="109" spans="1:11">
-      <c r="A109" s="4"/>
-      <c r="B109" s="4"/>
+      <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
       <c r="C109" s="2" t="s">
         <v>142</v>
       </c>
@@ -4448,8 +4448,8 @@
       </c>
     </row>
     <row r="110" spans="1:11">
-      <c r="A110" s="4"/>
-      <c r="B110" s="4"/>
+      <c r="A110" s="5"/>
+      <c r="B110" s="5"/>
       <c r="C110" s="2" t="s">
         <v>143</v>
       </c>
@@ -4479,8 +4479,8 @@
       </c>
     </row>
     <row r="111" spans="1:11">
-      <c r="A111" s="4"/>
-      <c r="B111" s="4" t="s">
+      <c r="A111" s="5"/>
+      <c r="B111" s="5" t="s">
         <v>144</v>
       </c>
       <c r="C111" s="2" t="s">
@@ -4512,8 +4512,8 @@
       </c>
     </row>
     <row r="112" spans="1:11">
-      <c r="A112" s="4"/>
-      <c r="B112" s="4"/>
+      <c r="A112" s="5"/>
+      <c r="B112" s="5"/>
       <c r="C112" s="2" t="s">
         <v>146</v>
       </c>
@@ -4543,8 +4543,8 @@
       </c>
     </row>
     <row r="113" spans="1:11">
-      <c r="A113" s="4"/>
-      <c r="B113" s="4"/>
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
       <c r="C113" s="2" t="s">
         <v>147</v>
       </c>
@@ -4574,8 +4574,8 @@
       </c>
     </row>
     <row r="114" spans="1:11">
-      <c r="A114" s="4"/>
-      <c r="B114" s="4"/>
+      <c r="A114" s="5"/>
+      <c r="B114" s="5"/>
       <c r="C114" s="2" t="s">
         <v>148</v>
       </c>
@@ -4605,8 +4605,8 @@
       </c>
     </row>
     <row r="115" spans="1:11">
-      <c r="A115" s="4"/>
-      <c r="B115" s="4"/>
+      <c r="A115" s="5"/>
+      <c r="B115" s="5"/>
       <c r="C115" s="2" t="s">
         <v>149</v>
       </c>
@@ -4636,8 +4636,8 @@
       </c>
     </row>
     <row r="116" spans="1:11">
-      <c r="A116" s="4"/>
-      <c r="B116" s="4" t="s">
+      <c r="A116" s="5"/>
+      <c r="B116" s="5" t="s">
         <v>150</v>
       </c>
       <c r="C116" s="2" t="s">
@@ -4669,8 +4669,8 @@
       </c>
     </row>
     <row r="117" spans="1:11">
-      <c r="A117" s="4"/>
-      <c r="B117" s="4"/>
+      <c r="A117" s="5"/>
+      <c r="B117" s="5"/>
       <c r="C117" s="2" t="s">
         <v>152</v>
       </c>
@@ -4700,8 +4700,8 @@
       </c>
     </row>
     <row r="118" spans="1:11">
-      <c r="A118" s="4"/>
-      <c r="B118" s="4"/>
+      <c r="A118" s="5"/>
+      <c r="B118" s="5"/>
       <c r="C118" s="2" t="s">
         <v>153</v>
       </c>
@@ -4731,8 +4731,8 @@
       </c>
     </row>
     <row r="119" spans="1:11">
-      <c r="A119" s="4"/>
-      <c r="B119" s="4"/>
+      <c r="A119" s="5"/>
+      <c r="B119" s="5"/>
       <c r="C119" s="2" t="s">
         <v>154</v>
       </c>
@@ -4762,8 +4762,8 @@
       </c>
     </row>
     <row r="120" spans="1:11">
-      <c r="A120" s="4"/>
-      <c r="B120" s="4"/>
+      <c r="A120" s="5"/>
+      <c r="B120" s="5"/>
       <c r="C120" s="2" t="s">
         <v>155</v>
       </c>
@@ -4793,8 +4793,8 @@
       </c>
     </row>
     <row r="121" spans="1:11">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
+      <c r="A121" s="5"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="2" t="s">
         <v>156</v>
       </c>
@@ -4824,8 +4824,8 @@
       </c>
     </row>
     <row r="122" spans="1:11">
-      <c r="A122" s="4"/>
-      <c r="B122" s="4"/>
+      <c r="A122" s="5"/>
+      <c r="B122" s="5"/>
       <c r="C122" s="2" t="s">
         <v>157</v>
       </c>
@@ -4855,8 +4855,8 @@
       </c>
     </row>
     <row r="123" spans="1:11">
-      <c r="A123" s="4"/>
-      <c r="B123" s="4" t="s">
+      <c r="A123" s="5"/>
+      <c r="B123" s="5" t="s">
         <v>158</v>
       </c>
       <c r="C123" s="2" t="s">
@@ -4888,8 +4888,8 @@
       </c>
     </row>
     <row r="124" spans="1:11">
-      <c r="A124" s="4"/>
-      <c r="B124" s="4"/>
+      <c r="A124" s="5"/>
+      <c r="B124" s="5"/>
       <c r="C124" s="2" t="s">
         <v>160</v>
       </c>
@@ -4919,8 +4919,8 @@
       </c>
     </row>
     <row r="125" spans="1:11">
-      <c r="A125" s="4"/>
-      <c r="B125" s="4"/>
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
       <c r="C125" s="2" t="s">
         <v>161</v>
       </c>
@@ -4950,8 +4950,8 @@
       </c>
     </row>
     <row r="126" spans="1:11">
-      <c r="A126" s="4"/>
-      <c r="B126" s="4"/>
+      <c r="A126" s="5"/>
+      <c r="B126" s="5"/>
       <c r="C126" s="2" t="s">
         <v>162</v>
       </c>
@@ -4981,8 +4981,8 @@
       </c>
     </row>
     <row r="127" spans="1:11">
-      <c r="A127" s="4"/>
-      <c r="B127" s="4"/>
+      <c r="A127" s="5"/>
+      <c r="B127" s="5"/>
       <c r="C127" s="2" t="s">
         <v>163</v>
       </c>
@@ -5012,132 +5012,516 @@
       </c>
     </row>
     <row r="128" spans="1:11">
-      <c r="A128" s="4" t="s">
+      <c r="A128" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B128" s="5" t="s">
         <v>165</v>
       </c>
       <c r="C128" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="129" spans="1:3">
-      <c r="A129" s="4"/>
-      <c r="B129" s="4"/>
+      <c r="D128">
+        <v>1</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>0</v>
+      </c>
+      <c r="G128">
+        <v>0</v>
+      </c>
+      <c r="H128">
+        <v>0</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11">
+      <c r="A129" s="5"/>
+      <c r="B129" s="5"/>
       <c r="C129" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="130" spans="1:3">
-      <c r="A130" s="4"/>
-      <c r="B130" s="4"/>
+      <c r="D129">
+        <v>1</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>0</v>
+      </c>
+      <c r="G129">
+        <v>0</v>
+      </c>
+      <c r="H129">
+        <v>0</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11">
+      <c r="A130" s="5"/>
+      <c r="B130" s="5"/>
       <c r="C130" s="3" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="131" spans="1:3">
-      <c r="A131" s="4" t="s">
+      <c r="D130">
+        <v>1</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>0</v>
+      </c>
+      <c r="G130">
+        <v>0</v>
+      </c>
+      <c r="H130">
+        <v>0</v>
+      </c>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11">
+      <c r="A131" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="4" t="s">
+      <c r="B131" s="5" t="s">
         <v>169</v>
       </c>
       <c r="C131" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+      <c r="F131">
+        <v>0</v>
+      </c>
+      <c r="G131">
+        <v>0</v>
+      </c>
+      <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11">
+      <c r="A132" s="5"/>
+      <c r="B132" s="5"/>
       <c r="C132" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+      <c r="F132">
+        <v>0</v>
+      </c>
+      <c r="G132">
+        <v>0</v>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11">
+      <c r="A133" s="5"/>
+      <c r="B133" s="5"/>
       <c r="C133" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
+      <c r="D133">
+        <v>1</v>
+      </c>
+      <c r="E133">
+        <v>0</v>
+      </c>
+      <c r="F133">
+        <v>0</v>
+      </c>
+      <c r="G133">
+        <v>0</v>
+      </c>
+      <c r="H133">
+        <v>0</v>
+      </c>
+      <c r="I133">
+        <v>0</v>
+      </c>
+      <c r="J133">
+        <v>0</v>
+      </c>
+      <c r="K133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11">
+      <c r="A134" s="5"/>
+      <c r="B134" s="5"/>
       <c r="C134" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134">
+        <v>0</v>
+      </c>
+      <c r="F134">
+        <v>0</v>
+      </c>
+      <c r="G134">
+        <v>0</v>
+      </c>
+      <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+      <c r="J134">
+        <v>0</v>
+      </c>
+      <c r="K134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11">
+      <c r="A135" s="5"/>
+      <c r="B135" s="5"/>
       <c r="C135" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="136" spans="1:3">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135">
+        <v>0</v>
+      </c>
+      <c r="F135">
+        <v>0</v>
+      </c>
+      <c r="G135">
+        <v>0</v>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11">
+      <c r="A136" s="5"/>
+      <c r="B136" s="5"/>
       <c r="C136" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="137" spans="1:3">
-      <c r="A137" s="4" t="s">
+      <c r="D136">
+        <v>1</v>
+      </c>
+      <c r="E136">
+        <v>0</v>
+      </c>
+      <c r="F136">
+        <v>0</v>
+      </c>
+      <c r="G136">
+        <v>0</v>
+      </c>
+      <c r="H136">
+        <v>0</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+      <c r="J136">
+        <v>0</v>
+      </c>
+      <c r="K136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11">
+      <c r="A137" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B137" s="4" t="s">
+      <c r="B137" s="5" t="s">
         <v>177</v>
       </c>
       <c r="C137" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="138" spans="1:3">
-      <c r="A138" s="4"/>
-      <c r="B138" s="4"/>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>1</v>
+      </c>
+      <c r="F137">
+        <v>1</v>
+      </c>
+      <c r="G137">
+        <v>1</v>
+      </c>
+      <c r="H137">
+        <v>1</v>
+      </c>
+      <c r="I137">
+        <v>1</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11">
+      <c r="A138" s="5"/>
+      <c r="B138" s="5"/>
       <c r="C138" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="139" spans="1:3">
-      <c r="A139" s="4"/>
-      <c r="B139" s="4"/>
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11">
+      <c r="A139" s="5"/>
+      <c r="B139" s="5"/>
       <c r="C139" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="140" spans="1:3">
-      <c r="A140" s="4"/>
-      <c r="B140" s="4"/>
+      <c r="D139">
+        <v>1</v>
+      </c>
+      <c r="E139">
+        <v>1</v>
+      </c>
+      <c r="F139">
+        <v>1</v>
+      </c>
+      <c r="G139">
+        <v>1</v>
+      </c>
+      <c r="H139">
+        <v>1</v>
+      </c>
+      <c r="I139">
+        <v>1</v>
+      </c>
+      <c r="J139">
+        <v>0</v>
+      </c>
+      <c r="K139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11">
+      <c r="A140" s="5"/>
+      <c r="B140" s="5"/>
       <c r="C140" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="141" spans="1:3">
-      <c r="A141" s="4"/>
-      <c r="B141" s="4"/>
+      <c r="D140">
+        <v>1</v>
+      </c>
+      <c r="E140">
+        <v>1</v>
+      </c>
+      <c r="F140">
+        <v>1</v>
+      </c>
+      <c r="G140">
+        <v>1</v>
+      </c>
+      <c r="H140">
+        <v>1</v>
+      </c>
+      <c r="I140">
+        <v>1</v>
+      </c>
+      <c r="J140">
+        <v>0</v>
+      </c>
+      <c r="K140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11">
+      <c r="A141" s="5"/>
+      <c r="B141" s="5"/>
       <c r="C141" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="142" spans="1:3">
-      <c r="A142" s="4"/>
-      <c r="B142" s="4" t="s">
+      <c r="D141">
+        <v>1</v>
+      </c>
+      <c r="E141">
+        <v>1</v>
+      </c>
+      <c r="F141">
+        <v>1</v>
+      </c>
+      <c r="G141">
+        <v>1</v>
+      </c>
+      <c r="H141">
+        <v>1</v>
+      </c>
+      <c r="I141">
+        <v>1</v>
+      </c>
+      <c r="J141">
+        <v>0</v>
+      </c>
+      <c r="K141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11">
+      <c r="A142" s="5"/>
+      <c r="B142" s="5" t="s">
         <v>183</v>
       </c>
       <c r="C142" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" s="4"/>
-      <c r="B143" s="4"/>
+      <c r="D142">
+        <v>1</v>
+      </c>
+      <c r="E142">
+        <v>1</v>
+      </c>
+      <c r="F142">
+        <v>1</v>
+      </c>
+      <c r="G142">
+        <v>1</v>
+      </c>
+      <c r="H142">
+        <v>1</v>
+      </c>
+      <c r="I142">
+        <v>1</v>
+      </c>
+      <c r="J142">
+        <v>0</v>
+      </c>
+      <c r="K142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11">
+      <c r="A143" s="5"/>
+      <c r="B143" s="5"/>
       <c r="C143" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="144" spans="1:3">
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143">
+        <v>1</v>
+      </c>
+      <c r="G143">
+        <v>1</v>
+      </c>
+      <c r="H143">
+        <v>1</v>
+      </c>
+      <c r="I143">
+        <v>1</v>
+      </c>
+      <c r="J143">
+        <v>0</v>
+      </c>
+      <c r="K143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11">
       <c r="A144" s="1" t="s">
         <v>164</v>
       </c>
@@ -5147,15 +5531,63 @@
       <c r="C144" t="s">
         <v>186</v>
       </c>
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
+        <v>1</v>
+      </c>
+      <c r="H144">
+        <v>1</v>
+      </c>
+      <c r="I144">
+        <v>1</v>
+      </c>
+      <c r="J144">
+        <v>1</v>
+      </c>
+      <c r="K144">
+        <v>1</v>
+      </c>
     </row>
     <row r="145" spans="3:3">
-      <c r="C145" s="5"/>
+      <c r="C145" s="4"/>
     </row>
     <row r="146" spans="3:3">
-      <c r="C146" s="5"/>
+      <c r="C146" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="A87:A101"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B87:B91"/>
+    <mergeCell ref="B92:B96"/>
+    <mergeCell ref="B97:B101"/>
     <mergeCell ref="A102:A127"/>
     <mergeCell ref="A128:A130"/>
     <mergeCell ref="A131:A136"/>
@@ -5169,30 +5601,6 @@
     <mergeCell ref="B131:B136"/>
     <mergeCell ref="B137:B141"/>
     <mergeCell ref="B142:B143"/>
-    <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A101"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B87:B91"/>
-    <mergeCell ref="B92:B96"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5200,6 +5608,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5208,15 +5625,6 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5409,20 +5817,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Data generators perms fix and academic calendar (#257)
* Filled excel file with roles and perms

* Added academic_calendar to seeder
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FCB22A-F8D1-4747-BE76-C5A0D56C2E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE6D5C1-5850-4799-8E3E-6CD3A8E2F55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -712,11 +712,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1046,10 +1046,10 @@
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
@@ -1081,8 +1081,8 @@
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -1112,8 +1112,8 @@
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
       <c r="C4" t="s">
         <v>13</v>
       </c>
@@ -1143,8 +1143,8 @@
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
       <c r="C5" t="s">
         <v>14</v>
       </c>
@@ -1174,8 +1174,8 @@
       </c>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
       <c r="C6" t="s">
         <v>15</v>
       </c>
@@ -1205,8 +1205,8 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
@@ -1238,8 +1238,8 @@
       </c>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
       <c r="C8" t="s">
         <v>18</v>
       </c>
@@ -1269,8 +1269,8 @@
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -1300,8 +1300,8 @@
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
       <c r="C10" t="s">
         <v>20</v>
       </c>
@@ -1331,8 +1331,8 @@
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
       <c r="C11" t="s">
         <v>21</v>
       </c>
@@ -1362,8 +1362,8 @@
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C12" t="s">
@@ -1395,8 +1395,8 @@
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
       <c r="C13" t="s">
         <v>24</v>
       </c>
@@ -1426,8 +1426,8 @@
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
       <c r="C14" t="s">
         <v>25</v>
       </c>
@@ -1457,8 +1457,8 @@
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
       <c r="C15" t="s">
         <v>26</v>
       </c>
@@ -1488,8 +1488,8 @@
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
       <c r="C16" t="s">
         <v>27</v>
       </c>
@@ -1519,8 +1519,8 @@
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C17" t="s">
@@ -1552,8 +1552,8 @@
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
       <c r="C18" t="s">
         <v>30</v>
       </c>
@@ -1583,8 +1583,8 @@
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
       <c r="C19" t="s">
         <v>31</v>
       </c>
@@ -1614,8 +1614,8 @@
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
       <c r="C20" t="s">
         <v>32</v>
       </c>
@@ -1645,8 +1645,8 @@
       </c>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
       <c r="C21" t="s">
         <v>33</v>
       </c>
@@ -1676,8 +1676,8 @@
       </c>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C22" t="s">
@@ -1709,8 +1709,8 @@
       </c>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
       <c r="C23" t="s">
         <v>36</v>
       </c>
@@ -1740,8 +1740,8 @@
       </c>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
       <c r="C24" t="s">
         <v>37</v>
       </c>
@@ -1771,8 +1771,8 @@
       </c>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
       <c r="C25" t="s">
         <v>38</v>
       </c>
@@ -1802,8 +1802,8 @@
       </c>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
       <c r="C26" t="s">
         <v>39</v>
       </c>
@@ -1833,10 +1833,10 @@
       </c>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1868,8 +1868,8 @@
       </c>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
       <c r="C28" t="s">
         <v>43</v>
       </c>
@@ -1899,8 +1899,8 @@
       </c>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
       <c r="C29" t="s">
         <v>44</v>
       </c>
@@ -1930,8 +1930,8 @@
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
       <c r="C30" t="s">
         <v>45</v>
       </c>
@@ -1961,8 +1961,8 @@
       </c>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
       <c r="C31" t="s">
         <v>46</v>
       </c>
@@ -1992,8 +1992,8 @@
       </c>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4" t="s">
+      <c r="A32" s="5"/>
+      <c r="B32" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C32" t="s">
@@ -2025,8 +2025,8 @@
       </c>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
       <c r="C33" t="s">
         <v>49</v>
       </c>
@@ -2056,8 +2056,8 @@
       </c>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
       <c r="C34" t="s">
         <v>50</v>
       </c>
@@ -2087,8 +2087,8 @@
       </c>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
       <c r="C35" t="s">
         <v>51</v>
       </c>
@@ -2118,8 +2118,8 @@
       </c>
     </row>
     <row r="36" spans="1:11">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
       <c r="C36" t="s">
         <v>52</v>
       </c>
@@ -2149,8 +2149,8 @@
       </c>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4" t="s">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C37" t="s">
@@ -2182,8 +2182,8 @@
       </c>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
       <c r="C38" t="s">
         <v>55</v>
       </c>
@@ -2213,8 +2213,8 @@
       </c>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
       <c r="C39" t="s">
         <v>56</v>
       </c>
@@ -2244,8 +2244,8 @@
       </c>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="4"/>
-      <c r="B40" s="4"/>
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
       <c r="C40" t="s">
         <v>57</v>
       </c>
@@ -2275,8 +2275,8 @@
       </c>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
       <c r="C41" t="s">
         <v>58</v>
       </c>
@@ -2306,8 +2306,8 @@
       </c>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4" t="s">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C42" t="s">
@@ -2339,8 +2339,8 @@
       </c>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4"/>
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
       <c r="C43" t="s">
         <v>61</v>
       </c>
@@ -2370,8 +2370,8 @@
       </c>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
       <c r="C44" t="s">
         <v>62</v>
       </c>
@@ -2401,8 +2401,8 @@
       </c>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
       <c r="C45" t="s">
         <v>63</v>
       </c>
@@ -2432,8 +2432,8 @@
       </c>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
       <c r="C46" t="s">
         <v>64</v>
       </c>
@@ -2463,8 +2463,8 @@
       </c>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4" t="s">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
         <v>65</v>
       </c>
       <c r="C47" t="s">
@@ -2496,8 +2496,8 @@
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
       <c r="C48" t="s">
         <v>67</v>
       </c>
@@ -2527,8 +2527,8 @@
       </c>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
       <c r="C49" t="s">
         <v>68</v>
       </c>
@@ -2558,8 +2558,8 @@
       </c>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2589,8 +2589,8 @@
       </c>
     </row>
     <row r="51" spans="1:11">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
       <c r="C51" t="s">
         <v>70</v>
       </c>
@@ -2620,8 +2620,8 @@
       </c>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4" t="s">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C52" t="s">
@@ -2653,8 +2653,8 @@
       </c>
     </row>
     <row r="53" spans="1:11">
-      <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
       <c r="C53" t="s">
         <v>72</v>
       </c>
@@ -2684,8 +2684,8 @@
       </c>
     </row>
     <row r="54" spans="1:11">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
+      <c r="A54" s="5"/>
+      <c r="B54" s="5"/>
       <c r="C54" t="s">
         <v>73</v>
       </c>
@@ -2715,8 +2715,8 @@
       </c>
     </row>
     <row r="55" spans="1:11">
-      <c r="A55" s="4"/>
-      <c r="B55" s="4"/>
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
       <c r="C55" t="s">
         <v>74</v>
       </c>
@@ -2746,8 +2746,8 @@
       </c>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
       <c r="C56" t="s">
         <v>75</v>
       </c>
@@ -2777,8 +2777,8 @@
       </c>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4" t="s">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C57" t="s">
@@ -2810,8 +2810,8 @@
       </c>
     </row>
     <row r="58" spans="1:11">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
       <c r="C58" t="s">
         <v>78</v>
       </c>
@@ -2841,8 +2841,8 @@
       </c>
     </row>
     <row r="59" spans="1:11">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
       <c r="C59" t="s">
         <v>79</v>
       </c>
@@ -2872,8 +2872,8 @@
       </c>
     </row>
     <row r="60" spans="1:11">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
       <c r="C60" t="s">
         <v>80</v>
       </c>
@@ -2903,8 +2903,8 @@
       </c>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
       <c r="C61" t="s">
         <v>81</v>
       </c>
@@ -2934,8 +2934,8 @@
       </c>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="4"/>
-      <c r="B62" s="4" t="s">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5" t="s">
         <v>82</v>
       </c>
       <c r="C62" t="s">
@@ -2967,8 +2967,8 @@
       </c>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="4"/>
-      <c r="B63" s="4"/>
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
       <c r="C63" t="s">
         <v>84</v>
       </c>
@@ -2998,8 +2998,8 @@
       </c>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="4"/>
-      <c r="B64" s="4"/>
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
       <c r="C64" t="s">
         <v>85</v>
       </c>
@@ -3029,8 +3029,8 @@
       </c>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="4"/>
-      <c r="B65" s="4"/>
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
       <c r="C65" t="s">
         <v>86</v>
       </c>
@@ -3060,8 +3060,8 @@
       </c>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="4"/>
-      <c r="B66" s="4"/>
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
       <c r="C66" t="s">
         <v>87</v>
       </c>
@@ -3091,10 +3091,10 @@
       </c>
     </row>
     <row r="67" spans="1:11">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C67" t="s">
@@ -3126,8 +3126,8 @@
       </c>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="4"/>
-      <c r="B68" s="4"/>
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
       <c r="C68" t="s">
         <v>91</v>
       </c>
@@ -3157,8 +3157,8 @@
       </c>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="4"/>
-      <c r="B69" s="4"/>
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
       <c r="C69" t="s">
         <v>92</v>
       </c>
@@ -3188,8 +3188,8 @@
       </c>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="4"/>
-      <c r="B70" s="4"/>
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
       <c r="C70" t="s">
         <v>93</v>
       </c>
@@ -3219,8 +3219,8 @@
       </c>
     </row>
     <row r="71" spans="1:11">
-      <c r="A71" s="4"/>
-      <c r="B71" s="4"/>
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
       <c r="C71" t="s">
         <v>94</v>
       </c>
@@ -3250,8 +3250,8 @@
       </c>
     </row>
     <row r="72" spans="1:11">
-      <c r="A72" s="4"/>
-      <c r="B72" s="4" t="s">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5" t="s">
         <v>95</v>
       </c>
       <c r="C72" t="s">
@@ -3283,8 +3283,8 @@
       </c>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="4"/>
-      <c r="B73" s="4"/>
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
       <c r="C73" t="s">
         <v>97</v>
       </c>
@@ -3314,8 +3314,8 @@
       </c>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="4"/>
-      <c r="B74" s="4"/>
+      <c r="A74" s="5"/>
+      <c r="B74" s="5"/>
       <c r="C74" t="s">
         <v>98</v>
       </c>
@@ -3345,8 +3345,8 @@
       </c>
     </row>
     <row r="75" spans="1:11">
-      <c r="A75" s="4"/>
-      <c r="B75" s="4"/>
+      <c r="A75" s="5"/>
+      <c r="B75" s="5"/>
       <c r="C75" t="s">
         <v>99</v>
       </c>
@@ -3376,8 +3376,8 @@
       </c>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="4"/>
-      <c r="B76" s="4"/>
+      <c r="A76" s="5"/>
+      <c r="B76" s="5"/>
       <c r="C76" t="s">
         <v>100</v>
       </c>
@@ -3407,8 +3407,8 @@
       </c>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="4"/>
-      <c r="B77" s="4" t="s">
+      <c r="A77" s="5"/>
+      <c r="B77" s="5" t="s">
         <v>101</v>
       </c>
       <c r="C77" t="s">
@@ -3440,8 +3440,8 @@
       </c>
     </row>
     <row r="78" spans="1:11">
-      <c r="A78" s="4"/>
-      <c r="B78" s="4"/>
+      <c r="A78" s="5"/>
+      <c r="B78" s="5"/>
       <c r="C78" t="s">
         <v>103</v>
       </c>
@@ -3471,8 +3471,8 @@
       </c>
     </row>
     <row r="79" spans="1:11">
-      <c r="A79" s="4"/>
-      <c r="B79" s="4"/>
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
       <c r="C79" t="s">
         <v>104</v>
       </c>
@@ -3502,8 +3502,8 @@
       </c>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="4"/>
-      <c r="B80" s="4"/>
+      <c r="A80" s="5"/>
+      <c r="B80" s="5"/>
       <c r="C80" t="s">
         <v>105</v>
       </c>
@@ -3533,8 +3533,8 @@
       </c>
     </row>
     <row r="81" spans="1:11">
-      <c r="A81" s="4"/>
-      <c r="B81" s="4"/>
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
       <c r="C81" t="s">
         <v>106</v>
       </c>
@@ -3564,8 +3564,8 @@
       </c>
     </row>
     <row r="82" spans="1:11">
-      <c r="A82" s="4"/>
-      <c r="B82" s="4" t="s">
+      <c r="A82" s="5"/>
+      <c r="B82" s="5" t="s">
         <v>107</v>
       </c>
       <c r="C82" t="s">
@@ -3597,8 +3597,8 @@
       </c>
     </row>
     <row r="83" spans="1:11">
-      <c r="A83" s="4"/>
-      <c r="B83" s="4"/>
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
       <c r="C83" t="s">
         <v>109</v>
       </c>
@@ -3628,8 +3628,8 @@
       </c>
     </row>
     <row r="84" spans="1:11">
-      <c r="A84" s="4"/>
-      <c r="B84" s="4"/>
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
       <c r="C84" t="s">
         <v>110</v>
       </c>
@@ -3659,8 +3659,8 @@
       </c>
     </row>
     <row r="85" spans="1:11">
-      <c r="A85" s="4"/>
-      <c r="B85" s="4"/>
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
       <c r="C85" t="s">
         <v>111</v>
       </c>
@@ -3690,8 +3690,8 @@
       </c>
     </row>
     <row r="86" spans="1:11">
-      <c r="A86" s="4"/>
-      <c r="B86" s="4"/>
+      <c r="A86" s="5"/>
+      <c r="B86" s="5"/>
       <c r="C86" t="s">
         <v>112</v>
       </c>
@@ -3721,10 +3721,10 @@
       </c>
     </row>
     <row r="87" spans="1:11">
-      <c r="A87" s="4" t="s">
+      <c r="A87" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="B87" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C87" t="s">
@@ -3756,8 +3756,8 @@
       </c>
     </row>
     <row r="88" spans="1:11">
-      <c r="A88" s="4"/>
-      <c r="B88" s="4"/>
+      <c r="A88" s="5"/>
+      <c r="B88" s="5"/>
       <c r="C88" t="s">
         <v>116</v>
       </c>
@@ -3787,8 +3787,8 @@
       </c>
     </row>
     <row r="89" spans="1:11">
-      <c r="A89" s="4"/>
-      <c r="B89" s="4"/>
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
       <c r="C89" t="s">
         <v>117</v>
       </c>
@@ -3818,8 +3818,8 @@
       </c>
     </row>
     <row r="90" spans="1:11">
-      <c r="A90" s="4"/>
-      <c r="B90" s="4"/>
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
       <c r="C90" t="s">
         <v>118</v>
       </c>
@@ -3849,8 +3849,8 @@
       </c>
     </row>
     <row r="91" spans="1:11">
-      <c r="A91" s="4"/>
-      <c r="B91" s="4"/>
+      <c r="A91" s="5"/>
+      <c r="B91" s="5"/>
       <c r="C91" t="s">
         <v>119</v>
       </c>
@@ -3880,8 +3880,8 @@
       </c>
     </row>
     <row r="92" spans="1:11">
-      <c r="A92" s="4"/>
-      <c r="B92" s="4" t="s">
+      <c r="A92" s="5"/>
+      <c r="B92" s="5" t="s">
         <v>120</v>
       </c>
       <c r="C92" t="s">
@@ -3913,8 +3913,8 @@
       </c>
     </row>
     <row r="93" spans="1:11">
-      <c r="A93" s="4"/>
-      <c r="B93" s="4"/>
+      <c r="A93" s="5"/>
+      <c r="B93" s="5"/>
       <c r="C93" t="s">
         <v>122</v>
       </c>
@@ -3944,8 +3944,8 @@
       </c>
     </row>
     <row r="94" spans="1:11">
-      <c r="A94" s="4"/>
-      <c r="B94" s="4"/>
+      <c r="A94" s="5"/>
+      <c r="B94" s="5"/>
       <c r="C94" t="s">
         <v>123</v>
       </c>
@@ -3975,8 +3975,8 @@
       </c>
     </row>
     <row r="95" spans="1:11">
-      <c r="A95" s="4"/>
-      <c r="B95" s="4"/>
+      <c r="A95" s="5"/>
+      <c r="B95" s="5"/>
       <c r="C95" t="s">
         <v>124</v>
       </c>
@@ -4006,8 +4006,8 @@
       </c>
     </row>
     <row r="96" spans="1:11">
-      <c r="A96" s="4"/>
-      <c r="B96" s="4"/>
+      <c r="A96" s="5"/>
+      <c r="B96" s="5"/>
       <c r="C96" t="s">
         <v>125</v>
       </c>
@@ -4037,8 +4037,8 @@
       </c>
     </row>
     <row r="97" spans="1:11">
-      <c r="A97" s="4"/>
-      <c r="B97" s="4" t="s">
+      <c r="A97" s="5"/>
+      <c r="B97" s="5" t="s">
         <v>126</v>
       </c>
       <c r="C97" t="s">
@@ -4070,8 +4070,8 @@
       </c>
     </row>
     <row r="98" spans="1:11">
-      <c r="A98" s="4"/>
-      <c r="B98" s="4"/>
+      <c r="A98" s="5"/>
+      <c r="B98" s="5"/>
       <c r="C98" t="s">
         <v>128</v>
       </c>
@@ -4101,8 +4101,8 @@
       </c>
     </row>
     <row r="99" spans="1:11">
-      <c r="A99" s="4"/>
-      <c r="B99" s="4"/>
+      <c r="A99" s="5"/>
+      <c r="B99" s="5"/>
       <c r="C99" t="s">
         <v>129</v>
       </c>
@@ -4132,8 +4132,8 @@
       </c>
     </row>
     <row r="100" spans="1:11">
-      <c r="A100" s="4"/>
-      <c r="B100" s="4"/>
+      <c r="A100" s="5"/>
+      <c r="B100" s="5"/>
       <c r="C100" t="s">
         <v>130</v>
       </c>
@@ -4163,8 +4163,8 @@
       </c>
     </row>
     <row r="101" spans="1:11">
-      <c r="A101" s="4"/>
-      <c r="B101" s="4"/>
+      <c r="A101" s="5"/>
+      <c r="B101" s="5"/>
       <c r="C101" t="s">
         <v>131</v>
       </c>
@@ -4194,10 +4194,10 @@
       </c>
     </row>
     <row r="102" spans="1:11">
-      <c r="A102" s="4" t="s">
+      <c r="A102" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="5" t="s">
         <v>133</v>
       </c>
       <c r="C102" s="2" t="s">
@@ -4229,8 +4229,8 @@
       </c>
     </row>
     <row r="103" spans="1:11">
-      <c r="A103" s="4"/>
-      <c r="B103" s="4"/>
+      <c r="A103" s="5"/>
+      <c r="B103" s="5"/>
       <c r="C103" s="2" t="s">
         <v>135</v>
       </c>
@@ -4260,8 +4260,8 @@
       </c>
     </row>
     <row r="104" spans="1:11">
-      <c r="A104" s="4"/>
-      <c r="B104" s="4"/>
+      <c r="A104" s="5"/>
+      <c r="B104" s="5"/>
       <c r="C104" s="2" t="s">
         <v>136</v>
       </c>
@@ -4291,8 +4291,8 @@
       </c>
     </row>
     <row r="105" spans="1:11">
-      <c r="A105" s="4"/>
-      <c r="B105" s="4"/>
+      <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
       <c r="C105" s="2" t="s">
         <v>137</v>
       </c>
@@ -4322,8 +4322,8 @@
       </c>
     </row>
     <row r="106" spans="1:11">
-      <c r="A106" s="4"/>
-      <c r="B106" s="4"/>
+      <c r="A106" s="5"/>
+      <c r="B106" s="5"/>
       <c r="C106" s="2" t="s">
         <v>138</v>
       </c>
@@ -4353,8 +4353,8 @@
       </c>
     </row>
     <row r="107" spans="1:11">
-      <c r="A107" s="4"/>
-      <c r="B107" s="4"/>
+      <c r="A107" s="5"/>
+      <c r="B107" s="5"/>
       <c r="C107" s="2" t="s">
         <v>139</v>
       </c>
@@ -4384,8 +4384,8 @@
       </c>
     </row>
     <row r="108" spans="1:11">
-      <c r="A108" s="4"/>
-      <c r="B108" s="4" t="s">
+      <c r="A108" s="5"/>
+      <c r="B108" s="5" t="s">
         <v>140</v>
       </c>
       <c r="C108" s="2" t="s">
@@ -4417,8 +4417,8 @@
       </c>
     </row>
     <row r="109" spans="1:11">
-      <c r="A109" s="4"/>
-      <c r="B109" s="4"/>
+      <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
       <c r="C109" s="2" t="s">
         <v>142</v>
       </c>
@@ -4448,8 +4448,8 @@
       </c>
     </row>
     <row r="110" spans="1:11">
-      <c r="A110" s="4"/>
-      <c r="B110" s="4"/>
+      <c r="A110" s="5"/>
+      <c r="B110" s="5"/>
       <c r="C110" s="2" t="s">
         <v>143</v>
       </c>
@@ -4479,8 +4479,8 @@
       </c>
     </row>
     <row r="111" spans="1:11">
-      <c r="A111" s="4"/>
-      <c r="B111" s="4" t="s">
+      <c r="A111" s="5"/>
+      <c r="B111" s="5" t="s">
         <v>144</v>
       </c>
       <c r="C111" s="2" t="s">
@@ -4512,8 +4512,8 @@
       </c>
     </row>
     <row r="112" spans="1:11">
-      <c r="A112" s="4"/>
-      <c r="B112" s="4"/>
+      <c r="A112" s="5"/>
+      <c r="B112" s="5"/>
       <c r="C112" s="2" t="s">
         <v>146</v>
       </c>
@@ -4543,8 +4543,8 @@
       </c>
     </row>
     <row r="113" spans="1:11">
-      <c r="A113" s="4"/>
-      <c r="B113" s="4"/>
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
       <c r="C113" s="2" t="s">
         <v>147</v>
       </c>
@@ -4574,8 +4574,8 @@
       </c>
     </row>
     <row r="114" spans="1:11">
-      <c r="A114" s="4"/>
-      <c r="B114" s="4"/>
+      <c r="A114" s="5"/>
+      <c r="B114" s="5"/>
       <c r="C114" s="2" t="s">
         <v>148</v>
       </c>
@@ -4605,8 +4605,8 @@
       </c>
     </row>
     <row r="115" spans="1:11">
-      <c r="A115" s="4"/>
-      <c r="B115" s="4"/>
+      <c r="A115" s="5"/>
+      <c r="B115" s="5"/>
       <c r="C115" s="2" t="s">
         <v>149</v>
       </c>
@@ -4636,8 +4636,8 @@
       </c>
     </row>
     <row r="116" spans="1:11">
-      <c r="A116" s="4"/>
-      <c r="B116" s="4" t="s">
+      <c r="A116" s="5"/>
+      <c r="B116" s="5" t="s">
         <v>150</v>
       </c>
       <c r="C116" s="2" t="s">
@@ -4669,8 +4669,8 @@
       </c>
     </row>
     <row r="117" spans="1:11">
-      <c r="A117" s="4"/>
-      <c r="B117" s="4"/>
+      <c r="A117" s="5"/>
+      <c r="B117" s="5"/>
       <c r="C117" s="2" t="s">
         <v>152</v>
       </c>
@@ -4700,8 +4700,8 @@
       </c>
     </row>
     <row r="118" spans="1:11">
-      <c r="A118" s="4"/>
-      <c r="B118" s="4"/>
+      <c r="A118" s="5"/>
+      <c r="B118" s="5"/>
       <c r="C118" s="2" t="s">
         <v>153</v>
       </c>
@@ -4731,8 +4731,8 @@
       </c>
     </row>
     <row r="119" spans="1:11">
-      <c r="A119" s="4"/>
-      <c r="B119" s="4"/>
+      <c r="A119" s="5"/>
+      <c r="B119" s="5"/>
       <c r="C119" s="2" t="s">
         <v>154</v>
       </c>
@@ -4762,8 +4762,8 @@
       </c>
     </row>
     <row r="120" spans="1:11">
-      <c r="A120" s="4"/>
-      <c r="B120" s="4"/>
+      <c r="A120" s="5"/>
+      <c r="B120" s="5"/>
       <c r="C120" s="2" t="s">
         <v>155</v>
       </c>
@@ -4793,8 +4793,8 @@
       </c>
     </row>
     <row r="121" spans="1:11">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
+      <c r="A121" s="5"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="2" t="s">
         <v>156</v>
       </c>
@@ -4824,8 +4824,8 @@
       </c>
     </row>
     <row r="122" spans="1:11">
-      <c r="A122" s="4"/>
-      <c r="B122" s="4"/>
+      <c r="A122" s="5"/>
+      <c r="B122" s="5"/>
       <c r="C122" s="2" t="s">
         <v>157</v>
       </c>
@@ -4855,8 +4855,8 @@
       </c>
     </row>
     <row r="123" spans="1:11">
-      <c r="A123" s="4"/>
-      <c r="B123" s="4" t="s">
+      <c r="A123" s="5"/>
+      <c r="B123" s="5" t="s">
         <v>158</v>
       </c>
       <c r="C123" s="2" t="s">
@@ -4888,8 +4888,8 @@
       </c>
     </row>
     <row r="124" spans="1:11">
-      <c r="A124" s="4"/>
-      <c r="B124" s="4"/>
+      <c r="A124" s="5"/>
+      <c r="B124" s="5"/>
       <c r="C124" s="2" t="s">
         <v>160</v>
       </c>
@@ -4919,8 +4919,8 @@
       </c>
     </row>
     <row r="125" spans="1:11">
-      <c r="A125" s="4"/>
-      <c r="B125" s="4"/>
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
       <c r="C125" s="2" t="s">
         <v>161</v>
       </c>
@@ -4950,8 +4950,8 @@
       </c>
     </row>
     <row r="126" spans="1:11">
-      <c r="A126" s="4"/>
-      <c r="B126" s="4"/>
+      <c r="A126" s="5"/>
+      <c r="B126" s="5"/>
       <c r="C126" s="2" t="s">
         <v>162</v>
       </c>
@@ -4981,8 +4981,8 @@
       </c>
     </row>
     <row r="127" spans="1:11">
-      <c r="A127" s="4"/>
-      <c r="B127" s="4"/>
+      <c r="A127" s="5"/>
+      <c r="B127" s="5"/>
       <c r="C127" s="2" t="s">
         <v>163</v>
       </c>
@@ -5012,132 +5012,516 @@
       </c>
     </row>
     <row r="128" spans="1:11">
-      <c r="A128" s="4" t="s">
+      <c r="A128" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B128" s="5" t="s">
         <v>165</v>
       </c>
       <c r="C128" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="129" spans="1:3">
-      <c r="A129" s="4"/>
-      <c r="B129" s="4"/>
+      <c r="D128">
+        <v>1</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>0</v>
+      </c>
+      <c r="G128">
+        <v>0</v>
+      </c>
+      <c r="H128">
+        <v>0</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11">
+      <c r="A129" s="5"/>
+      <c r="B129" s="5"/>
       <c r="C129" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="130" spans="1:3">
-      <c r="A130" s="4"/>
-      <c r="B130" s="4"/>
+      <c r="D129">
+        <v>1</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>0</v>
+      </c>
+      <c r="G129">
+        <v>0</v>
+      </c>
+      <c r="H129">
+        <v>0</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11">
+      <c r="A130" s="5"/>
+      <c r="B130" s="5"/>
       <c r="C130" s="3" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="131" spans="1:3">
-      <c r="A131" s="4" t="s">
+      <c r="D130">
+        <v>1</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>0</v>
+      </c>
+      <c r="G130">
+        <v>0</v>
+      </c>
+      <c r="H130">
+        <v>0</v>
+      </c>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11">
+      <c r="A131" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="4" t="s">
+      <c r="B131" s="5" t="s">
         <v>169</v>
       </c>
       <c r="C131" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+      <c r="F131">
+        <v>0</v>
+      </c>
+      <c r="G131">
+        <v>0</v>
+      </c>
+      <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11">
+      <c r="A132" s="5"/>
+      <c r="B132" s="5"/>
       <c r="C132" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+      <c r="F132">
+        <v>0</v>
+      </c>
+      <c r="G132">
+        <v>0</v>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11">
+      <c r="A133" s="5"/>
+      <c r="B133" s="5"/>
       <c r="C133" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
+      <c r="D133">
+        <v>1</v>
+      </c>
+      <c r="E133">
+        <v>0</v>
+      </c>
+      <c r="F133">
+        <v>0</v>
+      </c>
+      <c r="G133">
+        <v>0</v>
+      </c>
+      <c r="H133">
+        <v>0</v>
+      </c>
+      <c r="I133">
+        <v>0</v>
+      </c>
+      <c r="J133">
+        <v>0</v>
+      </c>
+      <c r="K133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11">
+      <c r="A134" s="5"/>
+      <c r="B134" s="5"/>
       <c r="C134" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134">
+        <v>0</v>
+      </c>
+      <c r="F134">
+        <v>0</v>
+      </c>
+      <c r="G134">
+        <v>0</v>
+      </c>
+      <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+      <c r="J134">
+        <v>0</v>
+      </c>
+      <c r="K134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11">
+      <c r="A135" s="5"/>
+      <c r="B135" s="5"/>
       <c r="C135" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="136" spans="1:3">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135">
+        <v>0</v>
+      </c>
+      <c r="F135">
+        <v>0</v>
+      </c>
+      <c r="G135">
+        <v>0</v>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11">
+      <c r="A136" s="5"/>
+      <c r="B136" s="5"/>
       <c r="C136" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="137" spans="1:3">
-      <c r="A137" s="4" t="s">
+      <c r="D136">
+        <v>1</v>
+      </c>
+      <c r="E136">
+        <v>0</v>
+      </c>
+      <c r="F136">
+        <v>0</v>
+      </c>
+      <c r="G136">
+        <v>0</v>
+      </c>
+      <c r="H136">
+        <v>0</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+      <c r="J136">
+        <v>0</v>
+      </c>
+      <c r="K136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11">
+      <c r="A137" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B137" s="4" t="s">
+      <c r="B137" s="5" t="s">
         <v>177</v>
       </c>
       <c r="C137" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="138" spans="1:3">
-      <c r="A138" s="4"/>
-      <c r="B138" s="4"/>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>1</v>
+      </c>
+      <c r="F137">
+        <v>1</v>
+      </c>
+      <c r="G137">
+        <v>1</v>
+      </c>
+      <c r="H137">
+        <v>1</v>
+      </c>
+      <c r="I137">
+        <v>1</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11">
+      <c r="A138" s="5"/>
+      <c r="B138" s="5"/>
       <c r="C138" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="139" spans="1:3">
-      <c r="A139" s="4"/>
-      <c r="B139" s="4"/>
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11">
+      <c r="A139" s="5"/>
+      <c r="B139" s="5"/>
       <c r="C139" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="140" spans="1:3">
-      <c r="A140" s="4"/>
-      <c r="B140" s="4"/>
+      <c r="D139">
+        <v>1</v>
+      </c>
+      <c r="E139">
+        <v>1</v>
+      </c>
+      <c r="F139">
+        <v>1</v>
+      </c>
+      <c r="G139">
+        <v>1</v>
+      </c>
+      <c r="H139">
+        <v>1</v>
+      </c>
+      <c r="I139">
+        <v>1</v>
+      </c>
+      <c r="J139">
+        <v>0</v>
+      </c>
+      <c r="K139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11">
+      <c r="A140" s="5"/>
+      <c r="B140" s="5"/>
       <c r="C140" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="141" spans="1:3">
-      <c r="A141" s="4"/>
-      <c r="B141" s="4"/>
+      <c r="D140">
+        <v>1</v>
+      </c>
+      <c r="E140">
+        <v>1</v>
+      </c>
+      <c r="F140">
+        <v>1</v>
+      </c>
+      <c r="G140">
+        <v>1</v>
+      </c>
+      <c r="H140">
+        <v>1</v>
+      </c>
+      <c r="I140">
+        <v>1</v>
+      </c>
+      <c r="J140">
+        <v>0</v>
+      </c>
+      <c r="K140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11">
+      <c r="A141" s="5"/>
+      <c r="B141" s="5"/>
       <c r="C141" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="142" spans="1:3">
-      <c r="A142" s="4"/>
-      <c r="B142" s="4" t="s">
+      <c r="D141">
+        <v>1</v>
+      </c>
+      <c r="E141">
+        <v>1</v>
+      </c>
+      <c r="F141">
+        <v>1</v>
+      </c>
+      <c r="G141">
+        <v>1</v>
+      </c>
+      <c r="H141">
+        <v>1</v>
+      </c>
+      <c r="I141">
+        <v>1</v>
+      </c>
+      <c r="J141">
+        <v>0</v>
+      </c>
+      <c r="K141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11">
+      <c r="A142" s="5"/>
+      <c r="B142" s="5" t="s">
         <v>183</v>
       </c>
       <c r="C142" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" s="4"/>
-      <c r="B143" s="4"/>
+      <c r="D142">
+        <v>1</v>
+      </c>
+      <c r="E142">
+        <v>1</v>
+      </c>
+      <c r="F142">
+        <v>1</v>
+      </c>
+      <c r="G142">
+        <v>1</v>
+      </c>
+      <c r="H142">
+        <v>1</v>
+      </c>
+      <c r="I142">
+        <v>1</v>
+      </c>
+      <c r="J142">
+        <v>0</v>
+      </c>
+      <c r="K142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11">
+      <c r="A143" s="5"/>
+      <c r="B143" s="5"/>
       <c r="C143" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="144" spans="1:3">
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143">
+        <v>1</v>
+      </c>
+      <c r="G143">
+        <v>1</v>
+      </c>
+      <c r="H143">
+        <v>1</v>
+      </c>
+      <c r="I143">
+        <v>1</v>
+      </c>
+      <c r="J143">
+        <v>0</v>
+      </c>
+      <c r="K143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11">
       <c r="A144" s="1" t="s">
         <v>164</v>
       </c>
@@ -5147,15 +5531,63 @@
       <c r="C144" t="s">
         <v>186</v>
       </c>
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
+        <v>1</v>
+      </c>
+      <c r="H144">
+        <v>1</v>
+      </c>
+      <c r="I144">
+        <v>1</v>
+      </c>
+      <c r="J144">
+        <v>1</v>
+      </c>
+      <c r="K144">
+        <v>1</v>
+      </c>
     </row>
     <row r="145" spans="3:3">
-      <c r="C145" s="5"/>
+      <c r="C145" s="4"/>
     </row>
     <row r="146" spans="3:3">
-      <c r="C146" s="5"/>
+      <c r="C146" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="A87:A101"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B87:B91"/>
+    <mergeCell ref="B92:B96"/>
+    <mergeCell ref="B97:B101"/>
     <mergeCell ref="A102:A127"/>
     <mergeCell ref="A128:A130"/>
     <mergeCell ref="A131:A136"/>
@@ -5169,30 +5601,6 @@
     <mergeCell ref="B131:B136"/>
     <mergeCell ref="B137:B141"/>
     <mergeCell ref="B142:B143"/>
-    <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A101"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B87:B91"/>
-    <mergeCell ref="B92:B96"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5200,6 +5608,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5208,15 +5625,6 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5409,20 +5817,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Added settings perms to excel file in helpers
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE6D5C1-5850-4799-8E3E-6CD3A8E2F55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C568B3-4200-4E26-89A8-7C948583B1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="194">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -636,13 +636,31 @@
   </si>
   <si>
     <t>permission:delete</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>settings</t>
+  </si>
+  <si>
+    <t>settings:create</t>
+  </si>
+  <si>
+    <t>settings:view</t>
+  </si>
+  <si>
+    <t>settings:update</t>
+  </si>
+  <si>
+    <t>settings:delete</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -671,13 +689,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF6AAB73"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-      <charset val="238"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -705,16 +716,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -998,8 +1006,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K146"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:K148"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -1014,7 +1022,7 @@
     <col min="11" max="11" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" t="s">
@@ -1045,11 +1053,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
@@ -1080,9 +1088,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -1111,9 +1119,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
       <c r="C4" t="s">
         <v>13</v>
       </c>
@@ -1142,9 +1150,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
       <c r="C5" t="s">
         <v>14</v>
       </c>
@@ -1173,9 +1181,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
       <c r="C6" t="s">
         <v>15</v>
       </c>
@@ -1204,9 +1212,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
@@ -1237,9 +1245,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
       <c r="C8" t="s">
         <v>18</v>
       </c>
@@ -1268,9 +1276,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -1299,9 +1307,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
       <c r="C10" t="s">
         <v>20</v>
       </c>
@@ -1330,9 +1338,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
       <c r="C11" t="s">
         <v>21</v>
       </c>
@@ -1361,9 +1369,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C12" t="s">
@@ -1394,9 +1402,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
       <c r="C13" t="s">
         <v>24</v>
       </c>
@@ -1425,9 +1433,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
       <c r="C14" t="s">
         <v>25</v>
       </c>
@@ -1456,9 +1464,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
       <c r="C15" t="s">
         <v>26</v>
       </c>
@@ -1487,9 +1495,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
       <c r="C16" t="s">
         <v>27</v>
       </c>
@@ -1518,9 +1526,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5" t="s">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C17" t="s">
@@ -1551,9 +1559,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
       <c r="C18" t="s">
         <v>30</v>
       </c>
@@ -1582,9 +1590,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
       <c r="C19" t="s">
         <v>31</v>
       </c>
@@ -1613,9 +1621,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
       <c r="C20" t="s">
         <v>32</v>
       </c>
@@ -1644,9 +1652,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
       <c r="C21" t="s">
         <v>33</v>
       </c>
@@ -1675,9 +1683,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5" t="s">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C22" t="s">
@@ -1708,9 +1716,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
       <c r="C23" t="s">
         <v>36</v>
       </c>
@@ -1739,9 +1747,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
       <c r="C24" t="s">
         <v>37</v>
       </c>
@@ -1770,9 +1778,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
       <c r="C25" t="s">
         <v>38</v>
       </c>
@@ -1801,9 +1809,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
       <c r="C26" t="s">
         <v>39</v>
       </c>
@@ -1832,11 +1840,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1867,9 +1875,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
       <c r="C28" t="s">
         <v>43</v>
       </c>
@@ -1898,9 +1906,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
       <c r="C29" t="s">
         <v>44</v>
       </c>
@@ -1929,9 +1937,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
       <c r="C30" t="s">
         <v>45</v>
       </c>
@@ -1960,9 +1968,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
       <c r="C31" t="s">
         <v>46</v>
       </c>
@@ -1991,9 +1999,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4" t="s">
         <v>47</v>
       </c>
       <c r="C32" t="s">
@@ -2024,9 +2032,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
       <c r="C33" t="s">
         <v>49</v>
       </c>
@@ -2055,9 +2063,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
       <c r="C34" t="s">
         <v>50</v>
       </c>
@@ -2086,9 +2094,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
       <c r="C35" t="s">
         <v>51</v>
       </c>
@@ -2117,9 +2125,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
       <c r="C36" t="s">
         <v>52</v>
       </c>
@@ -2148,9 +2156,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C37" t="s">
@@ -2181,9 +2189,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
       <c r="C38" t="s">
         <v>55</v>
       </c>
@@ -2212,9 +2220,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
       <c r="C39" t="s">
         <v>56</v>
       </c>
@@ -2243,9 +2251,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
       <c r="C40" t="s">
         <v>57</v>
       </c>
@@ -2274,9 +2282,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
       <c r="C41" t="s">
         <v>58</v>
       </c>
@@ -2305,9 +2313,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="4"/>
+      <c r="B42" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C42" t="s">
@@ -2338,9 +2346,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
       <c r="C43" t="s">
         <v>61</v>
       </c>
@@ -2369,9 +2377,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
       <c r="C44" t="s">
         <v>62</v>
       </c>
@@ -2400,9 +2408,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
       <c r="C45" t="s">
         <v>63</v>
       </c>
@@ -2431,9 +2439,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
       <c r="C46" t="s">
         <v>64</v>
       </c>
@@ -2462,9 +2470,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5" t="s">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="4"/>
+      <c r="B47" s="4" t="s">
         <v>65</v>
       </c>
       <c r="C47" t="s">
@@ -2495,9 +2503,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
       <c r="C48" t="s">
         <v>67</v>
       </c>
@@ -2526,9 +2534,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" s="4"/>
+      <c r="B49" s="4"/>
       <c r="C49" t="s">
         <v>68</v>
       </c>
@@ -2557,9 +2565,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2588,9 +2596,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
       <c r="C51" t="s">
         <v>70</v>
       </c>
@@ -2619,9 +2627,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5" t="s">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="4"/>
+      <c r="B52" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C52" t="s">
@@ -2652,9 +2660,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:11">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" s="4"/>
+      <c r="B53" s="4"/>
       <c r="C53" t="s">
         <v>72</v>
       </c>
@@ -2683,9 +2691,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:11">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
       <c r="C54" t="s">
         <v>73</v>
       </c>
@@ -2714,9 +2722,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
       <c r="C55" t="s">
         <v>74</v>
       </c>
@@ -2745,9 +2753,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="4"/>
+      <c r="B56" s="4"/>
       <c r="C56" t="s">
         <v>75</v>
       </c>
@@ -2776,9 +2784,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5" t="s">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" s="4"/>
+      <c r="B57" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C57" t="s">
@@ -2809,9 +2817,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:11">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
       <c r="C58" t="s">
         <v>78</v>
       </c>
@@ -2840,9 +2848,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:11">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
       <c r="C59" t="s">
         <v>79</v>
       </c>
@@ -2871,9 +2879,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
       <c r="C60" t="s">
         <v>80</v>
       </c>
@@ -2902,9 +2910,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
       <c r="C61" t="s">
         <v>81</v>
       </c>
@@ -2933,9 +2941,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5" t="s">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" s="4"/>
+      <c r="B62" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C62" t="s">
@@ -2966,9 +2974,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:11">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
       <c r="C63" t="s">
         <v>84</v>
       </c>
@@ -2997,9 +3005,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
       <c r="C64" t="s">
         <v>85</v>
       </c>
@@ -3028,9 +3036,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:11">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
       <c r="C65" t="s">
         <v>86</v>
       </c>
@@ -3059,9 +3067,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:11">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
       <c r="C66" t="s">
         <v>87</v>
       </c>
@@ -3090,11 +3098,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:11">
-      <c r="A67" s="5" t="s">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="4" t="s">
         <v>89</v>
       </c>
       <c r="C67" t="s">
@@ -3125,9 +3133,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:11">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
       <c r="C68" t="s">
         <v>91</v>
       </c>
@@ -3156,9 +3164,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:11">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
       <c r="C69" t="s">
         <v>92</v>
       </c>
@@ -3187,9 +3195,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:11">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" s="4"/>
+      <c r="B70" s="4"/>
       <c r="C70" t="s">
         <v>93</v>
       </c>
@@ -3218,9 +3226,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:11">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
       <c r="C71" t="s">
         <v>94</v>
       </c>
@@ -3249,9 +3257,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:11">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5" t="s">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" s="4"/>
+      <c r="B72" s="4" t="s">
         <v>95</v>
       </c>
       <c r="C72" t="s">
@@ -3282,9 +3290,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:11">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" s="4"/>
+      <c r="B73" s="4"/>
       <c r="C73" t="s">
         <v>97</v>
       </c>
@@ -3313,9 +3321,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" s="4"/>
+      <c r="B74" s="4"/>
       <c r="C74" t="s">
         <v>98</v>
       </c>
@@ -3344,9 +3352,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:11">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" s="4"/>
+      <c r="B75" s="4"/>
       <c r="C75" t="s">
         <v>99</v>
       </c>
@@ -3375,9 +3383,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:11">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
       <c r="C76" t="s">
         <v>100</v>
       </c>
@@ -3406,9 +3414,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:11">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5" t="s">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77" s="4"/>
+      <c r="B77" s="4" t="s">
         <v>101</v>
       </c>
       <c r="C77" t="s">
@@ -3439,9 +3447,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:11">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+      <c r="B78" s="4"/>
       <c r="C78" t="s">
         <v>103</v>
       </c>
@@ -3470,9 +3478,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79" s="4"/>
+      <c r="B79" s="4"/>
       <c r="C79" t="s">
         <v>104</v>
       </c>
@@ -3501,9 +3509,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:11">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80" s="4"/>
+      <c r="B80" s="4"/>
       <c r="C80" t="s">
         <v>105</v>
       </c>
@@ -3532,9 +3540,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:11">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81" s="4"/>
+      <c r="B81" s="4"/>
       <c r="C81" t="s">
         <v>106</v>
       </c>
@@ -3563,9 +3571,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:11">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5" t="s">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82" s="4"/>
+      <c r="B82" s="4" t="s">
         <v>107</v>
       </c>
       <c r="C82" t="s">
@@ -3596,9 +3604,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:11">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83" s="4"/>
+      <c r="B83" s="4"/>
       <c r="C83" t="s">
         <v>109</v>
       </c>
@@ -3627,9 +3635,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:11">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84" s="4"/>
+      <c r="B84" s="4"/>
       <c r="C84" t="s">
         <v>110</v>
       </c>
@@ -3658,9 +3666,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:11">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85" s="4"/>
+      <c r="B85" s="4"/>
       <c r="C85" t="s">
         <v>111</v>
       </c>
@@ -3689,9 +3697,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:11">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86" s="4"/>
+      <c r="B86" s="4"/>
       <c r="C86" t="s">
         <v>112</v>
       </c>
@@ -3720,11 +3728,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:11">
-      <c r="A87" s="5" t="s">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C87" t="s">
@@ -3755,9 +3763,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:11">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88" s="4"/>
+      <c r="B88" s="4"/>
       <c r="C88" t="s">
         <v>116</v>
       </c>
@@ -3786,9 +3794,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:11">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89" s="4"/>
+      <c r="B89" s="4"/>
       <c r="C89" t="s">
         <v>117</v>
       </c>
@@ -3817,9 +3825,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:11">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90" s="4"/>
+      <c r="B90" s="4"/>
       <c r="C90" t="s">
         <v>118</v>
       </c>
@@ -3848,9 +3856,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:11">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91" s="4"/>
+      <c r="B91" s="4"/>
       <c r="C91" t="s">
         <v>119</v>
       </c>
@@ -3879,9 +3887,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:11">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5" t="s">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92" s="4"/>
+      <c r="B92" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C92" t="s">
@@ -3912,9 +3920,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:11">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93" s="4"/>
+      <c r="B93" s="4"/>
       <c r="C93" t="s">
         <v>122</v>
       </c>
@@ -3943,9 +3951,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:11">
-      <c r="A94" s="5"/>
-      <c r="B94" s="5"/>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94" s="4"/>
+      <c r="B94" s="4"/>
       <c r="C94" t="s">
         <v>123</v>
       </c>
@@ -3974,9 +3982,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:11">
-      <c r="A95" s="5"/>
-      <c r="B95" s="5"/>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95" s="4"/>
+      <c r="B95" s="4"/>
       <c r="C95" t="s">
         <v>124</v>
       </c>
@@ -4005,9 +4013,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:11">
-      <c r="A96" s="5"/>
-      <c r="B96" s="5"/>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A96" s="4"/>
+      <c r="B96" s="4"/>
       <c r="C96" t="s">
         <v>125</v>
       </c>
@@ -4036,9 +4044,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
-      <c r="A97" s="5"/>
-      <c r="B97" s="5" t="s">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97" s="4"/>
+      <c r="B97" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C97" t="s">
@@ -4069,9 +4077,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
-      <c r="A98" s="5"/>
-      <c r="B98" s="5"/>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98" s="4"/>
+      <c r="B98" s="4"/>
       <c r="C98" t="s">
         <v>128</v>
       </c>
@@ -4100,9 +4108,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:11">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99" s="4"/>
+      <c r="B99" s="4"/>
       <c r="C99" t="s">
         <v>129</v>
       </c>
@@ -4131,9 +4139,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:11">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100" s="4"/>
+      <c r="B100" s="4"/>
       <c r="C100" t="s">
         <v>130</v>
       </c>
@@ -4162,9 +4170,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:11">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A101" s="4"/>
+      <c r="B101" s="4"/>
       <c r="C101" t="s">
         <v>131</v>
       </c>
@@ -4193,11 +4201,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:11">
-      <c r="A102" s="5" t="s">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B102" s="4" t="s">
         <v>133</v>
       </c>
       <c r="C102" s="2" t="s">
@@ -4228,9 +4236,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:11">
-      <c r="A103" s="5"/>
-      <c r="B103" s="5"/>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" s="4"/>
+      <c r="B103" s="4"/>
       <c r="C103" s="2" t="s">
         <v>135</v>
       </c>
@@ -4259,9 +4267,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:11">
-      <c r="A104" s="5"/>
-      <c r="B104" s="5"/>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="4"/>
+      <c r="B104" s="4"/>
       <c r="C104" s="2" t="s">
         <v>136</v>
       </c>
@@ -4290,9 +4298,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
-      <c r="A105" s="5"/>
-      <c r="B105" s="5"/>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A105" s="4"/>
+      <c r="B105" s="4"/>
       <c r="C105" s="2" t="s">
         <v>137</v>
       </c>
@@ -4321,9 +4329,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
-      <c r="A106" s="5"/>
-      <c r="B106" s="5"/>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A106" s="4"/>
+      <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
         <v>138</v>
       </c>
@@ -4352,9 +4360,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
-      <c r="A107" s="5"/>
-      <c r="B107" s="5"/>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A107" s="4"/>
+      <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
         <v>139</v>
       </c>
@@ -4383,9 +4391,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:11">
-      <c r="A108" s="5"/>
-      <c r="B108" s="5" t="s">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A108" s="4"/>
+      <c r="B108" s="4" t="s">
         <v>140</v>
       </c>
       <c r="C108" s="2" t="s">
@@ -4416,9 +4424,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:11">
-      <c r="A109" s="5"/>
-      <c r="B109" s="5"/>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A109" s="4"/>
+      <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
         <v>142</v>
       </c>
@@ -4447,9 +4455,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:11">
-      <c r="A110" s="5"/>
-      <c r="B110" s="5"/>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A110" s="4"/>
+      <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
         <v>143</v>
       </c>
@@ -4478,9 +4486,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:11">
-      <c r="A111" s="5"/>
-      <c r="B111" s="5" t="s">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A111" s="4"/>
+      <c r="B111" s="4" t="s">
         <v>144</v>
       </c>
       <c r="C111" s="2" t="s">
@@ -4511,9 +4519,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:11">
-      <c r="A112" s="5"/>
-      <c r="B112" s="5"/>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A112" s="4"/>
+      <c r="B112" s="4"/>
       <c r="C112" s="2" t="s">
         <v>146</v>
       </c>
@@ -4542,9 +4550,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:11">
-      <c r="A113" s="5"/>
-      <c r="B113" s="5"/>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113" s="4"/>
+      <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
         <v>147</v>
       </c>
@@ -4573,9 +4581,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:11">
-      <c r="A114" s="5"/>
-      <c r="B114" s="5"/>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114" s="4"/>
+      <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
         <v>148</v>
       </c>
@@ -4604,9 +4612,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:11">
-      <c r="A115" s="5"/>
-      <c r="B115" s="5"/>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" s="4"/>
+      <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
         <v>149</v>
       </c>
@@ -4635,9 +4643,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:11">
-      <c r="A116" s="5"/>
-      <c r="B116" s="5" t="s">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" s="4"/>
+      <c r="B116" s="4" t="s">
         <v>150</v>
       </c>
       <c r="C116" s="2" t="s">
@@ -4668,9 +4676,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:11">
-      <c r="A117" s="5"/>
-      <c r="B117" s="5"/>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" s="4"/>
+      <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
         <v>152</v>
       </c>
@@ -4699,9 +4707,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:11">
-      <c r="A118" s="5"/>
-      <c r="B118" s="5"/>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" s="4"/>
+      <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
         <v>153</v>
       </c>
@@ -4730,9 +4738,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:11">
-      <c r="A119" s="5"/>
-      <c r="B119" s="5"/>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119" s="4"/>
+      <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
         <v>154</v>
       </c>
@@ -4761,9 +4769,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:11">
-      <c r="A120" s="5"/>
-      <c r="B120" s="5"/>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120" s="4"/>
+      <c r="B120" s="4"/>
       <c r="C120" s="2" t="s">
         <v>155</v>
       </c>
@@ -4792,9 +4800,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:11">
-      <c r="A121" s="5"/>
-      <c r="B121" s="5"/>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121" s="4"/>
+      <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
         <v>156</v>
       </c>
@@ -4823,9 +4831,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:11">
-      <c r="A122" s="5"/>
-      <c r="B122" s="5"/>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A122" s="4"/>
+      <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
         <v>157</v>
       </c>
@@ -4854,9 +4862,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:11">
-      <c r="A123" s="5"/>
-      <c r="B123" s="5" t="s">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A123" s="4"/>
+      <c r="B123" s="4" t="s">
         <v>158</v>
       </c>
       <c r="C123" s="2" t="s">
@@ -4887,9 +4895,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:11">
-      <c r="A124" s="5"/>
-      <c r="B124" s="5"/>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="4"/>
+      <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
         <v>160</v>
       </c>
@@ -4918,9 +4926,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:11">
-      <c r="A125" s="5"/>
-      <c r="B125" s="5"/>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="4"/>
+      <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
         <v>161</v>
       </c>
@@ -4949,9 +4957,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:11">
-      <c r="A126" s="5"/>
-      <c r="B126" s="5"/>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A126" s="4"/>
+      <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
         <v>162</v>
       </c>
@@ -4980,9 +4988,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:11">
-      <c r="A127" s="5"/>
-      <c r="B127" s="5"/>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A127" s="4"/>
+      <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
         <v>163</v>
       </c>
@@ -5011,11 +5019,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:11">
-      <c r="A128" s="5" t="s">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A128" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="B128" s="4" t="s">
         <v>165</v>
       </c>
       <c r="C128" t="s">
@@ -5046,9 +5054,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:11">
-      <c r="A129" s="5"/>
-      <c r="B129" s="5"/>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A129" s="4"/>
+      <c r="B129" s="4"/>
       <c r="C129" s="3" t="s">
         <v>167</v>
       </c>
@@ -5077,9 +5085,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:11">
-      <c r="A130" s="5"/>
-      <c r="B130" s="5"/>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A130" s="4"/>
+      <c r="B130" s="4"/>
       <c r="C130" s="3" t="s">
         <v>187</v>
       </c>
@@ -5108,11 +5116,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:11">
-      <c r="A131" s="5" t="s">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A131" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="5" t="s">
+      <c r="B131" s="4" t="s">
         <v>169</v>
       </c>
       <c r="C131" t="s">
@@ -5143,9 +5151,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:11">
-      <c r="A132" s="5"/>
-      <c r="B132" s="5"/>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A132" s="4"/>
+      <c r="B132" s="4"/>
       <c r="C132" t="s">
         <v>171</v>
       </c>
@@ -5174,9 +5182,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:11">
-      <c r="A133" s="5"/>
-      <c r="B133" s="5"/>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A133" s="4"/>
+      <c r="B133" s="4"/>
       <c r="C133" t="s">
         <v>172</v>
       </c>
@@ -5205,9 +5213,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:11">
-      <c r="A134" s="5"/>
-      <c r="B134" s="5"/>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A134" s="4"/>
+      <c r="B134" s="4"/>
       <c r="C134" t="s">
         <v>173</v>
       </c>
@@ -5236,9 +5244,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:11">
-      <c r="A135" s="5"/>
-      <c r="B135" s="5"/>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A135" s="4"/>
+      <c r="B135" s="4"/>
       <c r="C135" t="s">
         <v>174</v>
       </c>
@@ -5267,9 +5275,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:11">
-      <c r="A136" s="5"/>
-      <c r="B136" s="5"/>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A136" s="4"/>
+      <c r="B136" s="4"/>
       <c r="C136" t="s">
         <v>175</v>
       </c>
@@ -5298,11 +5306,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:11">
-      <c r="A137" s="5" t="s">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A137" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="B137" s="4" t="s">
         <v>177</v>
       </c>
       <c r="C137" t="s">
@@ -5333,9 +5341,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:11">
-      <c r="A138" s="5"/>
-      <c r="B138" s="5"/>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="4"/>
+      <c r="B138" s="4"/>
       <c r="C138" t="s">
         <v>179</v>
       </c>
@@ -5364,9 +5372,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:11">
-      <c r="A139" s="5"/>
-      <c r="B139" s="5"/>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="4"/>
+      <c r="B139" s="4"/>
       <c r="C139" t="s">
         <v>180</v>
       </c>
@@ -5395,9 +5403,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:11">
-      <c r="A140" s="5"/>
-      <c r="B140" s="5"/>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A140" s="4"/>
+      <c r="B140" s="4"/>
       <c r="C140" t="s">
         <v>181</v>
       </c>
@@ -5426,9 +5434,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:11">
-      <c r="A141" s="5"/>
-      <c r="B141" s="5"/>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A141" s="4"/>
+      <c r="B141" s="4"/>
       <c r="C141" t="s">
         <v>182</v>
       </c>
@@ -5457,9 +5465,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:11">
-      <c r="A142" s="5"/>
-      <c r="B142" s="5" t="s">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A142" s="4"/>
+      <c r="B142" s="4" t="s">
         <v>183</v>
       </c>
       <c r="C142" t="s">
@@ -5490,9 +5498,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:11">
-      <c r="A143" s="5"/>
-      <c r="B143" s="5"/>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A143" s="4"/>
+      <c r="B143" s="4"/>
       <c r="C143" t="s">
         <v>185</v>
       </c>
@@ -5521,7 +5529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:11">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>164</v>
       </c>
@@ -5556,25 +5564,151 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="3:3">
-      <c r="C145" s="4"/>
-    </row>
-    <row r="146" spans="3:3">
-      <c r="C146" s="4"/>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C145" t="s">
+        <v>190</v>
+      </c>
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145">
+        <v>0</v>
+      </c>
+      <c r="G145">
+        <v>0</v>
+      </c>
+      <c r="H145">
+        <v>0</v>
+      </c>
+      <c r="I145">
+        <v>0</v>
+      </c>
+      <c r="J145">
+        <v>0</v>
+      </c>
+      <c r="K145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A146" s="4"/>
+      <c r="B146" s="4"/>
+      <c r="C146" t="s">
+        <v>191</v>
+      </c>
+      <c r="D146">
+        <v>1</v>
+      </c>
+      <c r="E146">
+        <v>1</v>
+      </c>
+      <c r="F146">
+        <v>1</v>
+      </c>
+      <c r="G146">
+        <v>1</v>
+      </c>
+      <c r="H146">
+        <v>1</v>
+      </c>
+      <c r="I146">
+        <v>0</v>
+      </c>
+      <c r="J146">
+        <v>0</v>
+      </c>
+      <c r="K146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A147" s="4"/>
+      <c r="B147" s="4"/>
+      <c r="C147" t="s">
+        <v>192</v>
+      </c>
+      <c r="D147">
+        <v>1</v>
+      </c>
+      <c r="E147">
+        <v>1</v>
+      </c>
+      <c r="F147">
+        <v>0</v>
+      </c>
+      <c r="G147">
+        <v>0</v>
+      </c>
+      <c r="H147">
+        <v>0</v>
+      </c>
+      <c r="I147">
+        <v>0</v>
+      </c>
+      <c r="J147">
+        <v>0</v>
+      </c>
+      <c r="K147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A148" s="4"/>
+      <c r="B148" s="4"/>
+      <c r="C148" t="s">
+        <v>193</v>
+      </c>
+      <c r="D148">
+        <v>1</v>
+      </c>
+      <c r="E148">
+        <v>1</v>
+      </c>
+      <c r="F148">
+        <v>0</v>
+      </c>
+      <c r="G148">
+        <v>0</v>
+      </c>
+      <c r="H148">
+        <v>0</v>
+      </c>
+      <c r="I148">
+        <v>0</v>
+      </c>
+      <c r="J148">
+        <v>0</v>
+      </c>
+      <c r="K148">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
+  <mergeCells count="39">
+    <mergeCell ref="A145:A148"/>
+    <mergeCell ref="B145:B148"/>
+    <mergeCell ref="A102:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A131:A136"/>
+    <mergeCell ref="A137:A143"/>
+    <mergeCell ref="B102:B107"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B111:B115"/>
+    <mergeCell ref="B116:B122"/>
+    <mergeCell ref="B123:B127"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B131:B136"/>
+    <mergeCell ref="B137:B141"/>
+    <mergeCell ref="B142:B143"/>
     <mergeCell ref="A67:A86"/>
     <mergeCell ref="A87:A101"/>
     <mergeCell ref="B47:B51"/>
@@ -5588,19 +5722,17 @@
     <mergeCell ref="B87:B91"/>
     <mergeCell ref="B92:B96"/>
     <mergeCell ref="B97:B101"/>
-    <mergeCell ref="A102:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A131:A136"/>
-    <mergeCell ref="A137:A143"/>
-    <mergeCell ref="B102:B107"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B111:B115"/>
-    <mergeCell ref="B116:B122"/>
-    <mergeCell ref="B123:B127"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B136"/>
-    <mergeCell ref="B137:B141"/>
-    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5608,15 +5740,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5625,6 +5748,15 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5817,20 +5949,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Added settings:* permissions (#319)
* Added settings perms to excel file in helpers

* Updated role_mapping.json
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE6D5C1-5850-4799-8E3E-6CD3A8E2F55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C568B3-4200-4E26-89A8-7C948583B1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="194">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -636,13 +636,31 @@
   </si>
   <si>
     <t>permission:delete</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>settings</t>
+  </si>
+  <si>
+    <t>settings:create</t>
+  </si>
+  <si>
+    <t>settings:view</t>
+  </si>
+  <si>
+    <t>settings:update</t>
+  </si>
+  <si>
+    <t>settings:delete</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -671,13 +689,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF6AAB73"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-      <charset val="238"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -705,16 +716,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -998,8 +1006,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K146"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:K148"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -1014,7 +1022,7 @@
     <col min="11" max="11" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" t="s">
@@ -1045,11 +1053,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
@@ -1080,9 +1088,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -1111,9 +1119,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
       <c r="C4" t="s">
         <v>13</v>
       </c>
@@ -1142,9 +1150,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
       <c r="C5" t="s">
         <v>14</v>
       </c>
@@ -1173,9 +1181,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
       <c r="C6" t="s">
         <v>15</v>
       </c>
@@ -1204,9 +1212,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
@@ -1237,9 +1245,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
       <c r="C8" t="s">
         <v>18</v>
       </c>
@@ -1268,9 +1276,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -1299,9 +1307,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
       <c r="C10" t="s">
         <v>20</v>
       </c>
@@ -1330,9 +1338,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
       <c r="C11" t="s">
         <v>21</v>
       </c>
@@ -1361,9 +1369,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C12" t="s">
@@ -1394,9 +1402,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
       <c r="C13" t="s">
         <v>24</v>
       </c>
@@ -1425,9 +1433,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
       <c r="C14" t="s">
         <v>25</v>
       </c>
@@ -1456,9 +1464,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
       <c r="C15" t="s">
         <v>26</v>
       </c>
@@ -1487,9 +1495,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
       <c r="C16" t="s">
         <v>27</v>
       </c>
@@ -1518,9 +1526,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5" t="s">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C17" t="s">
@@ -1551,9 +1559,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
       <c r="C18" t="s">
         <v>30</v>
       </c>
@@ -1582,9 +1590,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
       <c r="C19" t="s">
         <v>31</v>
       </c>
@@ -1613,9 +1621,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
       <c r="C20" t="s">
         <v>32</v>
       </c>
@@ -1644,9 +1652,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
       <c r="C21" t="s">
         <v>33</v>
       </c>
@@ -1675,9 +1683,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5" t="s">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C22" t="s">
@@ -1708,9 +1716,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
       <c r="C23" t="s">
         <v>36</v>
       </c>
@@ -1739,9 +1747,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
       <c r="C24" t="s">
         <v>37</v>
       </c>
@@ -1770,9 +1778,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
       <c r="C25" t="s">
         <v>38</v>
       </c>
@@ -1801,9 +1809,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
       <c r="C26" t="s">
         <v>39</v>
       </c>
@@ -1832,11 +1840,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C27" t="s">
@@ -1867,9 +1875,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
       <c r="C28" t="s">
         <v>43</v>
       </c>
@@ -1898,9 +1906,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
       <c r="C29" t="s">
         <v>44</v>
       </c>
@@ -1929,9 +1937,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
       <c r="C30" t="s">
         <v>45</v>
       </c>
@@ -1960,9 +1968,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
       <c r="C31" t="s">
         <v>46</v>
       </c>
@@ -1991,9 +1999,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4" t="s">
         <v>47</v>
       </c>
       <c r="C32" t="s">
@@ -2024,9 +2032,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
       <c r="C33" t="s">
         <v>49</v>
       </c>
@@ -2055,9 +2063,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
       <c r="C34" t="s">
         <v>50</v>
       </c>
@@ -2086,9 +2094,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
       <c r="C35" t="s">
         <v>51</v>
       </c>
@@ -2117,9 +2125,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
       <c r="C36" t="s">
         <v>52</v>
       </c>
@@ -2148,9 +2156,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C37" t="s">
@@ -2181,9 +2189,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
       <c r="C38" t="s">
         <v>55</v>
       </c>
@@ -2212,9 +2220,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
       <c r="C39" t="s">
         <v>56</v>
       </c>
@@ -2243,9 +2251,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
       <c r="C40" t="s">
         <v>57</v>
       </c>
@@ -2274,9 +2282,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
       <c r="C41" t="s">
         <v>58</v>
       </c>
@@ -2305,9 +2313,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="4"/>
+      <c r="B42" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C42" t="s">
@@ -2338,9 +2346,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
       <c r="C43" t="s">
         <v>61</v>
       </c>
@@ -2369,9 +2377,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
       <c r="C44" t="s">
         <v>62</v>
       </c>
@@ -2400,9 +2408,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
       <c r="C45" t="s">
         <v>63</v>
       </c>
@@ -2431,9 +2439,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
       <c r="C46" t="s">
         <v>64</v>
       </c>
@@ -2462,9 +2470,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5" t="s">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="4"/>
+      <c r="B47" s="4" t="s">
         <v>65</v>
       </c>
       <c r="C47" t="s">
@@ -2495,9 +2503,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
       <c r="C48" t="s">
         <v>67</v>
       </c>
@@ -2526,9 +2534,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" s="4"/>
+      <c r="B49" s="4"/>
       <c r="C49" t="s">
         <v>68</v>
       </c>
@@ -2557,9 +2565,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2588,9 +2596,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
       <c r="C51" t="s">
         <v>70</v>
       </c>
@@ -2619,9 +2627,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5" t="s">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="4"/>
+      <c r="B52" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C52" t="s">
@@ -2652,9 +2660,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:11">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" s="4"/>
+      <c r="B53" s="4"/>
       <c r="C53" t="s">
         <v>72</v>
       </c>
@@ -2683,9 +2691,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:11">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
       <c r="C54" t="s">
         <v>73</v>
       </c>
@@ -2714,9 +2722,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
       <c r="C55" t="s">
         <v>74</v>
       </c>
@@ -2745,9 +2753,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="4"/>
+      <c r="B56" s="4"/>
       <c r="C56" t="s">
         <v>75</v>
       </c>
@@ -2776,9 +2784,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5" t="s">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" s="4"/>
+      <c r="B57" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C57" t="s">
@@ -2809,9 +2817,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:11">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
       <c r="C58" t="s">
         <v>78</v>
       </c>
@@ -2840,9 +2848,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:11">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
       <c r="C59" t="s">
         <v>79</v>
       </c>
@@ -2871,9 +2879,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
       <c r="C60" t="s">
         <v>80</v>
       </c>
@@ -2902,9 +2910,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
       <c r="C61" t="s">
         <v>81</v>
       </c>
@@ -2933,9 +2941,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5" t="s">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" s="4"/>
+      <c r="B62" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C62" t="s">
@@ -2966,9 +2974,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:11">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
       <c r="C63" t="s">
         <v>84</v>
       </c>
@@ -2997,9 +3005,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
       <c r="C64" t="s">
         <v>85</v>
       </c>
@@ -3028,9 +3036,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:11">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
       <c r="C65" t="s">
         <v>86</v>
       </c>
@@ -3059,9 +3067,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:11">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
       <c r="C66" t="s">
         <v>87</v>
       </c>
@@ -3090,11 +3098,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:11">
-      <c r="A67" s="5" t="s">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="4" t="s">
         <v>89</v>
       </c>
       <c r="C67" t="s">
@@ -3125,9 +3133,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:11">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
       <c r="C68" t="s">
         <v>91</v>
       </c>
@@ -3156,9 +3164,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:11">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
       <c r="C69" t="s">
         <v>92</v>
       </c>
@@ -3187,9 +3195,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:11">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" s="4"/>
+      <c r="B70" s="4"/>
       <c r="C70" t="s">
         <v>93</v>
       </c>
@@ -3218,9 +3226,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:11">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
       <c r="C71" t="s">
         <v>94</v>
       </c>
@@ -3249,9 +3257,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:11">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5" t="s">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" s="4"/>
+      <c r="B72" s="4" t="s">
         <v>95</v>
       </c>
       <c r="C72" t="s">
@@ -3282,9 +3290,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:11">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" s="4"/>
+      <c r="B73" s="4"/>
       <c r="C73" t="s">
         <v>97</v>
       </c>
@@ -3313,9 +3321,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" s="4"/>
+      <c r="B74" s="4"/>
       <c r="C74" t="s">
         <v>98</v>
       </c>
@@ -3344,9 +3352,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:11">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" s="4"/>
+      <c r="B75" s="4"/>
       <c r="C75" t="s">
         <v>99</v>
       </c>
@@ -3375,9 +3383,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:11">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
       <c r="C76" t="s">
         <v>100</v>
       </c>
@@ -3406,9 +3414,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:11">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5" t="s">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77" s="4"/>
+      <c r="B77" s="4" t="s">
         <v>101</v>
       </c>
       <c r="C77" t="s">
@@ -3439,9 +3447,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:11">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+      <c r="B78" s="4"/>
       <c r="C78" t="s">
         <v>103</v>
       </c>
@@ -3470,9 +3478,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79" s="4"/>
+      <c r="B79" s="4"/>
       <c r="C79" t="s">
         <v>104</v>
       </c>
@@ -3501,9 +3509,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:11">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80" s="4"/>
+      <c r="B80" s="4"/>
       <c r="C80" t="s">
         <v>105</v>
       </c>
@@ -3532,9 +3540,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:11">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81" s="4"/>
+      <c r="B81" s="4"/>
       <c r="C81" t="s">
         <v>106</v>
       </c>
@@ -3563,9 +3571,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:11">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5" t="s">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82" s="4"/>
+      <c r="B82" s="4" t="s">
         <v>107</v>
       </c>
       <c r="C82" t="s">
@@ -3596,9 +3604,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:11">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83" s="4"/>
+      <c r="B83" s="4"/>
       <c r="C83" t="s">
         <v>109</v>
       </c>
@@ -3627,9 +3635,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:11">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84" s="4"/>
+      <c r="B84" s="4"/>
       <c r="C84" t="s">
         <v>110</v>
       </c>
@@ -3658,9 +3666,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:11">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85" s="4"/>
+      <c r="B85" s="4"/>
       <c r="C85" t="s">
         <v>111</v>
       </c>
@@ -3689,9 +3697,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:11">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86" s="4"/>
+      <c r="B86" s="4"/>
       <c r="C86" t="s">
         <v>112</v>
       </c>
@@ -3720,11 +3728,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:11">
-      <c r="A87" s="5" t="s">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C87" t="s">
@@ -3755,9 +3763,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:11">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88" s="4"/>
+      <c r="B88" s="4"/>
       <c r="C88" t="s">
         <v>116</v>
       </c>
@@ -3786,9 +3794,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:11">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89" s="4"/>
+      <c r="B89" s="4"/>
       <c r="C89" t="s">
         <v>117</v>
       </c>
@@ -3817,9 +3825,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:11">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90" s="4"/>
+      <c r="B90" s="4"/>
       <c r="C90" t="s">
         <v>118</v>
       </c>
@@ -3848,9 +3856,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:11">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91" s="4"/>
+      <c r="B91" s="4"/>
       <c r="C91" t="s">
         <v>119</v>
       </c>
@@ -3879,9 +3887,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:11">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5" t="s">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92" s="4"/>
+      <c r="B92" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C92" t="s">
@@ -3912,9 +3920,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:11">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93" s="4"/>
+      <c r="B93" s="4"/>
       <c r="C93" t="s">
         <v>122</v>
       </c>
@@ -3943,9 +3951,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:11">
-      <c r="A94" s="5"/>
-      <c r="B94" s="5"/>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94" s="4"/>
+      <c r="B94" s="4"/>
       <c r="C94" t="s">
         <v>123</v>
       </c>
@@ -3974,9 +3982,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:11">
-      <c r="A95" s="5"/>
-      <c r="B95" s="5"/>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95" s="4"/>
+      <c r="B95" s="4"/>
       <c r="C95" t="s">
         <v>124</v>
       </c>
@@ -4005,9 +4013,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:11">
-      <c r="A96" s="5"/>
-      <c r="B96" s="5"/>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A96" s="4"/>
+      <c r="B96" s="4"/>
       <c r="C96" t="s">
         <v>125</v>
       </c>
@@ -4036,9 +4044,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
-      <c r="A97" s="5"/>
-      <c r="B97" s="5" t="s">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97" s="4"/>
+      <c r="B97" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C97" t="s">
@@ -4069,9 +4077,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
-      <c r="A98" s="5"/>
-      <c r="B98" s="5"/>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98" s="4"/>
+      <c r="B98" s="4"/>
       <c r="C98" t="s">
         <v>128</v>
       </c>
@@ -4100,9 +4108,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:11">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99" s="4"/>
+      <c r="B99" s="4"/>
       <c r="C99" t="s">
         <v>129</v>
       </c>
@@ -4131,9 +4139,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:11">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100" s="4"/>
+      <c r="B100" s="4"/>
       <c r="C100" t="s">
         <v>130</v>
       </c>
@@ -4162,9 +4170,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:11">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A101" s="4"/>
+      <c r="B101" s="4"/>
       <c r="C101" t="s">
         <v>131</v>
       </c>
@@ -4193,11 +4201,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:11">
-      <c r="A102" s="5" t="s">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B102" s="4" t="s">
         <v>133</v>
       </c>
       <c r="C102" s="2" t="s">
@@ -4228,9 +4236,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:11">
-      <c r="A103" s="5"/>
-      <c r="B103" s="5"/>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" s="4"/>
+      <c r="B103" s="4"/>
       <c r="C103" s="2" t="s">
         <v>135</v>
       </c>
@@ -4259,9 +4267,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:11">
-      <c r="A104" s="5"/>
-      <c r="B104" s="5"/>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="4"/>
+      <c r="B104" s="4"/>
       <c r="C104" s="2" t="s">
         <v>136</v>
       </c>
@@ -4290,9 +4298,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
-      <c r="A105" s="5"/>
-      <c r="B105" s="5"/>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A105" s="4"/>
+      <c r="B105" s="4"/>
       <c r="C105" s="2" t="s">
         <v>137</v>
       </c>
@@ -4321,9 +4329,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
-      <c r="A106" s="5"/>
-      <c r="B106" s="5"/>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A106" s="4"/>
+      <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
         <v>138</v>
       </c>
@@ -4352,9 +4360,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
-      <c r="A107" s="5"/>
-      <c r="B107" s="5"/>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A107" s="4"/>
+      <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
         <v>139</v>
       </c>
@@ -4383,9 +4391,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:11">
-      <c r="A108" s="5"/>
-      <c r="B108" s="5" t="s">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A108" s="4"/>
+      <c r="B108" s="4" t="s">
         <v>140</v>
       </c>
       <c r="C108" s="2" t="s">
@@ -4416,9 +4424,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:11">
-      <c r="A109" s="5"/>
-      <c r="B109" s="5"/>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A109" s="4"/>
+      <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
         <v>142</v>
       </c>
@@ -4447,9 +4455,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:11">
-      <c r="A110" s="5"/>
-      <c r="B110" s="5"/>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A110" s="4"/>
+      <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
         <v>143</v>
       </c>
@@ -4478,9 +4486,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:11">
-      <c r="A111" s="5"/>
-      <c r="B111" s="5" t="s">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A111" s="4"/>
+      <c r="B111" s="4" t="s">
         <v>144</v>
       </c>
       <c r="C111" s="2" t="s">
@@ -4511,9 +4519,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:11">
-      <c r="A112" s="5"/>
-      <c r="B112" s="5"/>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A112" s="4"/>
+      <c r="B112" s="4"/>
       <c r="C112" s="2" t="s">
         <v>146</v>
       </c>
@@ -4542,9 +4550,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:11">
-      <c r="A113" s="5"/>
-      <c r="B113" s="5"/>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113" s="4"/>
+      <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
         <v>147</v>
       </c>
@@ -4573,9 +4581,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:11">
-      <c r="A114" s="5"/>
-      <c r="B114" s="5"/>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114" s="4"/>
+      <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
         <v>148</v>
       </c>
@@ -4604,9 +4612,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:11">
-      <c r="A115" s="5"/>
-      <c r="B115" s="5"/>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" s="4"/>
+      <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
         <v>149</v>
       </c>
@@ -4635,9 +4643,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:11">
-      <c r="A116" s="5"/>
-      <c r="B116" s="5" t="s">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" s="4"/>
+      <c r="B116" s="4" t="s">
         <v>150</v>
       </c>
       <c r="C116" s="2" t="s">
@@ -4668,9 +4676,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:11">
-      <c r="A117" s="5"/>
-      <c r="B117" s="5"/>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" s="4"/>
+      <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
         <v>152</v>
       </c>
@@ -4699,9 +4707,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:11">
-      <c r="A118" s="5"/>
-      <c r="B118" s="5"/>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" s="4"/>
+      <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
         <v>153</v>
       </c>
@@ -4730,9 +4738,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:11">
-      <c r="A119" s="5"/>
-      <c r="B119" s="5"/>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119" s="4"/>
+      <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
         <v>154</v>
       </c>
@@ -4761,9 +4769,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:11">
-      <c r="A120" s="5"/>
-      <c r="B120" s="5"/>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120" s="4"/>
+      <c r="B120" s="4"/>
       <c r="C120" s="2" t="s">
         <v>155</v>
       </c>
@@ -4792,9 +4800,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:11">
-      <c r="A121" s="5"/>
-      <c r="B121" s="5"/>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121" s="4"/>
+      <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
         <v>156</v>
       </c>
@@ -4823,9 +4831,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:11">
-      <c r="A122" s="5"/>
-      <c r="B122" s="5"/>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A122" s="4"/>
+      <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
         <v>157</v>
       </c>
@@ -4854,9 +4862,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:11">
-      <c r="A123" s="5"/>
-      <c r="B123" s="5" t="s">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A123" s="4"/>
+      <c r="B123" s="4" t="s">
         <v>158</v>
       </c>
       <c r="C123" s="2" t="s">
@@ -4887,9 +4895,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:11">
-      <c r="A124" s="5"/>
-      <c r="B124" s="5"/>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="4"/>
+      <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
         <v>160</v>
       </c>
@@ -4918,9 +4926,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:11">
-      <c r="A125" s="5"/>
-      <c r="B125" s="5"/>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="4"/>
+      <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
         <v>161</v>
       </c>
@@ -4949,9 +4957,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:11">
-      <c r="A126" s="5"/>
-      <c r="B126" s="5"/>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A126" s="4"/>
+      <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
         <v>162</v>
       </c>
@@ -4980,9 +4988,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:11">
-      <c r="A127" s="5"/>
-      <c r="B127" s="5"/>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A127" s="4"/>
+      <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
         <v>163</v>
       </c>
@@ -5011,11 +5019,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:11">
-      <c r="A128" s="5" t="s">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A128" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="B128" s="4" t="s">
         <v>165</v>
       </c>
       <c r="C128" t="s">
@@ -5046,9 +5054,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:11">
-      <c r="A129" s="5"/>
-      <c r="B129" s="5"/>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A129" s="4"/>
+      <c r="B129" s="4"/>
       <c r="C129" s="3" t="s">
         <v>167</v>
       </c>
@@ -5077,9 +5085,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:11">
-      <c r="A130" s="5"/>
-      <c r="B130" s="5"/>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A130" s="4"/>
+      <c r="B130" s="4"/>
       <c r="C130" s="3" t="s">
         <v>187</v>
       </c>
@@ -5108,11 +5116,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:11">
-      <c r="A131" s="5" t="s">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A131" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="5" t="s">
+      <c r="B131" s="4" t="s">
         <v>169</v>
       </c>
       <c r="C131" t="s">
@@ -5143,9 +5151,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:11">
-      <c r="A132" s="5"/>
-      <c r="B132" s="5"/>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A132" s="4"/>
+      <c r="B132" s="4"/>
       <c r="C132" t="s">
         <v>171</v>
       </c>
@@ -5174,9 +5182,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:11">
-      <c r="A133" s="5"/>
-      <c r="B133" s="5"/>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A133" s="4"/>
+      <c r="B133" s="4"/>
       <c r="C133" t="s">
         <v>172</v>
       </c>
@@ -5205,9 +5213,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:11">
-      <c r="A134" s="5"/>
-      <c r="B134" s="5"/>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A134" s="4"/>
+      <c r="B134" s="4"/>
       <c r="C134" t="s">
         <v>173</v>
       </c>
@@ -5236,9 +5244,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:11">
-      <c r="A135" s="5"/>
-      <c r="B135" s="5"/>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A135" s="4"/>
+      <c r="B135" s="4"/>
       <c r="C135" t="s">
         <v>174</v>
       </c>
@@ -5267,9 +5275,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:11">
-      <c r="A136" s="5"/>
-      <c r="B136" s="5"/>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A136" s="4"/>
+      <c r="B136" s="4"/>
       <c r="C136" t="s">
         <v>175</v>
       </c>
@@ -5298,11 +5306,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:11">
-      <c r="A137" s="5" t="s">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A137" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="B137" s="4" t="s">
         <v>177</v>
       </c>
       <c r="C137" t="s">
@@ -5333,9 +5341,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:11">
-      <c r="A138" s="5"/>
-      <c r="B138" s="5"/>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="4"/>
+      <c r="B138" s="4"/>
       <c r="C138" t="s">
         <v>179</v>
       </c>
@@ -5364,9 +5372,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:11">
-      <c r="A139" s="5"/>
-      <c r="B139" s="5"/>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="4"/>
+      <c r="B139" s="4"/>
       <c r="C139" t="s">
         <v>180</v>
       </c>
@@ -5395,9 +5403,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:11">
-      <c r="A140" s="5"/>
-      <c r="B140" s="5"/>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A140" s="4"/>
+      <c r="B140" s="4"/>
       <c r="C140" t="s">
         <v>181</v>
       </c>
@@ -5426,9 +5434,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:11">
-      <c r="A141" s="5"/>
-      <c r="B141" s="5"/>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A141" s="4"/>
+      <c r="B141" s="4"/>
       <c r="C141" t="s">
         <v>182</v>
       </c>
@@ -5457,9 +5465,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:11">
-      <c r="A142" s="5"/>
-      <c r="B142" s="5" t="s">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A142" s="4"/>
+      <c r="B142" s="4" t="s">
         <v>183</v>
       </c>
       <c r="C142" t="s">
@@ -5490,9 +5498,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:11">
-      <c r="A143" s="5"/>
-      <c r="B143" s="5"/>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A143" s="4"/>
+      <c r="B143" s="4"/>
       <c r="C143" t="s">
         <v>185</v>
       </c>
@@ -5521,7 +5529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:11">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>164</v>
       </c>
@@ -5556,25 +5564,151 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="3:3">
-      <c r="C145" s="4"/>
-    </row>
-    <row r="146" spans="3:3">
-      <c r="C146" s="4"/>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C145" t="s">
+        <v>190</v>
+      </c>
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145">
+        <v>0</v>
+      </c>
+      <c r="G145">
+        <v>0</v>
+      </c>
+      <c r="H145">
+        <v>0</v>
+      </c>
+      <c r="I145">
+        <v>0</v>
+      </c>
+      <c r="J145">
+        <v>0</v>
+      </c>
+      <c r="K145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A146" s="4"/>
+      <c r="B146" s="4"/>
+      <c r="C146" t="s">
+        <v>191</v>
+      </c>
+      <c r="D146">
+        <v>1</v>
+      </c>
+      <c r="E146">
+        <v>1</v>
+      </c>
+      <c r="F146">
+        <v>1</v>
+      </c>
+      <c r="G146">
+        <v>1</v>
+      </c>
+      <c r="H146">
+        <v>1</v>
+      </c>
+      <c r="I146">
+        <v>0</v>
+      </c>
+      <c r="J146">
+        <v>0</v>
+      </c>
+      <c r="K146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A147" s="4"/>
+      <c r="B147" s="4"/>
+      <c r="C147" t="s">
+        <v>192</v>
+      </c>
+      <c r="D147">
+        <v>1</v>
+      </c>
+      <c r="E147">
+        <v>1</v>
+      </c>
+      <c r="F147">
+        <v>0</v>
+      </c>
+      <c r="G147">
+        <v>0</v>
+      </c>
+      <c r="H147">
+        <v>0</v>
+      </c>
+      <c r="I147">
+        <v>0</v>
+      </c>
+      <c r="J147">
+        <v>0</v>
+      </c>
+      <c r="K147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A148" s="4"/>
+      <c r="B148" s="4"/>
+      <c r="C148" t="s">
+        <v>193</v>
+      </c>
+      <c r="D148">
+        <v>1</v>
+      </c>
+      <c r="E148">
+        <v>1</v>
+      </c>
+      <c r="F148">
+        <v>0</v>
+      </c>
+      <c r="G148">
+        <v>0</v>
+      </c>
+      <c r="H148">
+        <v>0</v>
+      </c>
+      <c r="I148">
+        <v>0</v>
+      </c>
+      <c r="J148">
+        <v>0</v>
+      </c>
+      <c r="K148">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
+  <mergeCells count="39">
+    <mergeCell ref="A145:A148"/>
+    <mergeCell ref="B145:B148"/>
+    <mergeCell ref="A102:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A131:A136"/>
+    <mergeCell ref="A137:A143"/>
+    <mergeCell ref="B102:B107"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B111:B115"/>
+    <mergeCell ref="B116:B122"/>
+    <mergeCell ref="B123:B127"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B131:B136"/>
+    <mergeCell ref="B137:B141"/>
+    <mergeCell ref="B142:B143"/>
     <mergeCell ref="A67:A86"/>
     <mergeCell ref="A87:A101"/>
     <mergeCell ref="B47:B51"/>
@@ -5588,19 +5722,17 @@
     <mergeCell ref="B87:B91"/>
     <mergeCell ref="B92:B96"/>
     <mergeCell ref="B97:B101"/>
-    <mergeCell ref="A102:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A131:A136"/>
-    <mergeCell ref="A137:A143"/>
-    <mergeCell ref="B102:B107"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B111:B115"/>
-    <mergeCell ref="B116:B122"/>
-    <mergeCell ref="B123:B127"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B136"/>
-    <mergeCell ref="B137:B141"/>
-    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5608,15 +5740,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5625,6 +5748,15 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5817,20 +5949,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add permission code for viewing other user's plan
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17a9e6fd9bbdd953/Dokumenty/GitHub/Smart-University-Scheduler/helpers/db_seeder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C568B3-4200-4E26-89A8-7C948583B1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{79C568B3-4200-4E26-89A8-7C948583B1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B44B7B53-20BF-4B5B-9A1D-C19D5E316ABB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="195">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -654,6 +654,9 @@
   </si>
   <si>
     <t>settings:delete</t>
+  </si>
+  <si>
+    <t>schedule:view_others</t>
   </si>
 </sst>
 </file>
@@ -741,6 +744,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1006,7 +1013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K148"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -4271,7 +4278,7 @@
       <c r="A104" s="4"/>
       <c r="B104" s="4"/>
       <c r="C104" s="2" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="D104">
         <v>1</v>
@@ -4289,20 +4296,20 @@
         <v>1</v>
       </c>
       <c r="I104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K104">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D105">
         <v>1</v>
@@ -4314,26 +4321,26 @@
         <v>1</v>
       </c>
       <c r="G105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K105">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D106">
         <v>1</v>
@@ -4364,7 +4371,7 @@
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D107">
         <v>1</v>
@@ -4376,28 +4383,26 @@
         <v>1</v>
       </c>
       <c r="G107">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H107">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I107">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J107">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K107">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="4"/>
-      <c r="B108" s="4" t="s">
-        <v>140</v>
-      </c>
+      <c r="B108" s="4"/>
       <c r="C108" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -4426,15 +4431,17 @@
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="4"/>
-      <c r="B109" s="4"/>
+      <c r="B109" s="4" t="s">
+        <v>140</v>
+      </c>
       <c r="C109" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D109">
         <v>1</v>
       </c>
       <c r="E109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F109">
         <v>1</v>
@@ -4443,23 +4450,23 @@
         <v>1</v>
       </c>
       <c r="H109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K109">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D110">
         <v>1</v>
@@ -4488,17 +4495,15 @@
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
-      <c r="B111" s="4" t="s">
-        <v>144</v>
-      </c>
+      <c r="B111" s="4"/>
       <c r="C111" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F111">
         <v>1</v>
@@ -4507,23 +4512,25 @@
         <v>1</v>
       </c>
       <c r="H111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K111">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
-      <c r="B112" s="4"/>
+      <c r="B112" s="4" t="s">
+        <v>144</v>
+      </c>
       <c r="C112" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D112">
         <v>1</v>
@@ -4554,7 +4561,7 @@
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -4566,26 +4573,26 @@
         <v>1</v>
       </c>
       <c r="G113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K113">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D114">
         <v>1</v>
@@ -4616,7 +4623,7 @@
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4645,11 +4652,9 @@
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A116" s="4"/>
-      <c r="B116" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4661,16 +4666,16 @@
         <v>1</v>
       </c>
       <c r="G116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K116">
         <v>0</v>
@@ -4678,9 +4683,11 @@
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
-      <c r="B117" s="4"/>
+      <c r="B117" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="C117" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4711,7 +4718,7 @@
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4742,7 +4749,7 @@
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4754,16 +4761,16 @@
         <v>1</v>
       </c>
       <c r="G119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K119">
         <v>0</v>
@@ -4773,7 +4780,7 @@
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4804,7 +4811,7 @@
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4835,7 +4842,7 @@
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4864,11 +4871,9 @@
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A123" s="4"/>
-      <c r="B123" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="B123" s="4"/>
       <c r="C123" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4880,16 +4885,16 @@
         <v>1</v>
       </c>
       <c r="G123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K123">
         <v>0</v>
@@ -4897,9 +4902,11 @@
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A124" s="4"/>
-      <c r="B124" s="4"/>
+      <c r="B124" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="C124" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4930,13 +4937,13 @@
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D125">
         <v>1</v>
       </c>
       <c r="E125">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F125">
         <v>1</v>
@@ -4948,10 +4955,10 @@
         <v>1</v>
       </c>
       <c r="I125">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J125">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K125">
         <v>0</v>
@@ -4961,7 +4968,7 @@
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -4992,73 +4999,73 @@
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D127">
+        <v>1</v>
+      </c>
+      <c r="E127">
+        <v>0</v>
+      </c>
+      <c r="F127">
+        <v>1</v>
+      </c>
+      <c r="G127">
+        <v>1</v>
+      </c>
+      <c r="H127">
+        <v>1</v>
+      </c>
+      <c r="I127">
+        <v>0</v>
+      </c>
+      <c r="J127">
+        <v>0</v>
+      </c>
+      <c r="K127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A128" s="4"/>
+      <c r="B128" s="4"/>
+      <c r="C128" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D127">
-        <v>1</v>
-      </c>
-      <c r="E127">
-        <v>0</v>
-      </c>
-      <c r="F127">
-        <v>1</v>
-      </c>
-      <c r="G127">
-        <v>0</v>
-      </c>
-      <c r="H127">
-        <v>0</v>
-      </c>
-      <c r="I127">
-        <v>0</v>
-      </c>
-      <c r="J127">
-        <v>0</v>
-      </c>
-      <c r="K127">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A128" s="4" t="s">
+      <c r="D128">
+        <v>1</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>1</v>
+      </c>
+      <c r="G128">
+        <v>0</v>
+      </c>
+      <c r="H128">
+        <v>0</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A129" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B129" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C128" t="s">
+      <c r="C129" t="s">
         <v>166</v>
-      </c>
-      <c r="D128">
-        <v>1</v>
-      </c>
-      <c r="E128">
-        <v>0</v>
-      </c>
-      <c r="F128">
-        <v>0</v>
-      </c>
-      <c r="G128">
-        <v>0</v>
-      </c>
-      <c r="H128">
-        <v>0</v>
-      </c>
-      <c r="I128">
-        <v>0</v>
-      </c>
-      <c r="J128">
-        <v>0</v>
-      </c>
-      <c r="K128">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A129" s="4"/>
-      <c r="B129" s="4"/>
-      <c r="C129" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -5089,73 +5096,73 @@
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D130">
+        <v>1</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>0</v>
+      </c>
+      <c r="G130">
+        <v>0</v>
+      </c>
+      <c r="H130">
+        <v>0</v>
+      </c>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A131" s="4"/>
+      <c r="B131" s="4"/>
+      <c r="C131" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D130">
-        <v>1</v>
-      </c>
-      <c r="E130">
-        <v>0</v>
-      </c>
-      <c r="F130">
-        <v>0</v>
-      </c>
-      <c r="G130">
-        <v>0</v>
-      </c>
-      <c r="H130">
-        <v>0</v>
-      </c>
-      <c r="I130">
-        <v>0</v>
-      </c>
-      <c r="J130">
-        <v>0</v>
-      </c>
-      <c r="K130">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A131" s="4" t="s">
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+      <c r="F131">
+        <v>0</v>
+      </c>
+      <c r="G131">
+        <v>0</v>
+      </c>
+      <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A132" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="4" t="s">
+      <c r="B132" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C131" t="s">
+      <c r="C132" t="s">
         <v>170</v>
-      </c>
-      <c r="D131">
-        <v>1</v>
-      </c>
-      <c r="E131">
-        <v>0</v>
-      </c>
-      <c r="F131">
-        <v>0</v>
-      </c>
-      <c r="G131">
-        <v>0</v>
-      </c>
-      <c r="H131">
-        <v>0</v>
-      </c>
-      <c r="I131">
-        <v>0</v>
-      </c>
-      <c r="J131">
-        <v>0</v>
-      </c>
-      <c r="K131">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
-      <c r="C132" t="s">
-        <v>171</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -5186,7 +5193,7 @@
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -5217,7 +5224,7 @@
       <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -5248,7 +5255,7 @@
       <c r="A135" s="4"/>
       <c r="B135" s="4"/>
       <c r="C135" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -5279,91 +5286,91 @@
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
       <c r="C136" t="s">
+        <v>174</v>
+      </c>
+      <c r="D136">
+        <v>1</v>
+      </c>
+      <c r="E136">
+        <v>0</v>
+      </c>
+      <c r="F136">
+        <v>0</v>
+      </c>
+      <c r="G136">
+        <v>0</v>
+      </c>
+      <c r="H136">
+        <v>0</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+      <c r="J136">
+        <v>0</v>
+      </c>
+      <c r="K136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A137" s="4"/>
+      <c r="B137" s="4"/>
+      <c r="C137" t="s">
         <v>175</v>
       </c>
-      <c r="D136">
-        <v>1</v>
-      </c>
-      <c r="E136">
-        <v>0</v>
-      </c>
-      <c r="F136">
-        <v>0</v>
-      </c>
-      <c r="G136">
-        <v>0</v>
-      </c>
-      <c r="H136">
-        <v>0</v>
-      </c>
-      <c r="I136">
-        <v>0</v>
-      </c>
-      <c r="J136">
-        <v>0</v>
-      </c>
-      <c r="K136">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A137" s="4" t="s">
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>0</v>
+      </c>
+      <c r="F137">
+        <v>0</v>
+      </c>
+      <c r="G137">
+        <v>0</v>
+      </c>
+      <c r="H137">
+        <v>0</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B137" s="4" t="s">
+      <c r="B138" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C137" t="s">
+      <c r="C138" t="s">
         <v>178</v>
       </c>
-      <c r="D137">
-        <v>1</v>
-      </c>
-      <c r="E137">
-        <v>1</v>
-      </c>
-      <c r="F137">
-        <v>1</v>
-      </c>
-      <c r="G137">
-        <v>1</v>
-      </c>
-      <c r="H137">
-        <v>1</v>
-      </c>
-      <c r="I137">
-        <v>1</v>
-      </c>
-      <c r="J137">
-        <v>0</v>
-      </c>
-      <c r="K137">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A138" s="4"/>
-      <c r="B138" s="4"/>
-      <c r="C138" t="s">
-        <v>179</v>
-      </c>
       <c r="D138">
         <v>1</v>
       </c>
       <c r="E138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J138">
         <v>0</v>
@@ -5376,25 +5383,25 @@
       <c r="A139" s="4"/>
       <c r="B139" s="4"/>
       <c r="C139" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D139">
         <v>1</v>
       </c>
       <c r="E139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J139">
         <v>0</v>
@@ -5407,7 +5414,7 @@
       <c r="A140" s="4"/>
       <c r="B140" s="4"/>
       <c r="C140" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D140">
         <v>1</v>
@@ -5438,7 +5445,7 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -5467,11 +5474,9 @@
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142" s="4"/>
-      <c r="B142" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -5500,111 +5505,113 @@
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" s="4"/>
-      <c r="B143" s="4"/>
+      <c r="B143" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C143" t="s">
+        <v>184</v>
+      </c>
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143">
+        <v>1</v>
+      </c>
+      <c r="G143">
+        <v>1</v>
+      </c>
+      <c r="H143">
+        <v>1</v>
+      </c>
+      <c r="I143">
+        <v>1</v>
+      </c>
+      <c r="J143">
+        <v>0</v>
+      </c>
+      <c r="K143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A144" s="4"/>
+      <c r="B144" s="4"/>
+      <c r="C144" t="s">
         <v>185</v>
       </c>
-      <c r="D143">
-        <v>1</v>
-      </c>
-      <c r="E143">
-        <v>1</v>
-      </c>
-      <c r="F143">
-        <v>1</v>
-      </c>
-      <c r="G143">
-        <v>1</v>
-      </c>
-      <c r="H143">
-        <v>1</v>
-      </c>
-      <c r="I143">
-        <v>1</v>
-      </c>
-      <c r="J143">
-        <v>0</v>
-      </c>
-      <c r="K143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A144" s="1" t="s">
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
+        <v>1</v>
+      </c>
+      <c r="H144">
+        <v>1</v>
+      </c>
+      <c r="I144">
+        <v>1</v>
+      </c>
+      <c r="J144">
+        <v>0</v>
+      </c>
+      <c r="K144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B144" s="1" t="s">
+      <c r="B145" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C144" t="s">
+      <c r="C145" t="s">
         <v>186</v>
       </c>
-      <c r="D144">
-        <v>1</v>
-      </c>
-      <c r="E144">
-        <v>1</v>
-      </c>
-      <c r="F144">
-        <v>1</v>
-      </c>
-      <c r="G144">
-        <v>1</v>
-      </c>
-      <c r="H144">
-        <v>1</v>
-      </c>
-      <c r="I144">
-        <v>1</v>
-      </c>
-      <c r="J144">
-        <v>1</v>
-      </c>
-      <c r="K144">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A145" s="4" t="s">
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145">
+        <v>1</v>
+      </c>
+      <c r="G145">
+        <v>1</v>
+      </c>
+      <c r="H145">
+        <v>1</v>
+      </c>
+      <c r="I145">
+        <v>1</v>
+      </c>
+      <c r="J145">
+        <v>1</v>
+      </c>
+      <c r="K145">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A146" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B145" s="4" t="s">
+      <c r="B146" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C145" t="s">
+      <c r="C146" t="s">
         <v>190</v>
       </c>
-      <c r="D145">
-        <v>1</v>
-      </c>
-      <c r="E145">
-        <v>1</v>
-      </c>
-      <c r="F145">
-        <v>0</v>
-      </c>
-      <c r="G145">
-        <v>0</v>
-      </c>
-      <c r="H145">
-        <v>0</v>
-      </c>
-      <c r="I145">
-        <v>0</v>
-      </c>
-      <c r="J145">
-        <v>0</v>
-      </c>
-      <c r="K145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A146" s="4"/>
-      <c r="B146" s="4"/>
-      <c r="C146" t="s">
-        <v>191</v>
-      </c>
       <c r="D146">
         <v>1</v>
       </c>
@@ -5612,13 +5619,13 @@
         <v>1</v>
       </c>
       <c r="F146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I146">
         <v>0</v>
@@ -5634,7 +5641,7 @@
       <c r="A147" s="4"/>
       <c r="B147" s="4"/>
       <c r="C147" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -5643,13 +5650,13 @@
         <v>1</v>
       </c>
       <c r="F147">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G147">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H147">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I147">
         <v>0</v>
@@ -5665,50 +5672,81 @@
       <c r="A148" s="4"/>
       <c r="B148" s="4"/>
       <c r="C148" t="s">
+        <v>192</v>
+      </c>
+      <c r="D148">
+        <v>1</v>
+      </c>
+      <c r="E148">
+        <v>1</v>
+      </c>
+      <c r="F148">
+        <v>0</v>
+      </c>
+      <c r="G148">
+        <v>0</v>
+      </c>
+      <c r="H148">
+        <v>0</v>
+      </c>
+      <c r="I148">
+        <v>0</v>
+      </c>
+      <c r="J148">
+        <v>0</v>
+      </c>
+      <c r="K148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A149" s="4"/>
+      <c r="B149" s="4"/>
+      <c r="C149" t="s">
         <v>193</v>
       </c>
-      <c r="D148">
-        <v>1</v>
-      </c>
-      <c r="E148">
-        <v>1</v>
-      </c>
-      <c r="F148">
-        <v>0</v>
-      </c>
-      <c r="G148">
-        <v>0</v>
-      </c>
-      <c r="H148">
-        <v>0</v>
-      </c>
-      <c r="I148">
-        <v>0</v>
-      </c>
-      <c r="J148">
-        <v>0</v>
-      </c>
-      <c r="K148">
+      <c r="D149">
+        <v>1</v>
+      </c>
+      <c r="E149">
+        <v>1</v>
+      </c>
+      <c r="F149">
+        <v>0</v>
+      </c>
+      <c r="G149">
+        <v>0</v>
+      </c>
+      <c r="H149">
+        <v>0</v>
+      </c>
+      <c r="I149">
+        <v>0</v>
+      </c>
+      <c r="J149">
+        <v>0</v>
+      </c>
+      <c r="K149">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="A145:A148"/>
-    <mergeCell ref="B145:B148"/>
-    <mergeCell ref="A102:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A131:A136"/>
-    <mergeCell ref="A137:A143"/>
-    <mergeCell ref="B102:B107"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B111:B115"/>
-    <mergeCell ref="B116:B122"/>
-    <mergeCell ref="B123:B127"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B136"/>
-    <mergeCell ref="B137:B141"/>
-    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="A102:A128"/>
+    <mergeCell ref="A129:A131"/>
+    <mergeCell ref="A132:A137"/>
+    <mergeCell ref="A138:A144"/>
+    <mergeCell ref="B102:B108"/>
+    <mergeCell ref="B109:B111"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="B117:B123"/>
+    <mergeCell ref="B124:B128"/>
+    <mergeCell ref="B129:B131"/>
+    <mergeCell ref="B132:B137"/>
+    <mergeCell ref="B138:B142"/>
+    <mergeCell ref="B143:B144"/>
     <mergeCell ref="A67:A86"/>
     <mergeCell ref="A87:A101"/>
     <mergeCell ref="B47:B51"/>
@@ -5735,7 +5773,8 @@
     <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added optimization:* perms (#336)
* Added optimization perms

* Conflict resolved
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17a9e6fd9bbdd953/Dokumenty/GitHub/Smart-University-Scheduler/helpers/db_seeder/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{79C568B3-4200-4E26-89A8-7C948583B1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B44B7B53-20BF-4B5B-9A1D-C19D5E316ABB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA7F6D3-A82B-490F-BBA9-B86E208CAE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="199">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -657,6 +657,18 @@
   </si>
   <si>
     <t>schedule:view_others</t>
+  </si>
+  <si>
+    <t>Optimization</t>
+  </si>
+  <si>
+    <t>optimization</t>
+  </si>
+  <si>
+    <t>optimization:run</t>
+  </si>
+  <si>
+    <t>optimization:view</t>
   </si>
 </sst>
 </file>
@@ -744,10 +756,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1013,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -5730,8 +5738,100 @@
         <v>0</v>
       </c>
     </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A150" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C150" t="s">
+        <v>197</v>
+      </c>
+      <c r="D150">
+        <v>1</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150">
+        <v>0</v>
+      </c>
+      <c r="G150">
+        <v>0</v>
+      </c>
+      <c r="H150">
+        <v>0</v>
+      </c>
+      <c r="I150">
+        <v>0</v>
+      </c>
+      <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A151" s="4"/>
+      <c r="B151" s="4"/>
+      <c r="C151" t="s">
+        <v>198</v>
+      </c>
+      <c r="D151">
+        <v>1</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151">
+        <v>0</v>
+      </c>
+      <c r="G151">
+        <v>0</v>
+      </c>
+      <c r="H151">
+        <v>0</v>
+      </c>
+      <c r="I151">
+        <v>0</v>
+      </c>
+      <c r="J151">
+        <v>0</v>
+      </c>
+      <c r="K151">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="41">
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="A87:A101"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B87:B91"/>
+    <mergeCell ref="B92:B96"/>
+    <mergeCell ref="B97:B101"/>
     <mergeCell ref="A146:A149"/>
     <mergeCell ref="B146:B149"/>
     <mergeCell ref="A102:A128"/>
@@ -5747,30 +5847,6 @@
     <mergeCell ref="B132:B137"/>
     <mergeCell ref="B138:B142"/>
     <mergeCell ref="B143:B144"/>
-    <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A101"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B87:B91"/>
-    <mergeCell ref="B92:B96"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5779,6 +5855,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5787,15 +5872,6 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5988,20 +6064,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update test database - excel file
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA7F6D3-A82B-490F-BBA9-B86E208CAE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AD8555-6173-43DC-8C46-77D4A074A5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="200">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -669,6 +669,9 @@
   </si>
   <si>
     <t>optimization:view</t>
+  </si>
+  <si>
+    <t>user-2fa:disable</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K151"/>
+  <dimension ref="A1:K152"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -3875,7 +3878,7 @@
       <c r="A91" s="4"/>
       <c r="B91" s="4"/>
       <c r="C91" t="s">
-        <v>119</v>
+        <v>199</v>
       </c>
       <c r="D91">
         <v>1</v>
@@ -3904,32 +3907,30 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A92" s="4"/>
-      <c r="B92" s="4" t="s">
-        <v>120</v>
-      </c>
+      <c r="B92" s="4"/>
       <c r="C92" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D92">
         <v>1</v>
       </c>
       <c r="E92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K92">
         <v>0</v>
@@ -3937,9 +3938,11 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93" s="4"/>
-      <c r="B93" s="4"/>
+      <c r="B93" s="4" t="s">
+        <v>120</v>
+      </c>
       <c r="C93" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D93">
         <v>1</v>
@@ -3970,7 +3973,7 @@
       <c r="A94" s="4"/>
       <c r="B94" s="4"/>
       <c r="C94" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D94">
         <v>1</v>
@@ -4001,7 +4004,7 @@
       <c r="A95" s="4"/>
       <c r="B95" s="4"/>
       <c r="C95" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -4032,7 +4035,7 @@
       <c r="A96" s="4"/>
       <c r="B96" s="4"/>
       <c r="C96" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D96">
         <v>1</v>
@@ -4061,11 +4064,9 @@
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="4"/>
-      <c r="B97" s="4" t="s">
-        <v>126</v>
-      </c>
+      <c r="B97" s="4"/>
       <c r="C97" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D97">
         <v>1</v>
@@ -4074,7 +4075,7 @@
         <v>0</v>
       </c>
       <c r="F97">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G97">
         <v>0</v>
@@ -4094,9 +4095,11 @@
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="4"/>
-      <c r="B98" s="4"/>
+      <c r="B98" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="C98" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D98">
         <v>1</v>
@@ -4127,7 +4130,7 @@
       <c r="A99" s="4"/>
       <c r="B99" s="4"/>
       <c r="C99" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D99">
         <v>1</v>
@@ -4158,7 +4161,7 @@
       <c r="A100" s="4"/>
       <c r="B100" s="4"/>
       <c r="C100" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D100">
         <v>1</v>
@@ -4189,74 +4192,74 @@
       <c r="A101" s="4"/>
       <c r="B101" s="4"/>
       <c r="C101" t="s">
+        <v>130</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>1</v>
+      </c>
+      <c r="G101">
+        <v>0</v>
+      </c>
+      <c r="H101">
+        <v>0</v>
+      </c>
+      <c r="I101">
+        <v>0</v>
+      </c>
+      <c r="J101">
+        <v>0</v>
+      </c>
+      <c r="K101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A102" s="4"/>
+      <c r="B102" s="4"/>
+      <c r="C102" t="s">
         <v>131</v>
       </c>
-      <c r="D101">
-        <v>1</v>
-      </c>
-      <c r="E101">
-        <v>0</v>
-      </c>
-      <c r="F101">
-        <v>1</v>
-      </c>
-      <c r="G101">
-        <v>0</v>
-      </c>
-      <c r="H101">
-        <v>0</v>
-      </c>
-      <c r="I101">
-        <v>0</v>
-      </c>
-      <c r="J101">
-        <v>0</v>
-      </c>
-      <c r="K101">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A102" s="4" t="s">
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>1</v>
+      </c>
+      <c r="G102">
+        <v>0</v>
+      </c>
+      <c r="H102">
+        <v>0</v>
+      </c>
+      <c r="I102">
+        <v>0</v>
+      </c>
+      <c r="J102">
+        <v>0</v>
+      </c>
+      <c r="K102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B103" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C102" s="2" t="s">
+      <c r="C103" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D102">
-        <v>1</v>
-      </c>
-      <c r="E102">
-        <v>1</v>
-      </c>
-      <c r="F102">
-        <v>1</v>
-      </c>
-      <c r="G102">
-        <v>0</v>
-      </c>
-      <c r="H102">
-        <v>0</v>
-      </c>
-      <c r="I102">
-        <v>0</v>
-      </c>
-      <c r="J102">
-        <v>0</v>
-      </c>
-      <c r="K102">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A103" s="4"/>
-      <c r="B103" s="4"/>
-      <c r="C103" s="2" t="s">
-        <v>135</v>
-      </c>
       <c r="D103">
         <v>1</v>
       </c>
@@ -4267,26 +4270,26 @@
         <v>1</v>
       </c>
       <c r="G103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K103">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104" s="4"/>
       <c r="B104" s="4"/>
       <c r="C104" s="2" t="s">
-        <v>194</v>
+        <v>135</v>
       </c>
       <c r="D104">
         <v>1</v>
@@ -4304,20 +4307,20 @@
         <v>1</v>
       </c>
       <c r="I104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K104">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="2" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="D105">
         <v>1</v>
@@ -4335,20 +4338,20 @@
         <v>1</v>
       </c>
       <c r="I105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K105">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D106">
         <v>1</v>
@@ -4360,26 +4363,26 @@
         <v>1</v>
       </c>
       <c r="G106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K106">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D107">
         <v>1</v>
@@ -4410,7 +4413,7 @@
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -4422,28 +4425,26 @@
         <v>1</v>
       </c>
       <c r="G108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K108">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="4"/>
-      <c r="B109" s="4" t="s">
-        <v>140</v>
-      </c>
+      <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D109">
         <v>1</v>
@@ -4472,15 +4473,17 @@
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
-      <c r="B110" s="4"/>
+      <c r="B110" s="4" t="s">
+        <v>140</v>
+      </c>
       <c r="C110" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D110">
         <v>1</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110">
         <v>1</v>
@@ -4489,23 +4492,23 @@
         <v>1</v>
       </c>
       <c r="H110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K110">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
       <c r="B111" s="4"/>
       <c r="C111" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D111">
         <v>1</v>
@@ -4534,17 +4537,15 @@
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
-      <c r="B112" s="4" t="s">
-        <v>144</v>
-      </c>
+      <c r="B112" s="4"/>
       <c r="C112" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D112">
         <v>1</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F112">
         <v>1</v>
@@ -4553,23 +4554,25 @@
         <v>1</v>
       </c>
       <c r="H112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K112">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
-      <c r="B113" s="4"/>
+      <c r="B113" s="4" t="s">
+        <v>144</v>
+      </c>
       <c r="C113" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -4600,7 +4603,7 @@
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D114">
         <v>1</v>
@@ -4612,26 +4615,26 @@
         <v>1</v>
       </c>
       <c r="G114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K114">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4662,7 +4665,7 @@
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4691,11 +4694,9 @@
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
-      <c r="B117" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4707,16 +4708,16 @@
         <v>1</v>
       </c>
       <c r="G117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K117">
         <v>0</v>
@@ -4724,9 +4725,11 @@
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A118" s="4"/>
-      <c r="B118" s="4"/>
+      <c r="B118" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="C118" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4757,7 +4760,7 @@
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4788,7 +4791,7 @@
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4800,16 +4803,16 @@
         <v>1</v>
       </c>
       <c r="G120">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H120">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I120">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J120">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K120">
         <v>0</v>
@@ -4819,7 +4822,7 @@
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4850,7 +4853,7 @@
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4881,7 +4884,7 @@
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4910,11 +4913,9 @@
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A124" s="4"/>
-      <c r="B124" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4926,16 +4927,16 @@
         <v>1</v>
       </c>
       <c r="G124">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H124">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I124">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J124">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K124">
         <v>0</v>
@@ -4943,9 +4944,11 @@
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A125" s="4"/>
-      <c r="B125" s="4"/>
+      <c r="B125" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="C125" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4976,13 +4979,13 @@
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D126">
         <v>1</v>
       </c>
       <c r="E126">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F126">
         <v>1</v>
@@ -4994,10 +4997,10 @@
         <v>1</v>
       </c>
       <c r="I126">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J126">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K126">
         <v>0</v>
@@ -5007,7 +5010,7 @@
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -5038,73 +5041,73 @@
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D128">
+        <v>1</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>1</v>
+      </c>
+      <c r="G128">
+        <v>1</v>
+      </c>
+      <c r="H128">
+        <v>1</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A129" s="4"/>
+      <c r="B129" s="4"/>
+      <c r="C129" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D128">
-        <v>1</v>
-      </c>
-      <c r="E128">
-        <v>0</v>
-      </c>
-      <c r="F128">
-        <v>1</v>
-      </c>
-      <c r="G128">
-        <v>0</v>
-      </c>
-      <c r="H128">
-        <v>0</v>
-      </c>
-      <c r="I128">
-        <v>0</v>
-      </c>
-      <c r="J128">
-        <v>0</v>
-      </c>
-      <c r="K128">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A129" s="4" t="s">
+      <c r="D129">
+        <v>1</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>1</v>
+      </c>
+      <c r="G129">
+        <v>0</v>
+      </c>
+      <c r="H129">
+        <v>0</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A130" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B129" s="4" t="s">
+      <c r="B130" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C129" t="s">
+      <c r="C130" t="s">
         <v>166</v>
-      </c>
-      <c r="D129">
-        <v>1</v>
-      </c>
-      <c r="E129">
-        <v>0</v>
-      </c>
-      <c r="F129">
-        <v>0</v>
-      </c>
-      <c r="G129">
-        <v>0</v>
-      </c>
-      <c r="H129">
-        <v>0</v>
-      </c>
-      <c r="I129">
-        <v>0</v>
-      </c>
-      <c r="J129">
-        <v>0</v>
-      </c>
-      <c r="K129">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A130" s="4"/>
-      <c r="B130" s="4"/>
-      <c r="C130" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -5135,73 +5138,73 @@
       <c r="A131" s="4"/>
       <c r="B131" s="4"/>
       <c r="C131" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+      <c r="F131">
+        <v>0</v>
+      </c>
+      <c r="G131">
+        <v>0</v>
+      </c>
+      <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A132" s="4"/>
+      <c r="B132" s="4"/>
+      <c r="C132" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D131">
-        <v>1</v>
-      </c>
-      <c r="E131">
-        <v>0</v>
-      </c>
-      <c r="F131">
-        <v>0</v>
-      </c>
-      <c r="G131">
-        <v>0</v>
-      </c>
-      <c r="H131">
-        <v>0</v>
-      </c>
-      <c r="I131">
-        <v>0</v>
-      </c>
-      <c r="J131">
-        <v>0</v>
-      </c>
-      <c r="K131">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A132" s="4" t="s">
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+      <c r="F132">
+        <v>0</v>
+      </c>
+      <c r="G132">
+        <v>0</v>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A133" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B132" s="4" t="s">
+      <c r="B133" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C132" t="s">
+      <c r="C133" t="s">
         <v>170</v>
-      </c>
-      <c r="D132">
-        <v>1</v>
-      </c>
-      <c r="E132">
-        <v>0</v>
-      </c>
-      <c r="F132">
-        <v>0</v>
-      </c>
-      <c r="G132">
-        <v>0</v>
-      </c>
-      <c r="H132">
-        <v>0</v>
-      </c>
-      <c r="I132">
-        <v>0</v>
-      </c>
-      <c r="J132">
-        <v>0</v>
-      </c>
-      <c r="K132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
-      <c r="C133" t="s">
-        <v>171</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -5232,7 +5235,7 @@
       <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -5263,7 +5266,7 @@
       <c r="A135" s="4"/>
       <c r="B135" s="4"/>
       <c r="C135" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -5294,7 +5297,7 @@
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
       <c r="C136" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -5325,91 +5328,91 @@
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" t="s">
+        <v>174</v>
+      </c>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>0</v>
+      </c>
+      <c r="F137">
+        <v>0</v>
+      </c>
+      <c r="G137">
+        <v>0</v>
+      </c>
+      <c r="H137">
+        <v>0</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="4"/>
+      <c r="B138" s="4"/>
+      <c r="C138" t="s">
         <v>175</v>
       </c>
-      <c r="D137">
-        <v>1</v>
-      </c>
-      <c r="E137">
-        <v>0</v>
-      </c>
-      <c r="F137">
-        <v>0</v>
-      </c>
-      <c r="G137">
-        <v>0</v>
-      </c>
-      <c r="H137">
-        <v>0</v>
-      </c>
-      <c r="I137">
-        <v>0</v>
-      </c>
-      <c r="J137">
-        <v>0</v>
-      </c>
-      <c r="K137">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A138" s="4" t="s">
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B138" s="4" t="s">
+      <c r="B139" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C139" t="s">
         <v>178</v>
       </c>
-      <c r="D138">
-        <v>1</v>
-      </c>
-      <c r="E138">
-        <v>1</v>
-      </c>
-      <c r="F138">
-        <v>1</v>
-      </c>
-      <c r="G138">
-        <v>1</v>
-      </c>
-      <c r="H138">
-        <v>1</v>
-      </c>
-      <c r="I138">
-        <v>1</v>
-      </c>
-      <c r="J138">
-        <v>0</v>
-      </c>
-      <c r="K138">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A139" s="4"/>
-      <c r="B139" s="4"/>
-      <c r="C139" t="s">
-        <v>179</v>
-      </c>
       <c r="D139">
         <v>1</v>
       </c>
       <c r="E139">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F139">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G139">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H139">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I139">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J139">
         <v>0</v>
@@ -5422,25 +5425,25 @@
       <c r="A140" s="4"/>
       <c r="B140" s="4"/>
       <c r="C140" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D140">
         <v>1</v>
       </c>
       <c r="E140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J140">
         <v>0</v>
@@ -5453,7 +5456,7 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -5484,7 +5487,7 @@
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -5513,11 +5516,9 @@
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" s="4"/>
-      <c r="B143" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B143" s="4"/>
       <c r="C143" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D143">
         <v>1</v>
@@ -5546,111 +5547,113 @@
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="4"/>
-      <c r="B144" s="4"/>
+      <c r="B144" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C144" t="s">
+        <v>184</v>
+      </c>
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
+        <v>1</v>
+      </c>
+      <c r="H144">
+        <v>1</v>
+      </c>
+      <c r="I144">
+        <v>1</v>
+      </c>
+      <c r="J144">
+        <v>0</v>
+      </c>
+      <c r="K144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="4"/>
+      <c r="B145" s="4"/>
+      <c r="C145" t="s">
         <v>185</v>
       </c>
-      <c r="D144">
-        <v>1</v>
-      </c>
-      <c r="E144">
-        <v>1</v>
-      </c>
-      <c r="F144">
-        <v>1</v>
-      </c>
-      <c r="G144">
-        <v>1</v>
-      </c>
-      <c r="H144">
-        <v>1</v>
-      </c>
-      <c r="I144">
-        <v>1</v>
-      </c>
-      <c r="J144">
-        <v>0</v>
-      </c>
-      <c r="K144">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A145" s="1" t="s">
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145">
+        <v>1</v>
+      </c>
+      <c r="G145">
+        <v>1</v>
+      </c>
+      <c r="H145">
+        <v>1</v>
+      </c>
+      <c r="I145">
+        <v>1</v>
+      </c>
+      <c r="J145">
+        <v>0</v>
+      </c>
+      <c r="K145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A146" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B145" s="1" t="s">
+      <c r="B146" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C145" t="s">
+      <c r="C146" t="s">
         <v>186</v>
       </c>
-      <c r="D145">
-        <v>1</v>
-      </c>
-      <c r="E145">
-        <v>1</v>
-      </c>
-      <c r="F145">
-        <v>1</v>
-      </c>
-      <c r="G145">
-        <v>1</v>
-      </c>
-      <c r="H145">
-        <v>1</v>
-      </c>
-      <c r="I145">
-        <v>1</v>
-      </c>
-      <c r="J145">
-        <v>1</v>
-      </c>
-      <c r="K145">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A146" s="4" t="s">
+      <c r="D146">
+        <v>1</v>
+      </c>
+      <c r="E146">
+        <v>1</v>
+      </c>
+      <c r="F146">
+        <v>1</v>
+      </c>
+      <c r="G146">
+        <v>1</v>
+      </c>
+      <c r="H146">
+        <v>1</v>
+      </c>
+      <c r="I146">
+        <v>1</v>
+      </c>
+      <c r="J146">
+        <v>1</v>
+      </c>
+      <c r="K146">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A147" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B146" s="4" t="s">
+      <c r="B147" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C146" t="s">
+      <c r="C147" t="s">
         <v>190</v>
       </c>
-      <c r="D146">
-        <v>1</v>
-      </c>
-      <c r="E146">
-        <v>1</v>
-      </c>
-      <c r="F146">
-        <v>0</v>
-      </c>
-      <c r="G146">
-        <v>0</v>
-      </c>
-      <c r="H146">
-        <v>0</v>
-      </c>
-      <c r="I146">
-        <v>0</v>
-      </c>
-      <c r="J146">
-        <v>0</v>
-      </c>
-      <c r="K146">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A147" s="4"/>
-      <c r="B147" s="4"/>
-      <c r="C147" t="s">
-        <v>191</v>
-      </c>
       <c r="D147">
         <v>1</v>
       </c>
@@ -5658,13 +5661,13 @@
         <v>1</v>
       </c>
       <c r="F147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I147">
         <v>0</v>
@@ -5680,7 +5683,7 @@
       <c r="A148" s="4"/>
       <c r="B148" s="4"/>
       <c r="C148" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -5689,13 +5692,13 @@
         <v>1</v>
       </c>
       <c r="F148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I148">
         <v>0</v>
@@ -5711,106 +5714,145 @@
       <c r="A149" s="4"/>
       <c r="B149" s="4"/>
       <c r="C149" t="s">
+        <v>192</v>
+      </c>
+      <c r="D149">
+        <v>1</v>
+      </c>
+      <c r="E149">
+        <v>1</v>
+      </c>
+      <c r="F149">
+        <v>0</v>
+      </c>
+      <c r="G149">
+        <v>0</v>
+      </c>
+      <c r="H149">
+        <v>0</v>
+      </c>
+      <c r="I149">
+        <v>0</v>
+      </c>
+      <c r="J149">
+        <v>0</v>
+      </c>
+      <c r="K149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A150" s="4"/>
+      <c r="B150" s="4"/>
+      <c r="C150" t="s">
         <v>193</v>
       </c>
-      <c r="D149">
-        <v>1</v>
-      </c>
-      <c r="E149">
-        <v>1</v>
-      </c>
-      <c r="F149">
-        <v>0</v>
-      </c>
-      <c r="G149">
-        <v>0</v>
-      </c>
-      <c r="H149">
-        <v>0</v>
-      </c>
-      <c r="I149">
-        <v>0</v>
-      </c>
-      <c r="J149">
-        <v>0</v>
-      </c>
-      <c r="K149">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A150" s="4" t="s">
+      <c r="D150">
+        <v>1</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150">
+        <v>0</v>
+      </c>
+      <c r="G150">
+        <v>0</v>
+      </c>
+      <c r="H150">
+        <v>0</v>
+      </c>
+      <c r="I150">
+        <v>0</v>
+      </c>
+      <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A151" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B150" s="4" t="s">
+      <c r="B151" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C150" t="s">
+      <c r="C151" t="s">
         <v>197</v>
       </c>
-      <c r="D150">
-        <v>1</v>
-      </c>
-      <c r="E150">
-        <v>1</v>
-      </c>
-      <c r="F150">
-        <v>0</v>
-      </c>
-      <c r="G150">
-        <v>0</v>
-      </c>
-      <c r="H150">
-        <v>0</v>
-      </c>
-      <c r="I150">
-        <v>0</v>
-      </c>
-      <c r="J150">
-        <v>0</v>
-      </c>
-      <c r="K150">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="4"/>
-      <c r="B151" s="4"/>
-      <c r="C151" t="s">
+      <c r="D151">
+        <v>1</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151">
+        <v>0</v>
+      </c>
+      <c r="G151">
+        <v>0</v>
+      </c>
+      <c r="H151">
+        <v>0</v>
+      </c>
+      <c r="I151">
+        <v>0</v>
+      </c>
+      <c r="J151">
+        <v>0</v>
+      </c>
+      <c r="K151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A152" s="4"/>
+      <c r="B152" s="4"/>
+      <c r="C152" t="s">
         <v>198</v>
       </c>
-      <c r="D151">
-        <v>1</v>
-      </c>
-      <c r="E151">
-        <v>1</v>
-      </c>
-      <c r="F151">
-        <v>0</v>
-      </c>
-      <c r="G151">
-        <v>0</v>
-      </c>
-      <c r="H151">
-        <v>0</v>
-      </c>
-      <c r="I151">
-        <v>0</v>
-      </c>
-      <c r="J151">
-        <v>0</v>
-      </c>
-      <c r="K151">
+      <c r="D152">
+        <v>1</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152">
+        <v>0</v>
+      </c>
+      <c r="G152">
+        <v>0</v>
+      </c>
+      <c r="H152">
+        <v>0</v>
+      </c>
+      <c r="I152">
+        <v>0</v>
+      </c>
+      <c r="J152">
+        <v>0</v>
+      </c>
+      <c r="K152">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A103:A129"/>
+    <mergeCell ref="A130:A132"/>
+    <mergeCell ref="A133:A138"/>
+    <mergeCell ref="A139:A145"/>
+    <mergeCell ref="B103:B109"/>
+    <mergeCell ref="B110:B112"/>
+    <mergeCell ref="B113:B117"/>
+    <mergeCell ref="B118:B124"/>
+    <mergeCell ref="B125:B129"/>
+    <mergeCell ref="B130:B132"/>
+    <mergeCell ref="B133:B138"/>
+    <mergeCell ref="B139:B143"/>
+    <mergeCell ref="B144:B145"/>
     <mergeCell ref="A2:A26"/>
     <mergeCell ref="A27:A66"/>
     <mergeCell ref="B2:B6"/>
@@ -5819,34 +5861,26 @@
     <mergeCell ref="B17:B21"/>
     <mergeCell ref="B22:B26"/>
     <mergeCell ref="B27:B31"/>
-    <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A101"/>
     <mergeCell ref="B47:B51"/>
     <mergeCell ref="B52:B56"/>
     <mergeCell ref="B57:B61"/>
     <mergeCell ref="B62:B66"/>
+    <mergeCell ref="A151:A152"/>
+    <mergeCell ref="B151:B152"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="A87:A102"/>
     <mergeCell ref="B67:B71"/>
     <mergeCell ref="B72:B76"/>
     <mergeCell ref="B77:B81"/>
     <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B87:B91"/>
-    <mergeCell ref="B92:B96"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="A102:A128"/>
-    <mergeCell ref="A129:A131"/>
-    <mergeCell ref="A132:A137"/>
-    <mergeCell ref="A138:A144"/>
-    <mergeCell ref="B102:B108"/>
-    <mergeCell ref="B109:B111"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="B117:B123"/>
-    <mergeCell ref="B124:B128"/>
-    <mergeCell ref="B129:B131"/>
-    <mergeCell ref="B132:B137"/>
-    <mergeCell ref="B138:B142"/>
-    <mergeCell ref="B143:B144"/>
+    <mergeCell ref="B87:B92"/>
+    <mergeCell ref="B93:B97"/>
+    <mergeCell ref="B98:B102"/>
+    <mergeCell ref="A147:A150"/>
+    <mergeCell ref="B147:B150"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5855,15 +5889,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5872,6 +5897,15 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6064,20 +6098,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Removed schedule-view for admin in excel file
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AD8555-6173-43DC-8C46-77D4A074A5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A5DD48-D00B-40E4-B9FF-0EA516942B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4354,7 +4354,7 @@
         <v>136</v>
       </c>
       <c r="D106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -5840,31 +5840,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="A103:A129"/>
-    <mergeCell ref="A130:A132"/>
-    <mergeCell ref="A133:A138"/>
-    <mergeCell ref="A139:A145"/>
-    <mergeCell ref="B103:B109"/>
-    <mergeCell ref="B110:B112"/>
-    <mergeCell ref="B113:B117"/>
-    <mergeCell ref="B118:B124"/>
-    <mergeCell ref="B125:B129"/>
-    <mergeCell ref="B130:B132"/>
-    <mergeCell ref="B133:B138"/>
-    <mergeCell ref="B139:B143"/>
-    <mergeCell ref="B144:B145"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
     <mergeCell ref="A151:A152"/>
     <mergeCell ref="B151:B152"/>
     <mergeCell ref="B32:B36"/>
@@ -5881,6 +5856,31 @@
     <mergeCell ref="B98:B102"/>
     <mergeCell ref="A147:A150"/>
     <mergeCell ref="B147:B150"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="A103:A129"/>
+    <mergeCell ref="A130:A132"/>
+    <mergeCell ref="A133:A138"/>
+    <mergeCell ref="A139:A145"/>
+    <mergeCell ref="B103:B109"/>
+    <mergeCell ref="B110:B112"/>
+    <mergeCell ref="B113:B117"/>
+    <mergeCell ref="B118:B124"/>
+    <mergeCell ref="B125:B129"/>
+    <mergeCell ref="B130:B132"/>
+    <mergeCell ref="B133:B138"/>
+    <mergeCell ref="B139:B143"/>
+    <mergeCell ref="B144:B145"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5889,6 +5889,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5897,15 +5906,6 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6098,20 +6098,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Admin has option to edit plan - endpoint (#371)
* Added schemas

* Added update_schedule_session endpoint

* Added schedule:update permission

* Changed error message

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>

* Added session validation

* Fixed TOCTOU

* Uncomment permission

* Refactor

* Refactor

* Uncomment permission

* Romoved applyOnce

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>

* Added todo in UpdateScheduleSessionRequest

* Standardized DayOfWeek enum

---------

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AD8555-6173-43DC-8C46-77D4A074A5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D53998-2A0D-42E9-AEB0-A6A4EE38304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="201">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -672,6 +672,9 @@
   </si>
   <si>
     <t>user-2fa:disable</t>
+  </si>
+  <si>
+    <t>schedule:update</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K152"/>
+  <dimension ref="A1:K153"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -4473,48 +4476,48 @@
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
-      <c r="B110" s="4" t="s">
-        <v>140</v>
-      </c>
+      <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
-        <v>141</v>
+        <v>200</v>
       </c>
       <c r="D110">
         <v>1</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K110">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
-      <c r="B111" s="4"/>
+      <c r="B111" s="4" t="s">
+        <v>140</v>
+      </c>
       <c r="C111" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F111">
         <v>1</v>
@@ -4523,23 +4526,23 @@
         <v>1</v>
       </c>
       <c r="H111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K111">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
       <c r="B112" s="4"/>
       <c r="C112" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D112">
         <v>1</v>
@@ -4568,17 +4571,15 @@
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
-      <c r="B113" s="4" t="s">
-        <v>144</v>
-      </c>
+      <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D113">
         <v>1</v>
       </c>
       <c r="E113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F113">
         <v>1</v>
@@ -4587,23 +4588,25 @@
         <v>1</v>
       </c>
       <c r="H113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K113">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
-      <c r="B114" s="4"/>
+      <c r="B114" s="4" t="s">
+        <v>144</v>
+      </c>
       <c r="C114" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D114">
         <v>1</v>
@@ -4634,7 +4637,7 @@
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4646,26 +4649,26 @@
         <v>1</v>
       </c>
       <c r="G115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K115">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4696,7 +4699,7 @@
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4725,11 +4728,9 @@
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A118" s="4"/>
-      <c r="B118" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4741,16 +4742,16 @@
         <v>1</v>
       </c>
       <c r="G118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K118">
         <v>0</v>
@@ -4758,9 +4759,11 @@
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
-      <c r="B119" s="4"/>
+      <c r="B119" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="C119" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4791,7 +4794,7 @@
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4822,7 +4825,7 @@
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4834,16 +4837,16 @@
         <v>1</v>
       </c>
       <c r="G121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K121">
         <v>0</v>
@@ -4853,7 +4856,7 @@
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4884,7 +4887,7 @@
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4915,7 +4918,7 @@
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4944,11 +4947,9 @@
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A125" s="4"/>
-      <c r="B125" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4960,16 +4961,16 @@
         <v>1</v>
       </c>
       <c r="G125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K125">
         <v>0</v>
@@ -4977,9 +4978,11 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126" s="4"/>
-      <c r="B126" s="4"/>
+      <c r="B126" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="C126" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -5010,13 +5013,13 @@
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D127">
         <v>1</v>
       </c>
       <c r="E127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F127">
         <v>1</v>
@@ -5028,10 +5031,10 @@
         <v>1</v>
       </c>
       <c r="I127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K127">
         <v>0</v>
@@ -5041,7 +5044,7 @@
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -5072,73 +5075,73 @@
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D129">
+        <v>1</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>1</v>
+      </c>
+      <c r="G129">
+        <v>1</v>
+      </c>
+      <c r="H129">
+        <v>1</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A130" s="4"/>
+      <c r="B130" s="4"/>
+      <c r="C130" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D129">
-        <v>1</v>
-      </c>
-      <c r="E129">
-        <v>0</v>
-      </c>
-      <c r="F129">
-        <v>1</v>
-      </c>
-      <c r="G129">
-        <v>0</v>
-      </c>
-      <c r="H129">
-        <v>0</v>
-      </c>
-      <c r="I129">
-        <v>0</v>
-      </c>
-      <c r="J129">
-        <v>0</v>
-      </c>
-      <c r="K129">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A130" s="4" t="s">
+      <c r="D130">
+        <v>1</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>1</v>
+      </c>
+      <c r="G130">
+        <v>0</v>
+      </c>
+      <c r="H130">
+        <v>0</v>
+      </c>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A131" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B130" s="4" t="s">
+      <c r="B131" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C130" t="s">
+      <c r="C131" t="s">
         <v>166</v>
-      </c>
-      <c r="D130">
-        <v>1</v>
-      </c>
-      <c r="E130">
-        <v>0</v>
-      </c>
-      <c r="F130">
-        <v>0</v>
-      </c>
-      <c r="G130">
-        <v>0</v>
-      </c>
-      <c r="H130">
-        <v>0</v>
-      </c>
-      <c r="I130">
-        <v>0</v>
-      </c>
-      <c r="J130">
-        <v>0</v>
-      </c>
-      <c r="K130">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A131" s="4"/>
-      <c r="B131" s="4"/>
-      <c r="C131" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -5169,73 +5172,73 @@
       <c r="A132" s="4"/>
       <c r="B132" s="4"/>
       <c r="C132" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+      <c r="F132">
+        <v>0</v>
+      </c>
+      <c r="G132">
+        <v>0</v>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A133" s="4"/>
+      <c r="B133" s="4"/>
+      <c r="C133" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D132">
-        <v>1</v>
-      </c>
-      <c r="E132">
-        <v>0</v>
-      </c>
-      <c r="F132">
-        <v>0</v>
-      </c>
-      <c r="G132">
-        <v>0</v>
-      </c>
-      <c r="H132">
-        <v>0</v>
-      </c>
-      <c r="I132">
-        <v>0</v>
-      </c>
-      <c r="J132">
-        <v>0</v>
-      </c>
-      <c r="K132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A133" s="4" t="s">
+      <c r="D133">
+        <v>1</v>
+      </c>
+      <c r="E133">
+        <v>0</v>
+      </c>
+      <c r="F133">
+        <v>0</v>
+      </c>
+      <c r="G133">
+        <v>0</v>
+      </c>
+      <c r="H133">
+        <v>0</v>
+      </c>
+      <c r="I133">
+        <v>0</v>
+      </c>
+      <c r="J133">
+        <v>0</v>
+      </c>
+      <c r="K133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A134" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B133" s="4" t="s">
+      <c r="B134" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C133" t="s">
+      <c r="C134" t="s">
         <v>170</v>
-      </c>
-      <c r="D133">
-        <v>1</v>
-      </c>
-      <c r="E133">
-        <v>0</v>
-      </c>
-      <c r="F133">
-        <v>0</v>
-      </c>
-      <c r="G133">
-        <v>0</v>
-      </c>
-      <c r="H133">
-        <v>0</v>
-      </c>
-      <c r="I133">
-        <v>0</v>
-      </c>
-      <c r="J133">
-        <v>0</v>
-      </c>
-      <c r="K133">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
-      <c r="C134" t="s">
-        <v>171</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -5266,7 +5269,7 @@
       <c r="A135" s="4"/>
       <c r="B135" s="4"/>
       <c r="C135" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -5297,7 +5300,7 @@
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
       <c r="C136" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -5328,7 +5331,7 @@
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -5359,91 +5362,91 @@
       <c r="A138" s="4"/>
       <c r="B138" s="4"/>
       <c r="C138" t="s">
+        <v>174</v>
+      </c>
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="4"/>
+      <c r="B139" s="4"/>
+      <c r="C139" t="s">
         <v>175</v>
       </c>
-      <c r="D138">
-        <v>1</v>
-      </c>
-      <c r="E138">
-        <v>0</v>
-      </c>
-      <c r="F138">
-        <v>0</v>
-      </c>
-      <c r="G138">
-        <v>0</v>
-      </c>
-      <c r="H138">
-        <v>0</v>
-      </c>
-      <c r="I138">
-        <v>0</v>
-      </c>
-      <c r="J138">
-        <v>0</v>
-      </c>
-      <c r="K138">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A139" s="4" t="s">
+      <c r="D139">
+        <v>1</v>
+      </c>
+      <c r="E139">
+        <v>0</v>
+      </c>
+      <c r="F139">
+        <v>0</v>
+      </c>
+      <c r="G139">
+        <v>0</v>
+      </c>
+      <c r="H139">
+        <v>0</v>
+      </c>
+      <c r="I139">
+        <v>0</v>
+      </c>
+      <c r="J139">
+        <v>0</v>
+      </c>
+      <c r="K139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A140" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B139" s="4" t="s">
+      <c r="B140" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C139" t="s">
+      <c r="C140" t="s">
         <v>178</v>
       </c>
-      <c r="D139">
-        <v>1</v>
-      </c>
-      <c r="E139">
-        <v>1</v>
-      </c>
-      <c r="F139">
-        <v>1</v>
-      </c>
-      <c r="G139">
-        <v>1</v>
-      </c>
-      <c r="H139">
-        <v>1</v>
-      </c>
-      <c r="I139">
-        <v>1</v>
-      </c>
-      <c r="J139">
-        <v>0</v>
-      </c>
-      <c r="K139">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A140" s="4"/>
-      <c r="B140" s="4"/>
-      <c r="C140" t="s">
-        <v>179</v>
-      </c>
       <c r="D140">
         <v>1</v>
       </c>
       <c r="E140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J140">
         <v>0</v>
@@ -5456,25 +5459,25 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D141">
         <v>1</v>
       </c>
       <c r="E141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J141">
         <v>0</v>
@@ -5487,7 +5490,7 @@
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -5518,7 +5521,7 @@
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D143">
         <v>1</v>
@@ -5547,11 +5550,9 @@
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="4"/>
-      <c r="B144" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B144" s="4"/>
       <c r="C144" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D144">
         <v>1</v>
@@ -5580,111 +5581,113 @@
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145" s="4"/>
-      <c r="B145" s="4"/>
+      <c r="B145" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C145" t="s">
+        <v>184</v>
+      </c>
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145">
+        <v>1</v>
+      </c>
+      <c r="G145">
+        <v>1</v>
+      </c>
+      <c r="H145">
+        <v>1</v>
+      </c>
+      <c r="I145">
+        <v>1</v>
+      </c>
+      <c r="J145">
+        <v>0</v>
+      </c>
+      <c r="K145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A146" s="4"/>
+      <c r="B146" s="4"/>
+      <c r="C146" t="s">
         <v>185</v>
       </c>
-      <c r="D145">
-        <v>1</v>
-      </c>
-      <c r="E145">
-        <v>1</v>
-      </c>
-      <c r="F145">
-        <v>1</v>
-      </c>
-      <c r="G145">
-        <v>1</v>
-      </c>
-      <c r="H145">
-        <v>1</v>
-      </c>
-      <c r="I145">
-        <v>1</v>
-      </c>
-      <c r="J145">
-        <v>0</v>
-      </c>
-      <c r="K145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A146" s="1" t="s">
+      <c r="D146">
+        <v>1</v>
+      </c>
+      <c r="E146">
+        <v>1</v>
+      </c>
+      <c r="F146">
+        <v>1</v>
+      </c>
+      <c r="G146">
+        <v>1</v>
+      </c>
+      <c r="H146">
+        <v>1</v>
+      </c>
+      <c r="I146">
+        <v>1</v>
+      </c>
+      <c r="J146">
+        <v>0</v>
+      </c>
+      <c r="K146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A147" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B146" s="1" t="s">
+      <c r="B147" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C146" t="s">
+      <c r="C147" t="s">
         <v>186</v>
       </c>
-      <c r="D146">
-        <v>1</v>
-      </c>
-      <c r="E146">
-        <v>1</v>
-      </c>
-      <c r="F146">
-        <v>1</v>
-      </c>
-      <c r="G146">
-        <v>1</v>
-      </c>
-      <c r="H146">
-        <v>1</v>
-      </c>
-      <c r="I146">
-        <v>1</v>
-      </c>
-      <c r="J146">
-        <v>1</v>
-      </c>
-      <c r="K146">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A147" s="4" t="s">
+      <c r="D147">
+        <v>1</v>
+      </c>
+      <c r="E147">
+        <v>1</v>
+      </c>
+      <c r="F147">
+        <v>1</v>
+      </c>
+      <c r="G147">
+        <v>1</v>
+      </c>
+      <c r="H147">
+        <v>1</v>
+      </c>
+      <c r="I147">
+        <v>1</v>
+      </c>
+      <c r="J147">
+        <v>1</v>
+      </c>
+      <c r="K147">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A148" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B147" s="4" t="s">
+      <c r="B148" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C147" t="s">
+      <c r="C148" t="s">
         <v>190</v>
       </c>
-      <c r="D147">
-        <v>1</v>
-      </c>
-      <c r="E147">
-        <v>1</v>
-      </c>
-      <c r="F147">
-        <v>0</v>
-      </c>
-      <c r="G147">
-        <v>0</v>
-      </c>
-      <c r="H147">
-        <v>0</v>
-      </c>
-      <c r="I147">
-        <v>0</v>
-      </c>
-      <c r="J147">
-        <v>0</v>
-      </c>
-      <c r="K147">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A148" s="4"/>
-      <c r="B148" s="4"/>
-      <c r="C148" t="s">
-        <v>191</v>
-      </c>
       <c r="D148">
         <v>1</v>
       </c>
@@ -5692,13 +5695,13 @@
         <v>1</v>
       </c>
       <c r="F148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I148">
         <v>0</v>
@@ -5714,7 +5717,7 @@
       <c r="A149" s="4"/>
       <c r="B149" s="4"/>
       <c r="C149" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -5723,13 +5726,13 @@
         <v>1</v>
       </c>
       <c r="F149">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G149">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H149">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I149">
         <v>0</v>
@@ -5745,114 +5748,148 @@
       <c r="A150" s="4"/>
       <c r="B150" s="4"/>
       <c r="C150" t="s">
+        <v>192</v>
+      </c>
+      <c r="D150">
+        <v>1</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150">
+        <v>0</v>
+      </c>
+      <c r="G150">
+        <v>0</v>
+      </c>
+      <c r="H150">
+        <v>0</v>
+      </c>
+      <c r="I150">
+        <v>0</v>
+      </c>
+      <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A151" s="4"/>
+      <c r="B151" s="4"/>
+      <c r="C151" t="s">
         <v>193</v>
       </c>
-      <c r="D150">
-        <v>1</v>
-      </c>
-      <c r="E150">
-        <v>1</v>
-      </c>
-      <c r="F150">
-        <v>0</v>
-      </c>
-      <c r="G150">
-        <v>0</v>
-      </c>
-      <c r="H150">
-        <v>0</v>
-      </c>
-      <c r="I150">
-        <v>0</v>
-      </c>
-      <c r="J150">
-        <v>0</v>
-      </c>
-      <c r="K150">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="4" t="s">
+      <c r="D151">
+        <v>1</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151">
+        <v>0</v>
+      </c>
+      <c r="G151">
+        <v>0</v>
+      </c>
+      <c r="H151">
+        <v>0</v>
+      </c>
+      <c r="I151">
+        <v>0</v>
+      </c>
+      <c r="J151">
+        <v>0</v>
+      </c>
+      <c r="K151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A152" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B151" s="4" t="s">
+      <c r="B152" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C151" t="s">
+      <c r="C152" t="s">
         <v>197</v>
       </c>
-      <c r="D151">
-        <v>1</v>
-      </c>
-      <c r="E151">
-        <v>1</v>
-      </c>
-      <c r="F151">
-        <v>0</v>
-      </c>
-      <c r="G151">
-        <v>0</v>
-      </c>
-      <c r="H151">
-        <v>0</v>
-      </c>
-      <c r="I151">
-        <v>0</v>
-      </c>
-      <c r="J151">
-        <v>0</v>
-      </c>
-      <c r="K151">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A152" s="4"/>
-      <c r="B152" s="4"/>
-      <c r="C152" t="s">
+      <c r="D152">
+        <v>1</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152">
+        <v>0</v>
+      </c>
+      <c r="G152">
+        <v>0</v>
+      </c>
+      <c r="H152">
+        <v>0</v>
+      </c>
+      <c r="I152">
+        <v>0</v>
+      </c>
+      <c r="J152">
+        <v>0</v>
+      </c>
+      <c r="K152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A153" s="4"/>
+      <c r="B153" s="4"/>
+      <c r="C153" t="s">
         <v>198</v>
       </c>
-      <c r="D152">
-        <v>1</v>
-      </c>
-      <c r="E152">
-        <v>1</v>
-      </c>
-      <c r="F152">
-        <v>0</v>
-      </c>
-      <c r="G152">
-        <v>0</v>
-      </c>
-      <c r="H152">
-        <v>0</v>
-      </c>
-      <c r="I152">
-        <v>0</v>
-      </c>
-      <c r="J152">
-        <v>0</v>
-      </c>
-      <c r="K152">
+      <c r="D153">
+        <v>1</v>
+      </c>
+      <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153">
+        <v>0</v>
+      </c>
+      <c r="G153">
+        <v>0</v>
+      </c>
+      <c r="H153">
+        <v>0</v>
+      </c>
+      <c r="I153">
+        <v>0</v>
+      </c>
+      <c r="J153">
+        <v>0</v>
+      </c>
+      <c r="K153">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="A103:A129"/>
-    <mergeCell ref="A130:A132"/>
-    <mergeCell ref="A133:A138"/>
-    <mergeCell ref="A139:A145"/>
-    <mergeCell ref="B103:B109"/>
-    <mergeCell ref="B110:B112"/>
-    <mergeCell ref="B113:B117"/>
-    <mergeCell ref="B118:B124"/>
-    <mergeCell ref="B125:B129"/>
-    <mergeCell ref="B130:B132"/>
-    <mergeCell ref="B133:B138"/>
-    <mergeCell ref="B139:B143"/>
-    <mergeCell ref="B144:B145"/>
+    <mergeCell ref="A152:A153"/>
+    <mergeCell ref="B152:B153"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="A87:A102"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B87:B92"/>
+    <mergeCell ref="B93:B97"/>
+    <mergeCell ref="B98:B102"/>
+    <mergeCell ref="A148:A151"/>
+    <mergeCell ref="B148:B151"/>
     <mergeCell ref="A2:A26"/>
     <mergeCell ref="A27:A66"/>
     <mergeCell ref="B2:B6"/>
@@ -5865,22 +5902,19 @@
     <mergeCell ref="B52:B56"/>
     <mergeCell ref="B57:B61"/>
     <mergeCell ref="B62:B66"/>
-    <mergeCell ref="A151:A152"/>
-    <mergeCell ref="B151:B152"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A102"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B87:B92"/>
-    <mergeCell ref="B93:B97"/>
-    <mergeCell ref="B98:B102"/>
-    <mergeCell ref="A147:A150"/>
-    <mergeCell ref="B147:B150"/>
+    <mergeCell ref="A103:A130"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="A134:A139"/>
+    <mergeCell ref="A140:A146"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B118"/>
+    <mergeCell ref="B119:B125"/>
+    <mergeCell ref="B126:B130"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="B134:B139"/>
+    <mergeCell ref="B140:B144"/>
+    <mergeCell ref="B145:B146"/>
+    <mergeCell ref="B103:B110"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5889,6 +5923,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
@@ -5897,15 +5940,6 @@
     <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6098,20 +6132,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
     <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add ability to add sessions that are not in the curriculum
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17a9e6fd9bbdd953/Dokumenty/GitHub/Smart-University-Scheduler/helpers/db_seeder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D53998-2A0D-42E9-AEB0-A6A4EE38304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{84D53998-2A0D-42E9-AEB0-A6A4EE38304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E613629-5ACB-401D-9DDF-CC5F953A7925}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="206">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -675,6 +675,21 @@
   </si>
   <si>
     <t>schedule:update</t>
+  </si>
+  <si>
+    <t>custom-events</t>
+  </si>
+  <si>
+    <t>custom-events:delete</t>
+  </si>
+  <si>
+    <t>custom-events:update</t>
+  </si>
+  <si>
+    <t>custom-events:view</t>
+  </si>
+  <si>
+    <t>custom-events:create</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K153"/>
+  <dimension ref="A1:K157"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -5134,23 +5149,21 @@
       </c>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A131" s="4" t="s">
-        <v>164</v>
-      </c>
+      <c r="A131" s="4"/>
       <c r="B131" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C131" t="s">
-        <v>166</v>
+        <v>201</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>205</v>
       </c>
       <c r="D131">
         <v>1</v>
       </c>
       <c r="E131">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G131">
         <v>0</v>
@@ -5171,29 +5184,29 @@
     <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
       <c r="B132" s="4"/>
-      <c r="C132" s="3" t="s">
-        <v>167</v>
+      <c r="C132" s="2" t="s">
+        <v>204</v>
       </c>
       <c r="D132">
         <v>1</v>
       </c>
       <c r="E132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K132">
         <v>0</v>
@@ -5202,17 +5215,17 @@
     <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
-      <c r="C133" s="3" t="s">
-        <v>187</v>
+      <c r="C133" s="2" t="s">
+        <v>203</v>
       </c>
       <c r="D133">
         <v>1</v>
       </c>
       <c r="E133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G133">
         <v>0</v>
@@ -5231,23 +5244,19 @@
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A134" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B134" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C134" t="s">
-        <v>170</v>
+      <c r="A134" s="4"/>
+      <c r="B134" s="4"/>
+      <c r="C134" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="D134">
         <v>1</v>
       </c>
       <c r="E134">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F134">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G134">
         <v>0</v>
@@ -5266,10 +5275,14 @@
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
+      <c r="A135" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>165</v>
+      </c>
       <c r="C135" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -5299,8 +5312,8 @@
     <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
-      <c r="C136" t="s">
-        <v>172</v>
+      <c r="C136" s="3" t="s">
+        <v>167</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -5330,8 +5343,8 @@
     <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
-      <c r="C137" t="s">
-        <v>173</v>
+      <c r="C137" s="3" t="s">
+        <v>187</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -5359,10 +5372,14 @@
       </c>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A138" s="4"/>
-      <c r="B138" s="4"/>
+      <c r="A138" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>169</v>
+      </c>
       <c r="C138" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D138">
         <v>1</v>
@@ -5393,7 +5410,7 @@
       <c r="A139" s="4"/>
       <c r="B139" s="4"/>
       <c r="C139" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -5421,32 +5438,28 @@
       </c>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A140" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="B140" s="4" t="s">
-        <v>177</v>
-      </c>
+      <c r="A140" s="4"/>
+      <c r="B140" s="4"/>
       <c r="C140" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D140">
         <v>1</v>
       </c>
       <c r="E140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J140">
         <v>0</v>
@@ -5459,7 +5472,7 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -5490,25 +5503,25 @@
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D142">
         <v>1</v>
       </c>
       <c r="E142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J142">
         <v>0</v>
@@ -5521,25 +5534,25 @@
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D143">
         <v>1</v>
       </c>
       <c r="E143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J143">
         <v>0</v>
@@ -5549,10 +5562,14 @@
       </c>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A144" s="4"/>
-      <c r="B144" s="4"/>
+      <c r="A144" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>177</v>
+      </c>
       <c r="C144" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D144">
         <v>1</v>
@@ -5581,29 +5598,27 @@
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145" s="4"/>
-      <c r="B145" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B145" s="4"/>
       <c r="C145" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D145">
         <v>1</v>
       </c>
       <c r="E145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J145">
         <v>0</v>
@@ -5616,7 +5631,7 @@
       <c r="A146" s="4"/>
       <c r="B146" s="4"/>
       <c r="C146" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -5644,14 +5659,10 @@
       </c>
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A147" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B147" s="1" t="s">
-        <v>114</v>
-      </c>
+      <c r="A147" s="4"/>
+      <c r="B147" s="4"/>
       <c r="C147" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -5672,21 +5683,17 @@
         <v>1</v>
       </c>
       <c r="J147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K147">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A148" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>189</v>
-      </c>
+      <c r="A148" s="4"/>
+      <c r="B148" s="4"/>
       <c r="C148" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -5695,16 +5702,16 @@
         <v>1</v>
       </c>
       <c r="F148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J148">
         <v>0</v>
@@ -5715,9 +5722,11 @@
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
-      <c r="B149" s="4"/>
+      <c r="B149" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C149" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -5735,7 +5744,7 @@
         <v>1</v>
       </c>
       <c r="I149">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J149">
         <v>0</v>
@@ -5748,7 +5757,7 @@
       <c r="A150" s="4"/>
       <c r="B150" s="4"/>
       <c r="C150" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D150">
         <v>1</v>
@@ -5757,16 +5766,16 @@
         <v>1</v>
       </c>
       <c r="F150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J150">
         <v>0</v>
@@ -5776,10 +5785,14 @@
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="4"/>
-      <c r="B151" s="4"/>
+      <c r="A151" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>114</v>
+      </c>
       <c r="C151" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D151">
         <v>1</v>
@@ -5788,33 +5801,33 @@
         <v>1</v>
       </c>
       <c r="F151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K151">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C152" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D152">
         <v>1</v>
@@ -5845,37 +5858,191 @@
       <c r="A153" s="4"/>
       <c r="B153" s="4"/>
       <c r="C153" t="s">
+        <v>191</v>
+      </c>
+      <c r="D153">
+        <v>1</v>
+      </c>
+      <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153">
+        <v>1</v>
+      </c>
+      <c r="G153">
+        <v>1</v>
+      </c>
+      <c r="H153">
+        <v>1</v>
+      </c>
+      <c r="I153">
+        <v>0</v>
+      </c>
+      <c r="J153">
+        <v>0</v>
+      </c>
+      <c r="K153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A154" s="4"/>
+      <c r="B154" s="4"/>
+      <c r="C154" t="s">
+        <v>192</v>
+      </c>
+      <c r="D154">
+        <v>1</v>
+      </c>
+      <c r="E154">
+        <v>1</v>
+      </c>
+      <c r="F154">
+        <v>0</v>
+      </c>
+      <c r="G154">
+        <v>0</v>
+      </c>
+      <c r="H154">
+        <v>0</v>
+      </c>
+      <c r="I154">
+        <v>0</v>
+      </c>
+      <c r="J154">
+        <v>0</v>
+      </c>
+      <c r="K154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A155" s="4"/>
+      <c r="B155" s="4"/>
+      <c r="C155" t="s">
+        <v>193</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155">
+        <v>0</v>
+      </c>
+      <c r="I155">
+        <v>0</v>
+      </c>
+      <c r="J155">
+        <v>0</v>
+      </c>
+      <c r="K155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A156" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C156" t="s">
+        <v>197</v>
+      </c>
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+      <c r="F156">
+        <v>0</v>
+      </c>
+      <c r="G156">
+        <v>0</v>
+      </c>
+      <c r="H156">
+        <v>0</v>
+      </c>
+      <c r="I156">
+        <v>0</v>
+      </c>
+      <c r="J156">
+        <v>0</v>
+      </c>
+      <c r="K156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A157" s="4"/>
+      <c r="B157" s="4"/>
+      <c r="C157" t="s">
         <v>198</v>
       </c>
-      <c r="D153">
-        <v>1</v>
-      </c>
-      <c r="E153">
-        <v>1</v>
-      </c>
-      <c r="F153">
-        <v>0</v>
-      </c>
-      <c r="G153">
-        <v>0</v>
-      </c>
-      <c r="H153">
-        <v>0</v>
-      </c>
-      <c r="I153">
-        <v>0</v>
-      </c>
-      <c r="J153">
-        <v>0</v>
-      </c>
-      <c r="K153">
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157">
+        <v>0</v>
+      </c>
+      <c r="G157">
+        <v>0</v>
+      </c>
+      <c r="H157">
+        <v>0</v>
+      </c>
+      <c r="I157">
+        <v>0</v>
+      </c>
+      <c r="J157">
+        <v>0</v>
+      </c>
+      <c r="K157">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="A152:A153"/>
-    <mergeCell ref="B152:B153"/>
+  <mergeCells count="42">
+    <mergeCell ref="B131:B134"/>
+    <mergeCell ref="A135:A137"/>
+    <mergeCell ref="A138:A143"/>
+    <mergeCell ref="A144:A150"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B118"/>
+    <mergeCell ref="B119:B125"/>
+    <mergeCell ref="B126:B130"/>
+    <mergeCell ref="B135:B137"/>
+    <mergeCell ref="B138:B143"/>
+    <mergeCell ref="B144:B148"/>
+    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="B103:B110"/>
+    <mergeCell ref="A103:A134"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="A156:A157"/>
+    <mergeCell ref="B156:B157"/>
     <mergeCell ref="B32:B36"/>
     <mergeCell ref="B37:B41"/>
     <mergeCell ref="B42:B46"/>
@@ -5888,33 +6055,8 @@
     <mergeCell ref="B87:B92"/>
     <mergeCell ref="B93:B97"/>
     <mergeCell ref="B98:B102"/>
-    <mergeCell ref="A148:A151"/>
-    <mergeCell ref="B148:B151"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="A103:A130"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A139"/>
-    <mergeCell ref="A140:A146"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B118"/>
-    <mergeCell ref="B119:B125"/>
-    <mergeCell ref="B126:B130"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B134:B139"/>
-    <mergeCell ref="B140:B144"/>
-    <mergeCell ref="B145:B146"/>
-    <mergeCell ref="B103:B110"/>
+    <mergeCell ref="A152:A155"/>
+    <mergeCell ref="B152:B155"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5923,26 +6065,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EC4E686503E2F943B8E5E5655A7FD1F0" ma:contentTypeVersion="10" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="f2732ee9c33e97baf8920e24934e29c2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36e2ff40-ab52-4240-babf-7476b65fdfdc" xmlns:ns3="d3830623-0ee5-4634-96e5-1fabe66116f4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2a88aeb4517fc5801f374367f5cb1408" ns2:_="" ns3:_="">
     <xsd:import namespace="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
@@ -6131,10 +6253,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90CF6C77-55D4-44ED-8F28-2A0B0624A3F2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
+    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6151,20 +6304,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90CF6C77-55D4-44ED-8F28-2A0B0624A3F2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
-    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add ability to add sessions that are not in the curriculum (#395)
* Add ability to add sessions that are not in the curriculum

* Create 688d899652d6_add_custom_events_table.py

* Black reformat

* Fix user_id

* Fetch schedule entries for each week spanned by the event before computing overlaps

* Disable broad access to potentially private events

* Returning 404 for non-owners unless the caller is privileged

* Update router.py

* Renaming the path param to custom_event_id

* Black

* Delete import

* Fix cyclomatic complexity

* Black

* Change to neo4j

* Fix codacy

* Delete 688d899652d6_add_custom_events_table.py
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wojko\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17a9e6fd9bbdd953/Dokumenty/GitHub/Smart-University-Scheduler/helpers/db_seeder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D53998-2A0D-42E9-AEB0-A6A4EE38304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{84D53998-2A0D-42E9-AEB0-A6A4EE38304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E613629-5ACB-401D-9DDF-CC5F953A7925}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="206">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -675,6 +675,21 @@
   </si>
   <si>
     <t>schedule:update</t>
+  </si>
+  <si>
+    <t>custom-events</t>
+  </si>
+  <si>
+    <t>custom-events:delete</t>
+  </si>
+  <si>
+    <t>custom-events:update</t>
+  </si>
+  <si>
+    <t>custom-events:view</t>
+  </si>
+  <si>
+    <t>custom-events:create</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K153"/>
+  <dimension ref="A1:K157"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -5134,23 +5149,21 @@
       </c>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A131" s="4" t="s">
-        <v>164</v>
-      </c>
+      <c r="A131" s="4"/>
       <c r="B131" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C131" t="s">
-        <v>166</v>
+        <v>201</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>205</v>
       </c>
       <c r="D131">
         <v>1</v>
       </c>
       <c r="E131">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G131">
         <v>0</v>
@@ -5171,29 +5184,29 @@
     <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
       <c r="B132" s="4"/>
-      <c r="C132" s="3" t="s">
-        <v>167</v>
+      <c r="C132" s="2" t="s">
+        <v>204</v>
       </c>
       <c r="D132">
         <v>1</v>
       </c>
       <c r="E132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K132">
         <v>0</v>
@@ -5202,17 +5215,17 @@
     <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
-      <c r="C133" s="3" t="s">
-        <v>187</v>
+      <c r="C133" s="2" t="s">
+        <v>203</v>
       </c>
       <c r="D133">
         <v>1</v>
       </c>
       <c r="E133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G133">
         <v>0</v>
@@ -5231,23 +5244,19 @@
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A134" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B134" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C134" t="s">
-        <v>170</v>
+      <c r="A134" s="4"/>
+      <c r="B134" s="4"/>
+      <c r="C134" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="D134">
         <v>1</v>
       </c>
       <c r="E134">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F134">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G134">
         <v>0</v>
@@ -5266,10 +5275,14 @@
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
+      <c r="A135" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>165</v>
+      </c>
       <c r="C135" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -5299,8 +5312,8 @@
     <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
-      <c r="C136" t="s">
-        <v>172</v>
+      <c r="C136" s="3" t="s">
+        <v>167</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -5330,8 +5343,8 @@
     <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
-      <c r="C137" t="s">
-        <v>173</v>
+      <c r="C137" s="3" t="s">
+        <v>187</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -5359,10 +5372,14 @@
       </c>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A138" s="4"/>
-      <c r="B138" s="4"/>
+      <c r="A138" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>169</v>
+      </c>
       <c r="C138" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D138">
         <v>1</v>
@@ -5393,7 +5410,7 @@
       <c r="A139" s="4"/>
       <c r="B139" s="4"/>
       <c r="C139" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -5421,32 +5438,28 @@
       </c>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A140" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="B140" s="4" t="s">
-        <v>177</v>
-      </c>
+      <c r="A140" s="4"/>
+      <c r="B140" s="4"/>
       <c r="C140" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D140">
         <v>1</v>
       </c>
       <c r="E140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J140">
         <v>0</v>
@@ -5459,7 +5472,7 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -5490,25 +5503,25 @@
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D142">
         <v>1</v>
       </c>
       <c r="E142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J142">
         <v>0</v>
@@ -5521,25 +5534,25 @@
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D143">
         <v>1</v>
       </c>
       <c r="E143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J143">
         <v>0</v>
@@ -5549,10 +5562,14 @@
       </c>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A144" s="4"/>
-      <c r="B144" s="4"/>
+      <c r="A144" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>177</v>
+      </c>
       <c r="C144" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D144">
         <v>1</v>
@@ -5581,29 +5598,27 @@
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145" s="4"/>
-      <c r="B145" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B145" s="4"/>
       <c r="C145" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D145">
         <v>1</v>
       </c>
       <c r="E145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J145">
         <v>0</v>
@@ -5616,7 +5631,7 @@
       <c r="A146" s="4"/>
       <c r="B146" s="4"/>
       <c r="C146" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -5644,14 +5659,10 @@
       </c>
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A147" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B147" s="1" t="s">
-        <v>114</v>
-      </c>
+      <c r="A147" s="4"/>
+      <c r="B147" s="4"/>
       <c r="C147" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -5672,21 +5683,17 @@
         <v>1</v>
       </c>
       <c r="J147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K147">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A148" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>189</v>
-      </c>
+      <c r="A148" s="4"/>
+      <c r="B148" s="4"/>
       <c r="C148" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -5695,16 +5702,16 @@
         <v>1</v>
       </c>
       <c r="F148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J148">
         <v>0</v>
@@ -5715,9 +5722,11 @@
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
-      <c r="B149" s="4"/>
+      <c r="B149" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C149" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -5735,7 +5744,7 @@
         <v>1</v>
       </c>
       <c r="I149">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J149">
         <v>0</v>
@@ -5748,7 +5757,7 @@
       <c r="A150" s="4"/>
       <c r="B150" s="4"/>
       <c r="C150" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D150">
         <v>1</v>
@@ -5757,16 +5766,16 @@
         <v>1</v>
       </c>
       <c r="F150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J150">
         <v>0</v>
@@ -5776,10 +5785,14 @@
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="4"/>
-      <c r="B151" s="4"/>
+      <c r="A151" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>114</v>
+      </c>
       <c r="C151" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D151">
         <v>1</v>
@@ -5788,33 +5801,33 @@
         <v>1</v>
       </c>
       <c r="F151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K151">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C152" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D152">
         <v>1</v>
@@ -5845,37 +5858,191 @@
       <c r="A153" s="4"/>
       <c r="B153" s="4"/>
       <c r="C153" t="s">
+        <v>191</v>
+      </c>
+      <c r="D153">
+        <v>1</v>
+      </c>
+      <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153">
+        <v>1</v>
+      </c>
+      <c r="G153">
+        <v>1</v>
+      </c>
+      <c r="H153">
+        <v>1</v>
+      </c>
+      <c r="I153">
+        <v>0</v>
+      </c>
+      <c r="J153">
+        <v>0</v>
+      </c>
+      <c r="K153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A154" s="4"/>
+      <c r="B154" s="4"/>
+      <c r="C154" t="s">
+        <v>192</v>
+      </c>
+      <c r="D154">
+        <v>1</v>
+      </c>
+      <c r="E154">
+        <v>1</v>
+      </c>
+      <c r="F154">
+        <v>0</v>
+      </c>
+      <c r="G154">
+        <v>0</v>
+      </c>
+      <c r="H154">
+        <v>0</v>
+      </c>
+      <c r="I154">
+        <v>0</v>
+      </c>
+      <c r="J154">
+        <v>0</v>
+      </c>
+      <c r="K154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A155" s="4"/>
+      <c r="B155" s="4"/>
+      <c r="C155" t="s">
+        <v>193</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155">
+        <v>0</v>
+      </c>
+      <c r="I155">
+        <v>0</v>
+      </c>
+      <c r="J155">
+        <v>0</v>
+      </c>
+      <c r="K155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A156" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C156" t="s">
+        <v>197</v>
+      </c>
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+      <c r="F156">
+        <v>0</v>
+      </c>
+      <c r="G156">
+        <v>0</v>
+      </c>
+      <c r="H156">
+        <v>0</v>
+      </c>
+      <c r="I156">
+        <v>0</v>
+      </c>
+      <c r="J156">
+        <v>0</v>
+      </c>
+      <c r="K156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A157" s="4"/>
+      <c r="B157" s="4"/>
+      <c r="C157" t="s">
         <v>198</v>
       </c>
-      <c r="D153">
-        <v>1</v>
-      </c>
-      <c r="E153">
-        <v>1</v>
-      </c>
-      <c r="F153">
-        <v>0</v>
-      </c>
-      <c r="G153">
-        <v>0</v>
-      </c>
-      <c r="H153">
-        <v>0</v>
-      </c>
-      <c r="I153">
-        <v>0</v>
-      </c>
-      <c r="J153">
-        <v>0</v>
-      </c>
-      <c r="K153">
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157">
+        <v>0</v>
+      </c>
+      <c r="G157">
+        <v>0</v>
+      </c>
+      <c r="H157">
+        <v>0</v>
+      </c>
+      <c r="I157">
+        <v>0</v>
+      </c>
+      <c r="J157">
+        <v>0</v>
+      </c>
+      <c r="K157">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="A152:A153"/>
-    <mergeCell ref="B152:B153"/>
+  <mergeCells count="42">
+    <mergeCell ref="B131:B134"/>
+    <mergeCell ref="A135:A137"/>
+    <mergeCell ref="A138:A143"/>
+    <mergeCell ref="A144:A150"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B118"/>
+    <mergeCell ref="B119:B125"/>
+    <mergeCell ref="B126:B130"/>
+    <mergeCell ref="B135:B137"/>
+    <mergeCell ref="B138:B143"/>
+    <mergeCell ref="B144:B148"/>
+    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="B103:B110"/>
+    <mergeCell ref="A103:A134"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="A156:A157"/>
+    <mergeCell ref="B156:B157"/>
     <mergeCell ref="B32:B36"/>
     <mergeCell ref="B37:B41"/>
     <mergeCell ref="B42:B46"/>
@@ -5888,33 +6055,8 @@
     <mergeCell ref="B87:B92"/>
     <mergeCell ref="B93:B97"/>
     <mergeCell ref="B98:B102"/>
-    <mergeCell ref="A148:A151"/>
-    <mergeCell ref="B148:B151"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="A103:A130"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A139"/>
-    <mergeCell ref="A140:A146"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B118"/>
-    <mergeCell ref="B119:B125"/>
-    <mergeCell ref="B126:B130"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B134:B139"/>
-    <mergeCell ref="B140:B144"/>
-    <mergeCell ref="B145:B146"/>
-    <mergeCell ref="B103:B110"/>
+    <mergeCell ref="A152:A155"/>
+    <mergeCell ref="B152:B155"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5923,26 +6065,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EC4E686503E2F943B8E5E5655A7FD1F0" ma:contentTypeVersion="10" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="f2732ee9c33e97baf8920e24934e29c2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36e2ff40-ab52-4240-babf-7476b65fdfdc" xmlns:ns3="d3830623-0ee5-4634-96e5-1fabe66116f4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2a88aeb4517fc5801f374367f5cb1408" ns2:_="" ns3:_="">
     <xsd:import namespace="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
@@ -6131,10 +6253,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90CF6C77-55D4-44ED-8F28-2A0B0624A3F2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
+    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6151,20 +6304,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90CF6C77-55D4-44ED-8F28-2A0B0624A3F2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
-    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add basic public api UI
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\kompetencyjny\Smart-University-Scheduler\helpers\db_seeder\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Smart-University-Scheduler\helpers\db_seeder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F317874-4BC0-4E7B-B789-C2FB1D819C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8ED8031-B46D-49E0-B168-972FBA6C8EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="208">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -690,6 +690,12 @@
   </si>
   <si>
     <t>custom-events:create</t>
+  </si>
+  <si>
+    <t>api key</t>
+  </si>
+  <si>
+    <t>api-key:generate</t>
   </si>
 </sst>
 </file>
@@ -1042,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K157"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -4269,46 +4275,48 @@
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A103" s="4" t="s">
+      <c r="A103" s="4"/>
+      <c r="B103" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C103" t="s">
+        <v>207</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>0</v>
+      </c>
+      <c r="G103">
+        <v>0</v>
+      </c>
+      <c r="H103">
+        <v>0</v>
+      </c>
+      <c r="I103">
+        <v>0</v>
+      </c>
+      <c r="J103">
+        <v>0</v>
+      </c>
+      <c r="K103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B104" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C103" s="2" t="s">
+      <c r="C104" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D103">
-        <v>1</v>
-      </c>
-      <c r="E103">
-        <v>1</v>
-      </c>
-      <c r="F103">
-        <v>1</v>
-      </c>
-      <c r="G103">
-        <v>0</v>
-      </c>
-      <c r="H103">
-        <v>0</v>
-      </c>
-      <c r="I103">
-        <v>0</v>
-      </c>
-      <c r="J103">
-        <v>0</v>
-      </c>
-      <c r="K103">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A104" s="4"/>
-      <c r="B104" s="4"/>
-      <c r="C104" s="2" t="s">
-        <v>135</v>
-      </c>
       <c r="D104">
         <v>1</v>
       </c>
@@ -4319,26 +4327,26 @@
         <v>1</v>
       </c>
       <c r="G104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K104">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="2" t="s">
-        <v>194</v>
+        <v>135</v>
       </c>
       <c r="D105">
         <v>1</v>
@@ -4356,20 +4364,20 @@
         <v>1</v>
       </c>
       <c r="I105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K105">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="D106">
         <v>1</v>
@@ -4387,20 +4395,20 @@
         <v>1</v>
       </c>
       <c r="I106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K106">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D107">
         <v>1</v>
@@ -4412,26 +4420,26 @@
         <v>1</v>
       </c>
       <c r="G107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K107">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -4462,7 +4470,7 @@
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D109">
         <v>1</v>
@@ -4474,96 +4482,96 @@
         <v>1</v>
       </c>
       <c r="G109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K109">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
-        <v>200</v>
+        <v>139</v>
       </c>
       <c r="D110">
         <v>1</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K110">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
-      <c r="B111" s="4" t="s">
-        <v>140</v>
-      </c>
+      <c r="B111" s="4"/>
       <c r="C111" s="2" t="s">
-        <v>141</v>
+        <v>200</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K111">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
-      <c r="B112" s="4"/>
+      <c r="B112" s="4" t="s">
+        <v>140</v>
+      </c>
       <c r="C112" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D112">
         <v>1</v>
       </c>
       <c r="E112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F112">
         <v>1</v>
@@ -4572,23 +4580,23 @@
         <v>1</v>
       </c>
       <c r="H112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K112">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -4617,17 +4625,15 @@
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
-      <c r="B114" s="4" t="s">
-        <v>144</v>
-      </c>
+      <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D114">
         <v>1</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F114">
         <v>1</v>
@@ -4636,23 +4642,25 @@
         <v>1</v>
       </c>
       <c r="H114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K114">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A115" s="4"/>
-      <c r="B115" s="4"/>
+      <c r="B115" s="4" t="s">
+        <v>144</v>
+      </c>
       <c r="C115" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4683,7 +4691,7 @@
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4695,26 +4703,26 @@
         <v>1</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K116">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4745,7 +4753,7 @@
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4774,11 +4782,9 @@
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
-      <c r="B119" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4790,16 +4796,16 @@
         <v>1</v>
       </c>
       <c r="G119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K119">
         <v>0</v>
@@ -4807,9 +4813,11 @@
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120" s="4"/>
-      <c r="B120" s="4"/>
+      <c r="B120" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="C120" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4840,7 +4848,7 @@
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4871,7 +4879,7 @@
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4883,16 +4891,16 @@
         <v>1</v>
       </c>
       <c r="G122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K122">
         <v>0</v>
@@ -4902,7 +4910,7 @@
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4933,7 +4941,7 @@
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4964,7 +4972,7 @@
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4993,11 +5001,9 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126" s="4"/>
-      <c r="B126" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -5009,16 +5015,16 @@
         <v>1</v>
       </c>
       <c r="G126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K126">
         <v>0</v>
@@ -5026,9 +5032,11 @@
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A127" s="4"/>
-      <c r="B127" s="4"/>
+      <c r="B127" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="C127" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -5059,13 +5067,13 @@
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D128">
         <v>1</v>
       </c>
       <c r="E128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F128">
         <v>1</v>
@@ -5077,10 +5085,10 @@
         <v>1</v>
       </c>
       <c r="I128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K128">
         <v>0</v>
@@ -5090,7 +5098,7 @@
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -5121,7 +5129,7 @@
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -5133,10 +5141,10 @@
         <v>1</v>
       </c>
       <c r="G130">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H130">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I130">
         <v>0</v>
@@ -5150,17 +5158,15 @@
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" s="4"/>
-      <c r="B131" s="4" t="s">
-        <v>201</v>
-      </c>
+      <c r="B131" s="4"/>
       <c r="C131" s="2" t="s">
-        <v>205</v>
+        <v>163</v>
       </c>
       <c r="D131">
         <v>1</v>
       </c>
       <c r="E131">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F131">
         <v>1</v>
@@ -5183,9 +5189,11 @@
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
+      <c r="B132" s="4" t="s">
+        <v>201</v>
+      </c>
       <c r="C132" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -5197,16 +5205,16 @@
         <v>1</v>
       </c>
       <c r="G132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K132">
         <v>0</v>
@@ -5216,7 +5224,7 @@
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -5228,16 +5236,16 @@
         <v>1</v>
       </c>
       <c r="G133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K133">
         <v>0</v>
@@ -5247,73 +5255,73 @@
       <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134">
+        <v>1</v>
+      </c>
+      <c r="F134">
+        <v>1</v>
+      </c>
+      <c r="G134">
+        <v>0</v>
+      </c>
+      <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+      <c r="J134">
+        <v>0</v>
+      </c>
+      <c r="K134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A135" s="4"/>
+      <c r="B135" s="4"/>
+      <c r="C135" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D134">
-        <v>1</v>
-      </c>
-      <c r="E134">
-        <v>1</v>
-      </c>
-      <c r="F134">
-        <v>1</v>
-      </c>
-      <c r="G134">
-        <v>0</v>
-      </c>
-      <c r="H134">
-        <v>0</v>
-      </c>
-      <c r="I134">
-        <v>0</v>
-      </c>
-      <c r="J134">
-        <v>0</v>
-      </c>
-      <c r="K134">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A135" s="4" t="s">
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135">
+        <v>1</v>
+      </c>
+      <c r="F135">
+        <v>1</v>
+      </c>
+      <c r="G135">
+        <v>0</v>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A136" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B135" s="4" t="s">
+      <c r="B136" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C135" t="s">
+      <c r="C136" t="s">
         <v>166</v>
-      </c>
-      <c r="D135">
-        <v>1</v>
-      </c>
-      <c r="E135">
-        <v>0</v>
-      </c>
-      <c r="F135">
-        <v>0</v>
-      </c>
-      <c r="G135">
-        <v>0</v>
-      </c>
-      <c r="H135">
-        <v>0</v>
-      </c>
-      <c r="I135">
-        <v>0</v>
-      </c>
-      <c r="J135">
-        <v>0</v>
-      </c>
-      <c r="K135">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
-      <c r="C136" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -5344,73 +5352,73 @@
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>0</v>
+      </c>
+      <c r="F137">
+        <v>0</v>
+      </c>
+      <c r="G137">
+        <v>0</v>
+      </c>
+      <c r="H137">
+        <v>0</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="4"/>
+      <c r="B138" s="4"/>
+      <c r="C138" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D137">
-        <v>1</v>
-      </c>
-      <c r="E137">
-        <v>0</v>
-      </c>
-      <c r="F137">
-        <v>0</v>
-      </c>
-      <c r="G137">
-        <v>0</v>
-      </c>
-      <c r="H137">
-        <v>0</v>
-      </c>
-      <c r="I137">
-        <v>0</v>
-      </c>
-      <c r="J137">
-        <v>0</v>
-      </c>
-      <c r="K137">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A138" s="4" t="s">
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B138" s="4" t="s">
+      <c r="B139" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C139" t="s">
         <v>170</v>
-      </c>
-      <c r="D138">
-        <v>1</v>
-      </c>
-      <c r="E138">
-        <v>0</v>
-      </c>
-      <c r="F138">
-        <v>0</v>
-      </c>
-      <c r="G138">
-        <v>0</v>
-      </c>
-      <c r="H138">
-        <v>0</v>
-      </c>
-      <c r="I138">
-        <v>0</v>
-      </c>
-      <c r="J138">
-        <v>0</v>
-      </c>
-      <c r="K138">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A139" s="4"/>
-      <c r="B139" s="4"/>
-      <c r="C139" t="s">
-        <v>171</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -5441,7 +5449,7 @@
       <c r="A140" s="4"/>
       <c r="B140" s="4"/>
       <c r="C140" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D140">
         <v>1</v>
@@ -5472,7 +5480,7 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -5503,7 +5511,7 @@
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -5534,73 +5542,73 @@
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" t="s">
+        <v>174</v>
+      </c>
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>0</v>
+      </c>
+      <c r="F143">
+        <v>0</v>
+      </c>
+      <c r="G143">
+        <v>0</v>
+      </c>
+      <c r="H143">
+        <v>0</v>
+      </c>
+      <c r="I143">
+        <v>0</v>
+      </c>
+      <c r="J143">
+        <v>0</v>
+      </c>
+      <c r="K143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A144" s="4"/>
+      <c r="B144" s="4"/>
+      <c r="C144" t="s">
         <v>175</v>
       </c>
-      <c r="D143">
-        <v>1</v>
-      </c>
-      <c r="E143">
-        <v>0</v>
-      </c>
-      <c r="F143">
-        <v>0</v>
-      </c>
-      <c r="G143">
-        <v>0</v>
-      </c>
-      <c r="H143">
-        <v>0</v>
-      </c>
-      <c r="I143">
-        <v>0</v>
-      </c>
-      <c r="J143">
-        <v>0</v>
-      </c>
-      <c r="K143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A144" s="4" t="s">
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>0</v>
+      </c>
+      <c r="F144">
+        <v>0</v>
+      </c>
+      <c r="G144">
+        <v>0</v>
+      </c>
+      <c r="H144">
+        <v>0</v>
+      </c>
+      <c r="I144">
+        <v>0</v>
+      </c>
+      <c r="J144">
+        <v>0</v>
+      </c>
+      <c r="K144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B144" s="4" t="s">
+      <c r="B145" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C144" t="s">
+      <c r="C145" t="s">
         <v>178</v>
-      </c>
-      <c r="D144">
-        <v>1</v>
-      </c>
-      <c r="E144">
-        <v>1</v>
-      </c>
-      <c r="F144">
-        <v>1</v>
-      </c>
-      <c r="G144">
-        <v>1</v>
-      </c>
-      <c r="H144">
-        <v>1</v>
-      </c>
-      <c r="I144">
-        <v>1</v>
-      </c>
-      <c r="J144">
-        <v>0</v>
-      </c>
-      <c r="K144">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A145" s="4"/>
-      <c r="B145" s="4"/>
-      <c r="C145" t="s">
-        <v>179</v>
       </c>
       <c r="D145">
         <v>1</v>
@@ -5631,7 +5639,7 @@
       <c r="A146" s="4"/>
       <c r="B146" s="4"/>
       <c r="C146" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -5662,7 +5670,7 @@
       <c r="A147" s="4"/>
       <c r="B147" s="4"/>
       <c r="C147" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -5693,7 +5701,7 @@
       <c r="A148" s="4"/>
       <c r="B148" s="4"/>
       <c r="C148" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -5722,11 +5730,9 @@
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
-      <c r="B149" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B149" s="4"/>
       <c r="C149" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -5755,111 +5761,113 @@
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150" s="4"/>
-      <c r="B150" s="4"/>
+      <c r="B150" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C150" t="s">
+        <v>184</v>
+      </c>
+      <c r="D150">
+        <v>1</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150">
+        <v>1</v>
+      </c>
+      <c r="G150">
+        <v>1</v>
+      </c>
+      <c r="H150">
+        <v>1</v>
+      </c>
+      <c r="I150">
+        <v>1</v>
+      </c>
+      <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A151" s="4"/>
+      <c r="B151" s="4"/>
+      <c r="C151" t="s">
         <v>185</v>
       </c>
-      <c r="D150">
-        <v>1</v>
-      </c>
-      <c r="E150">
-        <v>1</v>
-      </c>
-      <c r="F150">
-        <v>1</v>
-      </c>
-      <c r="G150">
-        <v>1</v>
-      </c>
-      <c r="H150">
-        <v>1</v>
-      </c>
-      <c r="I150">
-        <v>1</v>
-      </c>
-      <c r="J150">
-        <v>0</v>
-      </c>
-      <c r="K150">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="1" t="s">
+      <c r="D151">
+        <v>1</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151">
+        <v>1</v>
+      </c>
+      <c r="G151">
+        <v>1</v>
+      </c>
+      <c r="H151">
+        <v>1</v>
+      </c>
+      <c r="I151">
+        <v>1</v>
+      </c>
+      <c r="J151">
+        <v>0</v>
+      </c>
+      <c r="K151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A152" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B152" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C151" t="s">
+      <c r="C152" t="s">
         <v>186</v>
       </c>
-      <c r="D151">
-        <v>1</v>
-      </c>
-      <c r="E151">
-        <v>1</v>
-      </c>
-      <c r="F151">
-        <v>1</v>
-      </c>
-      <c r="G151">
-        <v>1</v>
-      </c>
-      <c r="H151">
-        <v>1</v>
-      </c>
-      <c r="I151">
-        <v>1</v>
-      </c>
-      <c r="J151">
-        <v>1</v>
-      </c>
-      <c r="K151">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A152" s="4" t="s">
+      <c r="D152">
+        <v>1</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152">
+        <v>1</v>
+      </c>
+      <c r="G152">
+        <v>1</v>
+      </c>
+      <c r="H152">
+        <v>1</v>
+      </c>
+      <c r="I152">
+        <v>1</v>
+      </c>
+      <c r="J152">
+        <v>1</v>
+      </c>
+      <c r="K152">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A153" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B152" s="4" t="s">
+      <c r="B153" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C152" t="s">
+      <c r="C153" t="s">
         <v>190</v>
       </c>
-      <c r="D152">
-        <v>1</v>
-      </c>
-      <c r="E152">
-        <v>1</v>
-      </c>
-      <c r="F152">
-        <v>0</v>
-      </c>
-      <c r="G152">
-        <v>0</v>
-      </c>
-      <c r="H152">
-        <v>0</v>
-      </c>
-      <c r="I152">
-        <v>0</v>
-      </c>
-      <c r="J152">
-        <v>0</v>
-      </c>
-      <c r="K152">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A153" s="4"/>
-      <c r="B153" s="4"/>
-      <c r="C153" t="s">
-        <v>191</v>
-      </c>
       <c r="D153">
         <v>1</v>
       </c>
@@ -5867,13 +5875,13 @@
         <v>1</v>
       </c>
       <c r="F153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I153">
         <v>0</v>
@@ -5889,7 +5897,7 @@
       <c r="A154" s="4"/>
       <c r="B154" s="4"/>
       <c r="C154" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D154">
         <v>1</v>
@@ -5898,13 +5906,13 @@
         <v>1</v>
       </c>
       <c r="F154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I154">
         <v>0</v>
@@ -5920,108 +5928,138 @@
       <c r="A155" s="4"/>
       <c r="B155" s="4"/>
       <c r="C155" t="s">
+        <v>192</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155">
+        <v>0</v>
+      </c>
+      <c r="I155">
+        <v>0</v>
+      </c>
+      <c r="J155">
+        <v>0</v>
+      </c>
+      <c r="K155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A156" s="4"/>
+      <c r="B156" s="4"/>
+      <c r="C156" t="s">
         <v>193</v>
       </c>
-      <c r="D155">
-        <v>1</v>
-      </c>
-      <c r="E155">
-        <v>1</v>
-      </c>
-      <c r="F155">
-        <v>0</v>
-      </c>
-      <c r="G155">
-        <v>0</v>
-      </c>
-      <c r="H155">
-        <v>0</v>
-      </c>
-      <c r="I155">
-        <v>0</v>
-      </c>
-      <c r="J155">
-        <v>0</v>
-      </c>
-      <c r="K155">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A156" s="4" t="s">
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+      <c r="F156">
+        <v>0</v>
+      </c>
+      <c r="G156">
+        <v>0</v>
+      </c>
+      <c r="H156">
+        <v>0</v>
+      </c>
+      <c r="I156">
+        <v>0</v>
+      </c>
+      <c r="J156">
+        <v>0</v>
+      </c>
+      <c r="K156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A157" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B156" s="4" t="s">
+      <c r="B157" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C156" t="s">
+      <c r="C157" t="s">
         <v>197</v>
       </c>
-      <c r="D156">
-        <v>1</v>
-      </c>
-      <c r="E156">
-        <v>1</v>
-      </c>
-      <c r="F156">
-        <v>0</v>
-      </c>
-      <c r="G156">
-        <v>0</v>
-      </c>
-      <c r="H156">
-        <v>0</v>
-      </c>
-      <c r="I156">
-        <v>0</v>
-      </c>
-      <c r="J156">
-        <v>0</v>
-      </c>
-      <c r="K156">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A157" s="4"/>
-      <c r="B157" s="4"/>
-      <c r="C157" t="s">
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157">
+        <v>0</v>
+      </c>
+      <c r="G157">
+        <v>0</v>
+      </c>
+      <c r="H157">
+        <v>0</v>
+      </c>
+      <c r="I157">
+        <v>0</v>
+      </c>
+      <c r="J157">
+        <v>0</v>
+      </c>
+      <c r="K157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A158" s="4"/>
+      <c r="B158" s="4"/>
+      <c r="C158" t="s">
         <v>198</v>
       </c>
-      <c r="D157">
-        <v>1</v>
-      </c>
-      <c r="E157">
-        <v>1</v>
-      </c>
-      <c r="F157">
-        <v>0</v>
-      </c>
-      <c r="G157">
-        <v>0</v>
-      </c>
-      <c r="H157">
-        <v>0</v>
-      </c>
-      <c r="I157">
-        <v>0</v>
-      </c>
-      <c r="J157">
-        <v>0</v>
-      </c>
-      <c r="K157">
+      <c r="D158">
+        <v>1</v>
+      </c>
+      <c r="E158">
+        <v>1</v>
+      </c>
+      <c r="F158">
+        <v>0</v>
+      </c>
+      <c r="G158">
+        <v>0</v>
+      </c>
+      <c r="H158">
+        <v>0</v>
+      </c>
+      <c r="I158">
+        <v>0</v>
+      </c>
+      <c r="J158">
+        <v>0</v>
+      </c>
+      <c r="K158">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="A156:A157"/>
-    <mergeCell ref="B156:B157"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
     <mergeCell ref="B32:B36"/>
     <mergeCell ref="B37:B41"/>
     <mergeCell ref="B42:B46"/>
     <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A102"/>
     <mergeCell ref="B67:B71"/>
     <mergeCell ref="B72:B76"/>
     <mergeCell ref="B77:B81"/>
@@ -6029,10 +6067,10 @@
     <mergeCell ref="B87:B92"/>
     <mergeCell ref="B93:B97"/>
     <mergeCell ref="B98:B102"/>
-    <mergeCell ref="A152:A155"/>
-    <mergeCell ref="B152:B155"/>
-    <mergeCell ref="B103:B110"/>
-    <mergeCell ref="A103:A134"/>
+    <mergeCell ref="A153:A156"/>
+    <mergeCell ref="B153:B156"/>
+    <mergeCell ref="B104:B111"/>
+    <mergeCell ref="A104:A135"/>
     <mergeCell ref="A2:A26"/>
     <mergeCell ref="A27:A66"/>
     <mergeCell ref="B2:B6"/>
@@ -6045,18 +6083,19 @@
     <mergeCell ref="B52:B56"/>
     <mergeCell ref="B57:B61"/>
     <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B131:B134"/>
-    <mergeCell ref="A135:A137"/>
-    <mergeCell ref="A138:A143"/>
-    <mergeCell ref="A144:A150"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B118"/>
-    <mergeCell ref="B119:B125"/>
-    <mergeCell ref="B126:B130"/>
-    <mergeCell ref="B135:B137"/>
-    <mergeCell ref="B138:B143"/>
-    <mergeCell ref="B144:B148"/>
-    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="B132:B135"/>
+    <mergeCell ref="A87:A103"/>
+    <mergeCell ref="A136:A138"/>
+    <mergeCell ref="A139:A144"/>
+    <mergeCell ref="A145:A151"/>
+    <mergeCell ref="B112:B114"/>
+    <mergeCell ref="B115:B119"/>
+    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="B127:B131"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="B139:B144"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="B150:B151"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
basic public api UI (#463)
* add basic public api UI

* permission hotfix

* Potential fix

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>

* error message fix

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>

* code optimizations

* Optimize complexity and files length. Cleaned code.

---------

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\kompetencyjny\Smart-University-Scheduler\helpers\db_seeder\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Smart-University-Scheduler\helpers\db_seeder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F317874-4BC0-4E7B-B789-C2FB1D819C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8ED8031-B46D-49E0-B168-972FBA6C8EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="208">
   <si>
     <t>Uprawnienie \ Rola</t>
   </si>
@@ -690,6 +690,12 @@
   </si>
   <si>
     <t>custom-events:create</t>
+  </si>
+  <si>
+    <t>api key</t>
+  </si>
+  <si>
+    <t>api-key:generate</t>
   </si>
 </sst>
 </file>
@@ -1042,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K157"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
@@ -4269,46 +4275,48 @@
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A103" s="4" t="s">
+      <c r="A103" s="4"/>
+      <c r="B103" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C103" t="s">
+        <v>207</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>0</v>
+      </c>
+      <c r="G103">
+        <v>0</v>
+      </c>
+      <c r="H103">
+        <v>0</v>
+      </c>
+      <c r="I103">
+        <v>0</v>
+      </c>
+      <c r="J103">
+        <v>0</v>
+      </c>
+      <c r="K103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B104" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C103" s="2" t="s">
+      <c r="C104" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D103">
-        <v>1</v>
-      </c>
-      <c r="E103">
-        <v>1</v>
-      </c>
-      <c r="F103">
-        <v>1</v>
-      </c>
-      <c r="G103">
-        <v>0</v>
-      </c>
-      <c r="H103">
-        <v>0</v>
-      </c>
-      <c r="I103">
-        <v>0</v>
-      </c>
-      <c r="J103">
-        <v>0</v>
-      </c>
-      <c r="K103">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A104" s="4"/>
-      <c r="B104" s="4"/>
-      <c r="C104" s="2" t="s">
-        <v>135</v>
-      </c>
       <c r="D104">
         <v>1</v>
       </c>
@@ -4319,26 +4327,26 @@
         <v>1</v>
       </c>
       <c r="G104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K104">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="2" t="s">
-        <v>194</v>
+        <v>135</v>
       </c>
       <c r="D105">
         <v>1</v>
@@ -4356,20 +4364,20 @@
         <v>1</v>
       </c>
       <c r="I105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K105">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="2" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="D106">
         <v>1</v>
@@ -4387,20 +4395,20 @@
         <v>1</v>
       </c>
       <c r="I106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K106">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D107">
         <v>1</v>
@@ -4412,26 +4420,26 @@
         <v>1</v>
       </c>
       <c r="G107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K107">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -4462,7 +4470,7 @@
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D109">
         <v>1</v>
@@ -4474,96 +4482,96 @@
         <v>1</v>
       </c>
       <c r="G109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K109">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="2" t="s">
-        <v>200</v>
+        <v>139</v>
       </c>
       <c r="D110">
         <v>1</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K110">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
-      <c r="B111" s="4" t="s">
-        <v>140</v>
-      </c>
+      <c r="B111" s="4"/>
       <c r="C111" s="2" t="s">
-        <v>141</v>
+        <v>200</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K111">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
-      <c r="B112" s="4"/>
+      <c r="B112" s="4" t="s">
+        <v>140</v>
+      </c>
       <c r="C112" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D112">
         <v>1</v>
       </c>
       <c r="E112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F112">
         <v>1</v>
@@ -4572,23 +4580,23 @@
         <v>1</v>
       </c>
       <c r="H112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K112">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -4617,17 +4625,15 @@
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
-      <c r="B114" s="4" t="s">
-        <v>144</v>
-      </c>
+      <c r="B114" s="4"/>
       <c r="C114" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D114">
         <v>1</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F114">
         <v>1</v>
@@ -4636,23 +4642,25 @@
         <v>1</v>
       </c>
       <c r="H114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K114">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A115" s="4"/>
-      <c r="B115" s="4"/>
+      <c r="B115" s="4" t="s">
+        <v>144</v>
+      </c>
       <c r="C115" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4683,7 +4691,7 @@
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4695,26 +4703,26 @@
         <v>1</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K116">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4745,7 +4753,7 @@
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4774,11 +4782,9 @@
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
-      <c r="B119" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="B119" s="4"/>
       <c r="C119" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4790,16 +4796,16 @@
         <v>1</v>
       </c>
       <c r="G119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K119">
         <v>0</v>
@@ -4807,9 +4813,11 @@
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120" s="4"/>
-      <c r="B120" s="4"/>
+      <c r="B120" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="C120" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4840,7 +4848,7 @@
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4871,7 +4879,7 @@
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4883,16 +4891,16 @@
         <v>1</v>
       </c>
       <c r="G122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K122">
         <v>0</v>
@@ -4902,7 +4910,7 @@
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4933,7 +4941,7 @@
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4964,7 +4972,7 @@
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4993,11 +5001,9 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126" s="4"/>
-      <c r="B126" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="B126" s="4"/>
       <c r="C126" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -5009,16 +5015,16 @@
         <v>1</v>
       </c>
       <c r="G126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K126">
         <v>0</v>
@@ -5026,9 +5032,11 @@
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A127" s="4"/>
-      <c r="B127" s="4"/>
+      <c r="B127" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="C127" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -5059,13 +5067,13 @@
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D128">
         <v>1</v>
       </c>
       <c r="E128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F128">
         <v>1</v>
@@ -5077,10 +5085,10 @@
         <v>1</v>
       </c>
       <c r="I128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K128">
         <v>0</v>
@@ -5090,7 +5098,7 @@
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -5121,7 +5129,7 @@
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -5133,10 +5141,10 @@
         <v>1</v>
       </c>
       <c r="G130">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H130">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I130">
         <v>0</v>
@@ -5150,17 +5158,15 @@
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" s="4"/>
-      <c r="B131" s="4" t="s">
-        <v>201</v>
-      </c>
+      <c r="B131" s="4"/>
       <c r="C131" s="2" t="s">
-        <v>205</v>
+        <v>163</v>
       </c>
       <c r="D131">
         <v>1</v>
       </c>
       <c r="E131">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F131">
         <v>1</v>
@@ -5183,9 +5189,11 @@
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
+      <c r="B132" s="4" t="s">
+        <v>201</v>
+      </c>
       <c r="C132" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -5197,16 +5205,16 @@
         <v>1</v>
       </c>
       <c r="G132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K132">
         <v>0</v>
@@ -5216,7 +5224,7 @@
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -5228,16 +5236,16 @@
         <v>1</v>
       </c>
       <c r="G133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J133">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K133">
         <v>0</v>
@@ -5247,73 +5255,73 @@
       <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134">
+        <v>1</v>
+      </c>
+      <c r="F134">
+        <v>1</v>
+      </c>
+      <c r="G134">
+        <v>0</v>
+      </c>
+      <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+      <c r="J134">
+        <v>0</v>
+      </c>
+      <c r="K134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A135" s="4"/>
+      <c r="B135" s="4"/>
+      <c r="C135" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D134">
-        <v>1</v>
-      </c>
-      <c r="E134">
-        <v>1</v>
-      </c>
-      <c r="F134">
-        <v>1</v>
-      </c>
-      <c r="G134">
-        <v>0</v>
-      </c>
-      <c r="H134">
-        <v>0</v>
-      </c>
-      <c r="I134">
-        <v>0</v>
-      </c>
-      <c r="J134">
-        <v>0</v>
-      </c>
-      <c r="K134">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A135" s="4" t="s">
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135">
+        <v>1</v>
+      </c>
+      <c r="F135">
+        <v>1</v>
+      </c>
+      <c r="G135">
+        <v>0</v>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A136" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B135" s="4" t="s">
+      <c r="B136" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C135" t="s">
+      <c r="C136" t="s">
         <v>166</v>
-      </c>
-      <c r="D135">
-        <v>1</v>
-      </c>
-      <c r="E135">
-        <v>0</v>
-      </c>
-      <c r="F135">
-        <v>0</v>
-      </c>
-      <c r="G135">
-        <v>0</v>
-      </c>
-      <c r="H135">
-        <v>0</v>
-      </c>
-      <c r="I135">
-        <v>0</v>
-      </c>
-      <c r="J135">
-        <v>0</v>
-      </c>
-      <c r="K135">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
-      <c r="C136" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -5344,73 +5352,73 @@
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>0</v>
+      </c>
+      <c r="F137">
+        <v>0</v>
+      </c>
+      <c r="G137">
+        <v>0</v>
+      </c>
+      <c r="H137">
+        <v>0</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="4"/>
+      <c r="B138" s="4"/>
+      <c r="C138" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D137">
-        <v>1</v>
-      </c>
-      <c r="E137">
-        <v>0</v>
-      </c>
-      <c r="F137">
-        <v>0</v>
-      </c>
-      <c r="G137">
-        <v>0</v>
-      </c>
-      <c r="H137">
-        <v>0</v>
-      </c>
-      <c r="I137">
-        <v>0</v>
-      </c>
-      <c r="J137">
-        <v>0</v>
-      </c>
-      <c r="K137">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A138" s="4" t="s">
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B138" s="4" t="s">
+      <c r="B139" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C139" t="s">
         <v>170</v>
-      </c>
-      <c r="D138">
-        <v>1</v>
-      </c>
-      <c r="E138">
-        <v>0</v>
-      </c>
-      <c r="F138">
-        <v>0</v>
-      </c>
-      <c r="G138">
-        <v>0</v>
-      </c>
-      <c r="H138">
-        <v>0</v>
-      </c>
-      <c r="I138">
-        <v>0</v>
-      </c>
-      <c r="J138">
-        <v>0</v>
-      </c>
-      <c r="K138">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A139" s="4"/>
-      <c r="B139" s="4"/>
-      <c r="C139" t="s">
-        <v>171</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -5441,7 +5449,7 @@
       <c r="A140" s="4"/>
       <c r="B140" s="4"/>
       <c r="C140" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D140">
         <v>1</v>
@@ -5472,7 +5480,7 @@
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -5503,7 +5511,7 @@
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -5534,73 +5542,73 @@
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" t="s">
+        <v>174</v>
+      </c>
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>0</v>
+      </c>
+      <c r="F143">
+        <v>0</v>
+      </c>
+      <c r="G143">
+        <v>0</v>
+      </c>
+      <c r="H143">
+        <v>0</v>
+      </c>
+      <c r="I143">
+        <v>0</v>
+      </c>
+      <c r="J143">
+        <v>0</v>
+      </c>
+      <c r="K143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A144" s="4"/>
+      <c r="B144" s="4"/>
+      <c r="C144" t="s">
         <v>175</v>
       </c>
-      <c r="D143">
-        <v>1</v>
-      </c>
-      <c r="E143">
-        <v>0</v>
-      </c>
-      <c r="F143">
-        <v>0</v>
-      </c>
-      <c r="G143">
-        <v>0</v>
-      </c>
-      <c r="H143">
-        <v>0</v>
-      </c>
-      <c r="I143">
-        <v>0</v>
-      </c>
-      <c r="J143">
-        <v>0</v>
-      </c>
-      <c r="K143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A144" s="4" t="s">
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>0</v>
+      </c>
+      <c r="F144">
+        <v>0</v>
+      </c>
+      <c r="G144">
+        <v>0</v>
+      </c>
+      <c r="H144">
+        <v>0</v>
+      </c>
+      <c r="I144">
+        <v>0</v>
+      </c>
+      <c r="J144">
+        <v>0</v>
+      </c>
+      <c r="K144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B144" s="4" t="s">
+      <c r="B145" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C144" t="s">
+      <c r="C145" t="s">
         <v>178</v>
-      </c>
-      <c r="D144">
-        <v>1</v>
-      </c>
-      <c r="E144">
-        <v>1</v>
-      </c>
-      <c r="F144">
-        <v>1</v>
-      </c>
-      <c r="G144">
-        <v>1</v>
-      </c>
-      <c r="H144">
-        <v>1</v>
-      </c>
-      <c r="I144">
-        <v>1</v>
-      </c>
-      <c r="J144">
-        <v>0</v>
-      </c>
-      <c r="K144">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A145" s="4"/>
-      <c r="B145" s="4"/>
-      <c r="C145" t="s">
-        <v>179</v>
       </c>
       <c r="D145">
         <v>1</v>
@@ -5631,7 +5639,7 @@
       <c r="A146" s="4"/>
       <c r="B146" s="4"/>
       <c r="C146" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -5662,7 +5670,7 @@
       <c r="A147" s="4"/>
       <c r="B147" s="4"/>
       <c r="C147" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -5693,7 +5701,7 @@
       <c r="A148" s="4"/>
       <c r="B148" s="4"/>
       <c r="C148" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -5722,11 +5730,9 @@
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
-      <c r="B149" s="4" t="s">
-        <v>183</v>
-      </c>
+      <c r="B149" s="4"/>
       <c r="C149" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -5755,111 +5761,113 @@
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150" s="4"/>
-      <c r="B150" s="4"/>
+      <c r="B150" s="4" t="s">
+        <v>183</v>
+      </c>
       <c r="C150" t="s">
+        <v>184</v>
+      </c>
+      <c r="D150">
+        <v>1</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150">
+        <v>1</v>
+      </c>
+      <c r="G150">
+        <v>1</v>
+      </c>
+      <c r="H150">
+        <v>1</v>
+      </c>
+      <c r="I150">
+        <v>1</v>
+      </c>
+      <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A151" s="4"/>
+      <c r="B151" s="4"/>
+      <c r="C151" t="s">
         <v>185</v>
       </c>
-      <c r="D150">
-        <v>1</v>
-      </c>
-      <c r="E150">
-        <v>1</v>
-      </c>
-      <c r="F150">
-        <v>1</v>
-      </c>
-      <c r="G150">
-        <v>1</v>
-      </c>
-      <c r="H150">
-        <v>1</v>
-      </c>
-      <c r="I150">
-        <v>1</v>
-      </c>
-      <c r="J150">
-        <v>0</v>
-      </c>
-      <c r="K150">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="1" t="s">
+      <c r="D151">
+        <v>1</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151">
+        <v>1</v>
+      </c>
+      <c r="G151">
+        <v>1</v>
+      </c>
+      <c r="H151">
+        <v>1</v>
+      </c>
+      <c r="I151">
+        <v>1</v>
+      </c>
+      <c r="J151">
+        <v>0</v>
+      </c>
+      <c r="K151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A152" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B152" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C151" t="s">
+      <c r="C152" t="s">
         <v>186</v>
       </c>
-      <c r="D151">
-        <v>1</v>
-      </c>
-      <c r="E151">
-        <v>1</v>
-      </c>
-      <c r="F151">
-        <v>1</v>
-      </c>
-      <c r="G151">
-        <v>1</v>
-      </c>
-      <c r="H151">
-        <v>1</v>
-      </c>
-      <c r="I151">
-        <v>1</v>
-      </c>
-      <c r="J151">
-        <v>1</v>
-      </c>
-      <c r="K151">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A152" s="4" t="s">
+      <c r="D152">
+        <v>1</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152">
+        <v>1</v>
+      </c>
+      <c r="G152">
+        <v>1</v>
+      </c>
+      <c r="H152">
+        <v>1</v>
+      </c>
+      <c r="I152">
+        <v>1</v>
+      </c>
+      <c r="J152">
+        <v>1</v>
+      </c>
+      <c r="K152">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A153" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B152" s="4" t="s">
+      <c r="B153" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C152" t="s">
+      <c r="C153" t="s">
         <v>190</v>
       </c>
-      <c r="D152">
-        <v>1</v>
-      </c>
-      <c r="E152">
-        <v>1</v>
-      </c>
-      <c r="F152">
-        <v>0</v>
-      </c>
-      <c r="G152">
-        <v>0</v>
-      </c>
-      <c r="H152">
-        <v>0</v>
-      </c>
-      <c r="I152">
-        <v>0</v>
-      </c>
-      <c r="J152">
-        <v>0</v>
-      </c>
-      <c r="K152">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A153" s="4"/>
-      <c r="B153" s="4"/>
-      <c r="C153" t="s">
-        <v>191</v>
-      </c>
       <c r="D153">
         <v>1</v>
       </c>
@@ -5867,13 +5875,13 @@
         <v>1</v>
       </c>
       <c r="F153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I153">
         <v>0</v>
@@ -5889,7 +5897,7 @@
       <c r="A154" s="4"/>
       <c r="B154" s="4"/>
       <c r="C154" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D154">
         <v>1</v>
@@ -5898,13 +5906,13 @@
         <v>1</v>
       </c>
       <c r="F154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I154">
         <v>0</v>
@@ -5920,108 +5928,138 @@
       <c r="A155" s="4"/>
       <c r="B155" s="4"/>
       <c r="C155" t="s">
+        <v>192</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155">
+        <v>0</v>
+      </c>
+      <c r="I155">
+        <v>0</v>
+      </c>
+      <c r="J155">
+        <v>0</v>
+      </c>
+      <c r="K155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A156" s="4"/>
+      <c r="B156" s="4"/>
+      <c r="C156" t="s">
         <v>193</v>
       </c>
-      <c r="D155">
-        <v>1</v>
-      </c>
-      <c r="E155">
-        <v>1</v>
-      </c>
-      <c r="F155">
-        <v>0</v>
-      </c>
-      <c r="G155">
-        <v>0</v>
-      </c>
-      <c r="H155">
-        <v>0</v>
-      </c>
-      <c r="I155">
-        <v>0</v>
-      </c>
-      <c r="J155">
-        <v>0</v>
-      </c>
-      <c r="K155">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A156" s="4" t="s">
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+      <c r="F156">
+        <v>0</v>
+      </c>
+      <c r="G156">
+        <v>0</v>
+      </c>
+      <c r="H156">
+        <v>0</v>
+      </c>
+      <c r="I156">
+        <v>0</v>
+      </c>
+      <c r="J156">
+        <v>0</v>
+      </c>
+      <c r="K156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A157" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B156" s="4" t="s">
+      <c r="B157" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C156" t="s">
+      <c r="C157" t="s">
         <v>197</v>
       </c>
-      <c r="D156">
-        <v>1</v>
-      </c>
-      <c r="E156">
-        <v>1</v>
-      </c>
-      <c r="F156">
-        <v>0</v>
-      </c>
-      <c r="G156">
-        <v>0</v>
-      </c>
-      <c r="H156">
-        <v>0</v>
-      </c>
-      <c r="I156">
-        <v>0</v>
-      </c>
-      <c r="J156">
-        <v>0</v>
-      </c>
-      <c r="K156">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A157" s="4"/>
-      <c r="B157" s="4"/>
-      <c r="C157" t="s">
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157">
+        <v>0</v>
+      </c>
+      <c r="G157">
+        <v>0</v>
+      </c>
+      <c r="H157">
+        <v>0</v>
+      </c>
+      <c r="I157">
+        <v>0</v>
+      </c>
+      <c r="J157">
+        <v>0</v>
+      </c>
+      <c r="K157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A158" s="4"/>
+      <c r="B158" s="4"/>
+      <c r="C158" t="s">
         <v>198</v>
       </c>
-      <c r="D157">
-        <v>1</v>
-      </c>
-      <c r="E157">
-        <v>1</v>
-      </c>
-      <c r="F157">
-        <v>0</v>
-      </c>
-      <c r="G157">
-        <v>0</v>
-      </c>
-      <c r="H157">
-        <v>0</v>
-      </c>
-      <c r="I157">
-        <v>0</v>
-      </c>
-      <c r="J157">
-        <v>0</v>
-      </c>
-      <c r="K157">
+      <c r="D158">
+        <v>1</v>
+      </c>
+      <c r="E158">
+        <v>1</v>
+      </c>
+      <c r="F158">
+        <v>0</v>
+      </c>
+      <c r="G158">
+        <v>0</v>
+      </c>
+      <c r="H158">
+        <v>0</v>
+      </c>
+      <c r="I158">
+        <v>0</v>
+      </c>
+      <c r="J158">
+        <v>0</v>
+      </c>
+      <c r="K158">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="A156:A157"/>
-    <mergeCell ref="B156:B157"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
     <mergeCell ref="B32:B36"/>
     <mergeCell ref="B37:B41"/>
     <mergeCell ref="B42:B46"/>
     <mergeCell ref="A67:A86"/>
-    <mergeCell ref="A87:A102"/>
     <mergeCell ref="B67:B71"/>
     <mergeCell ref="B72:B76"/>
     <mergeCell ref="B77:B81"/>
@@ -6029,10 +6067,10 @@
     <mergeCell ref="B87:B92"/>
     <mergeCell ref="B93:B97"/>
     <mergeCell ref="B98:B102"/>
-    <mergeCell ref="A152:A155"/>
-    <mergeCell ref="B152:B155"/>
-    <mergeCell ref="B103:B110"/>
-    <mergeCell ref="A103:A134"/>
+    <mergeCell ref="A153:A156"/>
+    <mergeCell ref="B153:B156"/>
+    <mergeCell ref="B104:B111"/>
+    <mergeCell ref="A104:A135"/>
     <mergeCell ref="A2:A26"/>
     <mergeCell ref="A27:A66"/>
     <mergeCell ref="B2:B6"/>
@@ -6045,18 +6083,19 @@
     <mergeCell ref="B52:B56"/>
     <mergeCell ref="B57:B61"/>
     <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B131:B134"/>
-    <mergeCell ref="A135:A137"/>
-    <mergeCell ref="A138:A143"/>
-    <mergeCell ref="A144:A150"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B118"/>
-    <mergeCell ref="B119:B125"/>
-    <mergeCell ref="B126:B130"/>
-    <mergeCell ref="B135:B137"/>
-    <mergeCell ref="B138:B143"/>
-    <mergeCell ref="B144:B148"/>
-    <mergeCell ref="B149:B150"/>
+    <mergeCell ref="B132:B135"/>
+    <mergeCell ref="A87:A103"/>
+    <mergeCell ref="A136:A138"/>
+    <mergeCell ref="A139:A144"/>
+    <mergeCell ref="A145:A151"/>
+    <mergeCell ref="B112:B114"/>
+    <mergeCell ref="B115:B119"/>
+    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="B127:B131"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="B139:B144"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="B150:B151"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Deleted permission for student
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Smart-University-Scheduler\helpers\db_seeder\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Studia\semestr6\Projekt_kompetencyjny\Smart-University-Scheduler\helpers\db_seeder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8ED8031-B46D-49E0-B168-972FBA6C8EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B2B3B9-CCC1-45D4-A9A7-97FCF39D07A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4835,7 +4835,7 @@
         <v>1</v>
       </c>
       <c r="I120">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J120">
         <v>1</v>
@@ -4866,7 +4866,7 @@
         <v>1</v>
       </c>
       <c r="I121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J121">
         <v>1</v>
@@ -6054,6 +6054,32 @@
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="A136:A138"/>
+    <mergeCell ref="A139:A144"/>
+    <mergeCell ref="A145:A151"/>
+    <mergeCell ref="B112:B114"/>
+    <mergeCell ref="B115:B119"/>
+    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="B127:B131"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="B139:B144"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="A104:A135"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B132:B135"/>
+    <mergeCell ref="A87:A103"/>
     <mergeCell ref="A157:A158"/>
     <mergeCell ref="B157:B158"/>
     <mergeCell ref="B32:B36"/>
@@ -6070,32 +6096,6 @@
     <mergeCell ref="A153:A156"/>
     <mergeCell ref="B153:B156"/>
     <mergeCell ref="B104:B111"/>
-    <mergeCell ref="A104:A135"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B132:B135"/>
-    <mergeCell ref="A87:A103"/>
-    <mergeCell ref="A136:A138"/>
-    <mergeCell ref="A139:A144"/>
-    <mergeCell ref="A145:A151"/>
-    <mergeCell ref="B112:B114"/>
-    <mergeCell ref="B115:B119"/>
-    <mergeCell ref="B120:B126"/>
-    <mergeCell ref="B127:B131"/>
-    <mergeCell ref="B136:B138"/>
-    <mergeCell ref="B139:B144"/>
-    <mergeCell ref="B145:B149"/>
-    <mergeCell ref="B150:B151"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6104,14 +6104,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6304,21 +6302,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
-    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6343,9 +6340,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
+    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix suggestions frontend + backend (#504)
* Deleted permission for student

* Fixed suggestions frontend

* English
</commit_message>
<xml_diff>
--- a/helpers/db_seeder/data/role_uprawnienia.xlsx
+++ b/helpers/db_seeder/data/role_uprawnienia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Smart-University-Scheduler\helpers\db_seeder\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Studia\semestr6\Projekt_kompetencyjny\Smart-University-Scheduler\helpers\db_seeder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8ED8031-B46D-49E0-B168-972FBA6C8EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B2B3B9-CCC1-45D4-A9A7-97FCF39D07A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4835,7 +4835,7 @@
         <v>1</v>
       </c>
       <c r="I120">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J120">
         <v>1</v>
@@ -4866,7 +4866,7 @@
         <v>1</v>
       </c>
       <c r="I121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J121">
         <v>1</v>
@@ -6054,6 +6054,32 @@
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="A136:A138"/>
+    <mergeCell ref="A139:A144"/>
+    <mergeCell ref="A145:A151"/>
+    <mergeCell ref="B112:B114"/>
+    <mergeCell ref="B115:B119"/>
+    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="B127:B131"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="B139:B144"/>
+    <mergeCell ref="B145:B149"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="A104:A135"/>
+    <mergeCell ref="A2:A26"/>
+    <mergeCell ref="A27:A66"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B132:B135"/>
+    <mergeCell ref="A87:A103"/>
     <mergeCell ref="A157:A158"/>
     <mergeCell ref="B157:B158"/>
     <mergeCell ref="B32:B36"/>
@@ -6070,32 +6096,6 @@
     <mergeCell ref="A153:A156"/>
     <mergeCell ref="B153:B156"/>
     <mergeCell ref="B104:B111"/>
-    <mergeCell ref="A104:A135"/>
-    <mergeCell ref="A2:A26"/>
-    <mergeCell ref="A27:A66"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B132:B135"/>
-    <mergeCell ref="A87:A103"/>
-    <mergeCell ref="A136:A138"/>
-    <mergeCell ref="A139:A144"/>
-    <mergeCell ref="A145:A151"/>
-    <mergeCell ref="B112:B114"/>
-    <mergeCell ref="B115:B119"/>
-    <mergeCell ref="B120:B126"/>
-    <mergeCell ref="B127:B131"/>
-    <mergeCell ref="B136:B138"/>
-    <mergeCell ref="B139:B144"/>
-    <mergeCell ref="B145:B149"/>
-    <mergeCell ref="B150:B151"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6104,14 +6104,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6304,21 +6302,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36e2ff40-ab52-4240-babf-7476b65fdfdc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3830623-0ee5-4634-96e5-1fabe66116f4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
-    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6343,9 +6340,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{650941DE-E334-4AB5-BCE8-14AB52A4A807}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8710C31-AC30-4E45-B8BB-6B8E8A833604}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36e2ff40-ab52-4240-babf-7476b65fdfdc"/>
+    <ds:schemaRef ds:uri="d3830623-0ee5-4634-96e5-1fabe66116f4"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>